<commit_message>
AM added languages english and hindi
</commit_message>
<xml_diff>
--- a/server/RSS_FullText.xlsx
+++ b/server/RSS_FullText.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="201">
   <si>
     <t>Source</t>
   </si>
@@ -35,6 +35,270 @@
   </si>
   <si>
     <t>TheHindu</t>
+  </si>
+  <si>
+    <t>Centre releases pending Samagra Shiksha funds to Kerala</t>
+  </si>
+  <si>
+    <t>The Union government has released pending Samagra Shiksha funds to the tune of ₹92.41 crore to Kerala.
+Another ₹17 crore from the sanctioned amount of ₹109 crore is expected to be released in a few days.
+The funds for the Centrally sponsored Samagra Shiksha scheme that will reach the government account will be transferred to the Samagra Shiksha Kerala (SSK) account after the SSK sends a request to this effect.
+The total approved amount for the Samagra Shiksha scheme for 2025-26 is ₹761 crore of which ₹456 crore is the Central share.
+Kerala had signed up for the PM SHRI scheme recently after the Union government had withheld Samagra Shiksha funds to the tune of ₹1,158.13 crore.
+However, the scheme was put on hold following dissension within the ruling Left Democratic Front (LDF). Coalition partner the CPI was especially upset that the agreement was signed without any discussion in the Cabinet or within the front.
+It remained adamant about a review or withdrawal of the MoU signed with the Union government. Finally, the Cabinet agreed to freeze the scheme and announced a subcommittee to study the CPI’s concerns on the scheme. It was also decided to formally inform the Union government of the State’s decision.
+However, almost a week later Kerala is yet to send a letter in this regard. Minister for General Education V. Sivankutty on Tuesday said procedures were under way and the communication would be sent soon.
+The Union government had informed the Supreme Court recently that Samagra Shiksha funds due to Kerala will be released soon. The court was considering a case related to appointment of special educators in the State.
+Samagra Shiksha hopes to send another proposal soon for the second instalment. However, uncertainty surrounds further release of funds, particularly once the State sends the communication on PM SHRI.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/kerala/centre-releases-pending-samagra-shiksha-funds-to-kerala/article70241547.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:52:34 +0530</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/theme/images/og-image.png</t>
+  </si>
+  <si>
+    <t>BJP announces week-long campaign against garbage and pothole issues in Bengaluru</t>
+  </si>
+  <si>
+    <t>The Opposition Bharatiya Janata Party (BJP) has announced a week-long campaign against Bengaluru’s “garbage disposal problem and pothole issues”.
+BJP held a meeting of all Bengaluru MLAs and MPs on Tuesday, following which the party announced a signature campaign against the ruling Congress government.
+“Due to the misgovernance of the Congress government, Bengaluru has turned into a garbage city. Potholes and piles of garbage are visible on all roads. We need to fight against the government that has betrayed the city, and it has been decided to conduct inspections for one week. Along with this, a signature collection campaign will be held in every assembly constituency from November 6 to 15,” Leader of Opposition in the Assembly, R. Ashok announced after the meeting.
+“We will also collect people’s opinion on the B Khata to A Khata conversion scheme, which we think is a scheme to extract money. The government has no funds for Bengaluru’s development. There is no need to take such steps to arrange that money. People cannot afford to pay so much. People do not want such an expensive brand Bengaluru. We need a Bengaluru that thinks about common people,” he said.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/bjp-announces-week-long-campaign-against-garbage-and-pothole-issues-in-bengaluru/article70240783.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:49:54 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/iom0dd/article70241558.ece/alternates/LANDSCAPE_1200/_JAI1974.JPG</t>
+  </si>
+  <si>
+    <t>Minister promotes Andhra Pradesh tourism at World Travel Market 2025 in London</t>
+  </si>
+  <si>
+    <t>Andhra Pradesh Tourism Minister Kandula Durgesh on Tuesday said the State would soon find a prominent place on the global tourism map, given its rich tourism potential. Participating in the World Travel Market (WTM) 2025 being held in London from November 4 to 6, the Minister said Andhra Pradesh was striving to emerge as a global tourism leader through a series of investor-friendly initiatives. He said the State aims to promote its diverse attractions — including natural landscapes, heritage sites such as Gandikota, and spiritual destinations — while focusing on sustainable development and enhanced visitor experiences.
+Mr. Durgesh, along with Special Secretary (Tourism) Ajay Jain, inaugurated both the Indian Ministry of Tourism and Andhra Pradesh Tourism stalls at the event. The State’s stall featured a Kuchipudi dance performance, highlighting Andhra Pradesh’s vibrant culture, and showcased its scenic beauty, historical forts, coastline, and cultural heritage.
+The Minister held discussions with more than 20 international tour operators, hotel groups, and investors from the MICE (Meetings, Incentives, Conferences and Exhibitions) sector, as well as travel media and tourism boards. He apprised them of the investment opportunities and tourism packages offered by the Andhra Pradesh government. Visitors to the stall were also treated to Araku coffee, Pootharekulu, and displays of colourful Etikoppaka and Kondapalli toys.
+Mr. Durgesh briefed the international media on the Andhra Pradesh Tourism Policy 2024–29, which accords industrial status to the tourism sector, and assured full government support to investors. Addressing groups of international visitors, he reiterated the government’s commitment to earning global recognition for Andhra Pradesh Tourism.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/andhra-pradesh/minister-promotes-andhra-pradesh-tourism-at-world-travel-market-2025-in-london/article70241312.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:48:29 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/3yxdnd/article70241546.ece/alternates/LANDSCAPE_1200/9604_4_11_2025_22_4_28_1_IMG_20251104_WA0032.JPG</t>
+  </si>
+  <si>
+    <t>GSAT-7R will strengthen Indian Navy’s surveillance and communication in the Indian Ocean Region</t>
+  </si>
+  <si>
+    <t>The successful launch of India’s CMS-03 (GSAT-7R) satellite aboard the LVM3-M5 rocket on November 2, 2025, from the Satish Dhawan Space Centre in Sriharikota will provide a major boost to the country’s pursuit of maritime security and technological self-reliance.
+The 4,400 kg multi-band communication satellite, designed and developed indigenously by the Indian Space Research Organisation (ISRO), is the heaviest communication satellite launched into the Geosynchronous Transfer Orbit (GTO) from Indian soil. It will play a crucial role in enhancing the Indian Navy’s operational reach, situational awareness, and surveillance capabilities across the Indian Ocean Region.
+Secure communication coverage
+The GSAT-7R is the successor to the GSAT-7 “Rukmini,” India’s first dedicated military satellite, launched in 2013. While Rukmini revolutionised naval communications by providing real-time data links across the Arabian Sea and the Bay of Bengal, the GSAT-7R significantly upgrades these capabilities. Equipped with multi-band transponders (UHF, S, C, and Ku bands), the GSAT-7R enables seamless voice, data, and video communication between naval ships, submarines, aircraft, and Maritime Operations Centres (MOCs). The satellite’s advanced payload ensures high-capacity, secure, and jam-resistant communication — vital for network-centric warfare and joint operations with the Army and the Air Force.
+With a lifespan of 15 years, the GSAT-7R extends secure communication coverage up to 2,000 km from India’s coastline, encompassing vast stretches of the Indian Ocean Region. This expanded coverage will allow the Indian Navy to monitor critical sea lanes, chokepoints, and potential maritime threats more effectively. It will support continuous coordination among naval assets deployed on anti-piracy, anti-submarine, and humanitarian missions, ensuring real-time situational updates and rapid response capabilities.
+Moreover, the GSAT-7R will enhance maritime domain awareness (MDA) by integrating space-based communication with surveillance platforms, such as coastal radars, reconnaissance aircraft, and unmanned systems. This synergy will allow the Navy to maintain an uninterrupted watch over the region’s dynamic maritime environment, strengthening India’s ability to deter and respond to any hostile activity.
+According to experts, the launch of the GSAT-7R underscores India’s growing self-reliance in defence space technology under the vision of Aatmanirbhar Bharat. By securing robust and indigenous satellite communication infrastructure, the Navy can operate independently of foreign systems, ensuring confidentiality and reliability in strategic operations.
+Quantum leap
+In essence, the GSAT-7R represents a quantum leap in India’s maritime communication and surveillance architecture, empowering the Indian Navy to maintain a vigilant, connected, and technologically advanced presence across the Indian Ocean Region.
+The Navy’s satellites, sensors, radars, unmanned aerial vehicles, and surveillance aircraft relay real-time data to the Information Management and Analysis Centre (IMAC), now being upgraded into a National Maritime Domain Awareness (NMDA) platform. The NMDA will integrate data from multiple sources to create a unified operational picture for naval commanders. Using AI-enabled analytics, it will enhance situational awareness, improve surveillance, and support swift decision-making. The system will help detect and counter threats such as illegal fishing, smuggling, piracy, and maritime terrorism, strengthening India’s maritime security and safeguarding its strategic interests across the Indian Ocean Region.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/sci-tech/gsat-7r-will-strengthen-indian-navys-surveillance-and-communication-in-the-indian-ocean-region/article70240234.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:42:47 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/seagfz/article70240681.ece/alternates/LANDSCAPE_1200/02th-SAURABH-muG30F42DOF.4.jpg.jpg</t>
+  </si>
+  <si>
+    <t>Karnataka issues guidelines for use of fines collected under tobacco control law</t>
+  </si>
+  <si>
+    <t>The State Health Department has issued revised guidelines for the proper utilisation of fines collected under the Cigarettes and Other Tobacco Products Act (COTPA), 2003, in Karnataka.
+Under the National Tobacco Control Programme (NTCP), implemented as part of the National Health Mission, authorised officers are empowered to levy spot fines on violators of COTPA. The fines collected are to be deposited in a joint account operated by the Deputy Commissioner and the District Health and Family Welfare Officer.
+According to the latest circular issued by the Health Commissioner on Tuesday, the fine amount should be used exclusively for tobacco control activities at the district level. District Tobacco Control Cells have been directed to prepare annual action plans outlining the use of the funds, which must be discussed and approved by the District-Level Coordination Committee (DLCC), chaired by the Deputy Commissioner.
+At least 70% of the fine amount should be used for strengthening tobacco de-addiction services. The permissible activities include the purchase of Nicotine Replacement Therapy (NRT) drugs and equipment such as CO monitors and spirometers, conducting training programmes and workshops, implementing tobacco-free educational institution and village guidelines, and undertaking IEC (Information, Education and Communication) campaigns., according to the revised guidelines.
+Districts have also been instructed to maintain proper records and submit annual audit reports as per NHM norms. Any proposal involving expenditure of more than ₹1 lakh from the fine amount will require approval from the Commissioner, the circular stated.
+The order further clarified that the fines collected under COTPA are to be treated as additional funds and can be used only after fully utilising the regular annual allocation provided under the NTCP.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/karnataka-issues-guidelines-for-use-of-fines-collected-under-tobacco-control-law/article70241013.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:42:13 +0530</t>
+  </si>
+  <si>
+    <t>Eight killed in car-truck collision in Barabanki</t>
+  </si>
+  <si>
+    <t>Eight people were killed after a truck collided with a car on the Deva-Fatehpur road in Barabanki district on Tuesday, officials said.
+The incident occurred when a speeding truck collided head-on with an Ertiga vehicle that reportedly did not have a licence plate. The impact of the collision was severe, leaving the car completely crushed and causing panic among bystanders.
+Among the deceased identified are driver Shrikant Shukla, Pradeep Soni, his wife Madhuri Soni, and their son Nitin, all residents of Fatehpur town. The identities of the other victims are yet to be confirmed.
+According to officials, all occupants of the Ertiga were returning home after taking a holy dip in the Ganges at Bithoor in Kanpur.
+Uttar Pradesh Chief Minister Yogi Adityanath expressed grief over the loss of lives and directed district officials to expedite relief measures.
+“The loss of life in the unfortunate accident is extremely sad and heart-wrenching. My condolences are with the bereaved families. I pray to Lord Shri Ram to grant salvation to the departed souls, strength to the bereaved families to bear this immense loss, and speedy recovery to the injured. Om peace,” an official statement quoted the Chief Minister as saying.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/uttar-pradesh/eight-killed-in-car-truck-collision-in-barabanki/article70241421.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:30:18 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/news/national/gfvskd/article70241478.ece/alternates/LANDSCAPE_1200/Accident%20stock.jpeg</t>
+  </si>
+  <si>
+    <t>EBC voters hold the key to Bihar polls, Nitish remains their preferred choice</t>
+  </si>
+  <si>
+    <t>For Kaushalendra Chouhan, a daily wage labourer from Makhdumpur, work is erratic, often requiring him to travel long distances. Yet he claims that travel has become easier and far safer under the present government. “There is no fear of being robbed while travelling at night,” he says.
+Some 250 km at the Keoti Assembly constituency, Ram Nath Thakur says life has not materially changed for him. He works in Kolkata and has returned home for the festivals and elections. He is a barber by profession and caste. “One can’t make a living here. There are hardly any customers here,” he says.
+Mr. Chouhan and Mr. Thakur are both from the Extremely Backward Class (EBC), a diverse group of castes comprising 36% of the State’s population, as per the caste count in Bihar. This group is entirely Bihar Chief Minister and Janata Dal (United) leader Nitish Kumar’s creation, ostensibly for ensuring better reach of welfare policies. This classification is based on a reservation policy of 1978 implemented by Karpoori Thakur.
+Thakur, a Nai (barber) by caste, remains the tallest EBC leader in the State. He reserved 26% of new government positions for “Backward Classes”, in addition to existing quotas for Scheduled Castes and Adivasis (24% combined). The Backward Classes were further divided into two lists. Annexure I, who among the backwards were economically and socially worse off, got 12% reservation and 8% for Annexure II communities who were socially better placed. The Annexure II is now categorised as Other Backward Classes and include the Yadavs among others. The EBC has historically been loyal to Mr. Kumar. The Mahagatbandhan’s success in the upcoming elections will largely depend on its ability to win over a portion of this crucial vote bank.
+In the last two decades that Mr. Kumar has been in power, Mr. Chouhan’s and Mr. Thakur’s economic condition has not significantly improved. Yet, their electoral choice remains unchanged. Both have voted for the NDA in the past elections and continue to do so. Their choices are based partly on aversion for the Rashtriya Janata Dal (RJD) and partly on their loyalty for Mr. Kumar.
+In the 2020 Assembly elections, the victory margin was less than 5,000 in 52 of the 243 constituencies in Bihar. Even a minor shift in caste-based political loyalties could change the results.
+The Hilsa constituency in Nalanda district exemplifies this volatility. In the 2020 election, JD(U) won the seat. “People’s mandate was in my favour,” RJD leader Atri Muni says. He had been declared victor by a margin of 549 votes at 5 p.m. The JD(U)’s candidate Krishnamurari Sharan congratulated Mr. Muni and left the counting centre. But an hour later, Mr. Sharan was declared the winner with a difference of 12 votes. Mr. Muni had challenged the result, but the Patna High Court took three-and-a-half years to admit the plea, only to eventually dismiss it.
+Mr. Muni reels off the caste arithmetic of Hilsa: with Yadavs and Kurmis evenly matched, the fragmented EBC vote will once again be decisive.
+But not all are happy. Birendra Mistri is upset at the bribes he has to pay to get any paperwork done in the block office. He comes from the Badai caste that falls under EBC group. “Nitish stands for caste-based politics. He has filled the departments with officials from his caste… all his policies are limited to the paper. Nothing translates on the ground,” he says. Having voted for the JD(U) in multiple elections, he is now looking for options.
+Rajesh Kumar Sahu, also an EBC, nods along to Mr. Mistri’s appraisal. He runs a small grocery shop. The business has been slow. His quibble with the government is the mass migration. “If everyone leaves, then how will I have customers,” Mr. Sahu says. He too, like Mr. Mistri, is looking for options, but he rules out the RJD. “I could vote for Jan Suraaj,” he replies after thinking for a while. He is familiar with Jan Suraaj founder Prashant Kishor, but the candidate for Hilsa is not a familiar face. “I will see closer to the election, depending on which way everyone is voting,” he says.
+RJD, though aware of its limitation in breaking Mr. Kumar’s stranglehold, has only 13 EBC candidates, as opposed to JD(U) which has 21. The Mahagatbandhan this time has two EBC parties – Mukesh Sahani’s Vikashsheel Insaan Party that represents the Mallahs and Nishads, and I.P. Gupta’s Indian Inclusive Party that represents Tanti-Pan Samaj. But whether these relatively new entrants can mobilise enough support to shift the balance remains to be seen.
+For now, Nitish Kumar continues to be the preferred choice for a majority of EBC voters.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/elections/bihar-assembly/ebc-voters-hold-the-key-to-bihar-polls-nitish-remains-their-preferred-choice/article70240667.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:21:06 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/4irvh2/article70241485.ece/alternates/LANDSCAPE_1200/20251103256L.jpg</t>
+  </si>
+  <si>
+    <t>After visit to Vantara, global wildlife committee recommends India pause animal import</t>
+  </si>
+  <si>
+    <t>A committee of CITES, the globe’s most influential agreement on wildlife conservation, whose strictures on the cross-border movement of protected animal species inform national wildlife laws, has recommended that India’s wildlife authorities pause the issue of permits that allow endangered animals to be imported by zoos, and wildlife rescue and rehabilitation centres.
+This, CITES says, should be in place until India comprehensively reviews its practices and ensures that “due diligence is exercised systematically and consistently”, and animal trade is not carried out in “violation of the Convention”.
+India became a signatory to the Convention on International Trade in Endangered Species of Wild Flora and Fauna (CITES) in 1976. Currently, 185 countries are signatories.
+The recommendations are part of a report prepared by a CITES-designated committee after a visit to the Greens Zoological Rescue and Rehabilitation Centre (GZRRC) in Jamnagar, a part of the Vantara animal rescue and rehabilitation centre affiliated to the Reliance Foundation. The Radha Krishna Temple Elephant Welfare Trust (RKTEWT) is also a part of Vantara, and while primarily focussed on elephant welfare, also has permissions to manage other imported species of fauna.
+In September, a Supreme Court-appointed Special Investigation Team, constituted to conduct an “independent factual appraisal” of complaints against Vantara, said it found no statutory irregularities in the acquisition of animals.
+The CITES committee found that the facilities in Vantara kept “exceptionally high standards”, and had “advanced facilities” with appropriate “veterinary care standards”. It also noted that it “could not find evidence” that the facility brought in animals for commercial purposes nor evidence that animals being imported to India lacked import, export, and re-export CITES permits.
+However, the committee’s report, uploaded on October 31 on the CITES website, noted that “...several imports [by GZRRC and RKTEWT] still raise questions regarding the origin of the specimens… the use of source and purpose-of-transaction codes, and the exercise of due diligence by India”.
+The committee visited Vantara from September 15-20, after it was asked by the CITES Secretariat to look into India’s processes for verifying whether the manner in which live animals were procured reflected the conditions under which they were sourced (for example, ‘W’ — from the wild, or ‘C’ — bred in captivity) and purpose-of-transaction (’Z’ — to be placed in a zoo, or ‘B’ — breeding in captivity).
+The visit was following a 2023 recommendation by the Secretariat to look into “trade in live animals with purpose code Z” by the GZRRC.
+In the last two years, there have been several journalistic investigations into procurement practices at Vantara, as well as reports by environmental groups that alleged animals were being procured in large numbers, both within India and from abroad, in ways that contravened the CITES stipulation.
+The GZRRC is registered as a zoo, rescue centre, a conservation breeding centre, and a centre for studying animals. Under Indian laws, a “zoo” cannot function as a licensed dealer in captive animals. Moreover, rescued or confiscated animals shall not be displayed to the public.
+Under CITES conventions, it is legal to trade animals commercially, provided relevant conditions are met, and permits state so explicitly. It is also permissible to buy animals for the purposes of breeding in captivity for conservation purposes, provided paperwork attests to it, and it is registered under appropriate rules of the Convention.
+The CITES committee’s reservations stemmed from observations where permit codes did not appropriately reflect the arrangement between the exporting country and India.
+The GZRRC, for instance, imported several animals from the Republic of Czechia.
+That country, according to the committee, “had no doubts” that the animals were being “sold” to the GZRRC and were not exported for the “purpose of rescue”. The Czech authorities provided invoices showing lists of animals acquired, price per unit, and taxes.
+The GZRRC’s interpretation, however, was that the animals weren’t “sold”, and the expense involved was the “cost of insurance, freight and customs duties”. India’s wildlife authorities, in explaining this, cited a Supreme Court order of September 15 that said these were indeed costs as the GZRRC said so, and another order said that if an animal was procured under a “valid” export permit, it couldn’t be a contravention of Indian law or the CITES.
+In a case involving the import by the GZRRC of two captive-bred snow leopards from Germany, the latter issued permits under the codes ‘C’ (origin as captive bred) and ‘T’ (for commercial purposes). When the animals reached India, the Indian authorities raised a query on the purpose of import (because of the ‘T’ label). The GZRRC said the animals were ‘donated’ by a facility in Germany. Following this, the Indian authorities changed the ‘T’ label to a ‘Z’ (zoological). The committee said that India ideally ought to have checked with German authorities, their reason for labelling it a commercial transaction instead of “only relying on the information by the importer (GZRRC)”.
+The committee highlighted an instance where Indian authorities issued permission allowing the import of chimpanzees from Cameroon by the GZRRC. It later turned out that the export permits by Cameroon were forged. The GZRRC did not proceed with the import as it couldn’t verify the antecedents of the chimpanzees at the Cameroonian facility. The committee noted that, ideally, Indian authorities should have known that, based on the CITES database, which they can access, Cameroon has not traded any chimpanzees since 2000, and there was no captive breeding of chimpanzees ongoing in that country.
+“The fake permits brought to the attention of the Secretariat may suggest that the large number of acquisitions of live animals by the GZRRC.. has attracted attention, and that certain individuals or entities could attempt to exploit this as a way to traffic animals. This shows that there is a need for caution to ensure that imports of large numbers of animals by these facilities are not inadvertently creating a demand for illegally sourced animals. Reinforced due diligence in this regard is crucial,” the committee noted.
+There were a litany of similar other examples raised by the committee on imports that were permitted by the Indian authorities of hundreds of animals. Indian authorities seemed to be acknowledging these lapses. “...Representatives from India...expressed appreciation for the guidance provided on these issues and confirmed that they would work on improving their processes and procedures. The Indian Management Authority has reiterated this commitment in writing in its submission to the Secretariat for the preparation of the present document. The management of the GZRRC also indicated their willingness to be in full compliance with CITES and to develop their own due diligence approach,” the committee report noted.
+The Hindu reached out with detailed questionnaires to Vantara, and the Union Ministry of Environment, Forest and Climate Change for comment but had not heard back till the time of going to press.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/sci-tech/energy-and-environment/after-visit-to-vantara-global-wildlife-committee-recommends-india-pause-animal-import/article70241099.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:18:00 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/6w0de1/article70241464.ece/alternates/LANDSCAPE_1200/IMG_vantaraelephant_2_1_6SETEGBD.jpg</t>
+  </si>
+  <si>
+    <t>7 years on, 2 convicted for killing private firm employee in road rage incident</t>
+  </si>
+  <si>
+    <t>The Additional City Civil and Sessions Court on Monday convicted and sentenced two youths to rigorous life imprisonment for allegedly bludgeoning a 25-year-old private firm employee to death over a trivial road rage incident in the limits of the Mico Layout police station limits seven years ago.
+Coincidentally, the verdict came on the birthday of the victim, Siddarth Koushal, a native of Bihar, who was working for a private firm in the city.
+According to the prosecution, Siddarth and his friend — who owned a restaurant in Electronics City — were returning home in a car on June 26, 2018 around 3 a.m. after closing the eatery. Two of their friends followed them on a bike. The duo had stopped the car by the roadside to relieve themselves when the accused — Girish, son of a builder, and his friend Mahesh — brushed their bike against the car.
+An argument broke out after Siddarth noticed a dent and shouted at them. Enraged, the duo allegedly returned, picked up a stick lying nearby, and attacked Siddarth. By the time his friends rushed to his rescue, the assailants had fled, leaving him grievously injured.
+A nearby paan beeda shop owner, who was sleeping outside his shop near a bar and restaurant, woke up to the commotion and recognised one of the attackers. Siddarth, who was profusely bleeding, was rushed to a private hospital, where he succumbed to injuries later.
+Based on a complaint, then the Mico Layout Inspector, R.M. Ajay, registered a case of murder and, with the help of the shop owner’s statement, tracked down Girish and later arrested Mahesh. The police collected technical evidence and witness statements before filing a charge sheet in the court.
+While Girish remained in judicial custody due to the gravity of the offence, Mahesh was released on bail. During the trial, several eyewitnesses, including the paan shop owner and two of Siddarth’s friends, turned hostile, causing delays in the proceedings. However, strong technical evidence and the effective arguments of Public Prosecutor Mahalingappa ensured the conviction of both accused.
+Siddarth’s father, Koushalendra Kumar, an advocate by profession, attended every hearing, even during the COVID-19 lockdown. Following the verdict, he met the police team and distributed sweets as a gesture of gratitude.
+“Siddarth was my elder son. We have not celebrated any festival since his death, but today we lit a lamp after the judgment,” Mr. Kumar told the police team.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/7-years-on-2-convicted-for-killing-private-firm-employee-in-road-rage-incident/article70240915.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:17:24 +0530</t>
+  </si>
+  <si>
+    <t>SCTIMST an inspiration for all government institutions in the country: Vice-President</t>
+  </si>
+  <si>
+    <t>Vice-President C.P. Radhakrishnan has hailed the Sree Chitra Tirunal Institute for Medical Sciences and Technology (SCTIMST), which has performed heart valve surgeries on nearly two lakh patients, as an inspiration for all government institutions in the country.
+Research becomes a true success only when it touches common people and creates a larger and meaningful impact on society, a goal that the SCTIMST has achieved commendably, Mr. Radhakrishnan said.
+The Vice-President was addressing a gathering on Tuesday after visiting the SCTIMST’s newly inaugurated hospital building under the Pradhan Mantri Swastha Suraksha Yojana (PMSSY), which boasts high-end medical infrastructure, sophisticated medical equipment and expanded intensive care unit facilities.
+He also visited the medical exhibition arranged at the SCTIMST, showcasing the medical innovations and new technologies indegenously developed at the Institute. He said that the government’s ultimate goal was health for all and called for better services to the poorest of the poor.
+Governor Rajendra Vishwanath Arlekar, Union Minister of State for Petroleum, Natural Gas, and Tourism Suresh Gopi, State Finance Minister K.N. Balagopal, and SCTIMST Director Sanjay Behari also addressed the meeting.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/kerala/sctimst-an-inspiration-for-all-government-institutions-in-the-country-vice-president/article70241346.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:15:24 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/1i2jyy/article70241369.ece/alternates/LANDSCAPE_1200/20251104172L.jpg</t>
+  </si>
+  <si>
+    <t>MLA allegedly ousted from inaugural function</t>
+  </si>
+  <si>
+    <t>Kerala Pradesh Congress Committee president and Peravoor MLA Sunny Joseph was allegedly ousted from a function by Communist Party of India (Marxist) [CPI(M)] workers while he was inaugurating the Chavassery road project in Irrirty municipality on Tuesday.
+Mr. Joseph maintained that since the road work was funded by the government, the local legislator should inaugurate it as per official protocol. However, CPI(M )workers allegedly raised slogans against him, forcing him to leave the venue.
+Addressing supporters at a nearby venue later, the MLA said funds to renovate the road in the Peravoor Assembly constituency were sanctioned following complaints raised during the Navakerala Sadas.
+Meanwhile, CPI(M) workers alleged that the MLA had boycotted the Navakerala Sadas and was now attempting to claim credit for the project. Following the protest, the road was inaugurated by the Irrity municipal chairperson.
+Mr. Joseph said that he attended the function in his capacity as a people’s representative. He added that the road project received administrative sanction on September 19 this year and dismissed the CPI(M)’s claim that the approval came in 2024. The MLA said he had proposed ₹5.75 crore for Kakkayangad-Palapuzha road and ₹1.5 crore for Chavassery road, and that the government approved the projects accordingly.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/kerala/mla-allegedly-ousted-from-inaugural-function/article70239641.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:14:55 +0530</t>
+  </si>
+  <si>
+    <t>SP renews push for full-fledged AMU centre in Kishanganj as Akhilesh’s Bihar campaign gathers pace</t>
+  </si>
+  <si>
+    <t>As Samajwadi Party (SP) president Akhilesh Yadav campaigns extensively in Bihar for the Assembly polls, his party on Tuesday reiterated its demand for the completion and full functioning of the satellite branch of Aligarh Muslim University (AMU) in Kishanganj district of Bihar.
+The party described the educational backwardness of the Seemanchal region, of which Kishanganj is a part, as the primary cause of its economic underdevelopment and that of Bihar. It added that the SP is keen to address Seemanchal’s developmental needs, calling for a broader solidarity of socialist and democratic forces to create world-class educational infrastructure.
+“We did advocate for the AMU Kishanganj campus, aligning with our broader social justice and PDA rights agenda. Bureaucratic hurdles such as land acquisition and thus infrastructure planning contributed to the delay. The SP is keen to address Seemanchal’s development, especially after the Sachar Committee Report, raising this issue for which the SP stands for its secular and socialist ideologies and being the third largest party in Parliament is playing the role of a national-level secular alternative. Championing AMU Kishanganj will serve as a symbolic and substantive commitment to educational equity,” SP spokesperson Naseer Salim said.
+Mr. Salim, who is the great-grandson of Lady Anees Imam, one of the founders of modern Bihar who played a distinctive role in the anti-colonial movement before Independence, added that the PDA (Pichhda, Dalit, Alpsankhyak) plank, which also includes aadhi aabadi (women) and upper castes, remains central to the SP’s vision.
+The AMU Kishanganj campus remains incomplete even after more than a decade, operating from temporary buildings with only one functional course. The branch, established in 2011 as part of a nationwide initiative for higher education among Muslim populations following recommendations by the Ministry of Human Resource Development, currently functions from a temporary structure at Halim Chowk in Kishanganj.
+The Seemanchal region is considered one of the most backward parts of India in terms of education and nearly all other indices of human development.
+Another senior SP leader and national spokesperson, Ram Pratap Singh, said, “The PDA ideology of the Samajwadi Party is for creating infrastructure and delivery of world-class education at all levels. This would mean that we not only have to strengthen our existing institutions of higher learning but replicate successful models across the country.”
+Mr. Yadav is currently campaigning across Bihar, addressing multiple rallies daily in support of INDIA bloc candidates.
+Speaking about the activism of Lady Anees Imam, Mr. Salim said, “Lady Anees Imam’s activism was deeply intertwined with social reform and the educational upliftment of women in Bihar. Her struggle was not just political; it was cultural and educational, aimed at transforming the mindset of a society that had long excluded women from public and intellectual life.
+“Lady Imam was among the first Muslim women in Bihar to publicly reject purdah, challenging entrenched patriarchal norms across both Hindu and Muslim communities. She founded institutions like Aghor Kamini Shilpalaya and Aghor Nari Pratishan, which provided industrial and vocational education to women, especially in Patna and surrounding regions. Her struggle was not just about resisting colonial rule; it was about reshaping society from within, empowering women to become agents of change.”
+Asked whether Lady Imam contributed to the anti-colonial movement in the United Provinces, present-day Uttar Pradesh, Mr. Salim said her primary base was Bihar, though her influence extended beyond regional boundaries.
+“She led a delegation to England on behalf of the All-India Congress to oppose the Montague-Chelmsford Reforms of 1919, a national-level intervention that impacted policies across British India, including the Hindi belt. Her contributions were more national in scope, rather than geographically centred in the Hindi belt. Her work bridged elite and grassroots activism, showing that upper-caste Muslim women could be powerful agents of change in a deeply stratified society,” the SP spokesperson said.
+When asked whether the magnitude of social injustice against women has declined in recent decades or merely reinvented itself, SP national spokesperson Ram Pratap Singh said, “Yes and no is my answer. Yes, education, healthcare and social welfare have marginally become better. More is being talked about to generate political optics but in real terms the delivery on the ground is a distant dream. The West-inspired model of development of the last two decades has not created any significant opportunities for women, as is evident from an abysmally low, around 15%, female participation in the labour force in most Indian States. Rural infrastructure, which impacts women the most, has also not much improved.”</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/bihar/sp-renews-push-for-full-fledged-amu-centre-in-kishanganj-as-akhileshs-bihar-campaign-gathers-pace/article70240274.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:13:36 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/news/national/erscb1/article70241434.ece/alternates/LANDSCAPE_1200/THJVNALIGARHMUSLIMUNIVERSITY.jpg</t>
   </si>
   <si>
     <t>Karnataka releases a new Skill Development Policy; to train 3 million youth by 2033</t>
@@ -111,9 +375,6 @@
     <t>Tue, 04 Nov 2025 21:57:50 +0530</t>
   </si>
   <si>
-    <t>https://www.thehindu.com/theme/images/og-image.png</t>
-  </si>
-  <si>
     <t>Governor approves selection panel constitution for Calicut University V-C</t>
   </si>
   <si>
@@ -204,262 +465,6 @@
     <t>https://th-i.thgim.com/public/incoming/l2s16c/article70241337.ece/alternates/LANDSCAPE_1200/CCI_UDHindu_KSL_UDN326GBK_R1513333355_1_ddd1a627-152b-41f7-b20d-5505142318b1.jpg</t>
   </si>
   <si>
-    <t>Maharashtra announces ₹2.25 crore each for Jemimah, Smriti and Radha Yadav</t>
-  </si>
-  <si>
-    <t>The Maharashtra government on Tuesday announced a cash prize of ₹2.25 crore each for the State’s players in the Indian women’s cricket team that won the ICC Women’s World Cup recently.
-As per the State government’s policy, Jemimah Rodrigues, Smriti Mandhana and Radha Yadav will be given the cash award and felicitated by the government. Coach Amol Muzumdar, who hails from Mumbai, will receive a cash prize of ₹22.5 lakh.
-“Today, the Cabinet has passed a resolution to congratulate the women’s cricket team which has done a glorious job of winning the ICC World Cup. Similarly, three players from Maharashtra, Jemimah Rodrigues, Smriti Mandhana and Radha Yadav, will be felicitated by the Maharashtra government and will be given a cash prize as per our policy. They have made the country proud,” Chief Minister Devendra Fadnavis said on Tuesday, adding that the government will also felicitate the entire women’s cricket team when it visits Mumbai.
-As per the government’s sports policy, players winning gold medals in the Olympics or Paralympics receive ₹3.75 crore each, while their coaches are awarded ₹37.5 lakh. Those winning gold in World Cups, World Championships or Para World Championships are given ₹2.25 crore each, with coaches receiving ₹22.5 lakh.
-Athletes winning gold in the Asian Games or Commonwealth Games are given ₹75 lakh each, while Chess Olympiad champions receive ₹1 crore.
-India recently won its first ICC Women’s Cricket World Cup, defeating South Africa by 52 runs in the final played at Navi Mumbai. Shafali Verma was named Player of the Match, and Deepti Sharma was declared Player of the Tournament.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/maharashtra/maharashtra-announces-225-crore-each-for-jemimah-smriti-and-radha-yadav/article70241131.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:42:23 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/news/national/lsc2u5/article70241237.ece/alternates/LANDSCAPE_1200/TH04-LEAD-WC-WRGP5F47431.3.jpg.jpg</t>
-  </si>
-  <si>
-    <t>Trying to establish aviation varsity near Bhogapuram airport, says Union Minister</t>
-  </si>
-  <si>
-    <t>VIZIANAGARAM:
-Union Minister for Civil Aviation K. Rammohan Naidu on Tuesday said that the Centre was making all efforts to establish an Aviation University adjacent to the Bhogapuram international airport, which is expected to be ready within six months.
-After reviewing the construction progress, he said that 91.7% of the project works have been completed through the joint efforts of the Union and the State governments.
-He shared that the trial run of the first flight would likely take place in December 2025 or January, 2026. Mr. Rammohan Naidu hoped that the airport would spur economic activity, as it was evident with the on-going construction of several star hotels between the Bhogapuram-Vishakhapatnam route.
-The minister also said that an aviation university would transform the area into a prominant academic hub.
-Vizianagaram MP Kalisetti Appala Naidu, Bhogapuram MLA Lokam Madhavi, Vizianagaram Collector S.Ramsundar Reddy and others participated in the site review.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/andhra-pradesh/trying-to-establish-aviation-varsity-near-bhogapuram-airport-says-union-minister/article70240677.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:41:33 +0530</t>
-  </si>
-  <si>
-    <t>Two arrested for running fraudulent gold loan scheme; gold worth ₹1.8 crore seized</t>
-  </si>
-  <si>
-    <t>Bengaluru
-The Central Crime Branch (CCB) Economic Offences Wing arrested two persons for allegedly running a fraudulent ‘0% interest gold loan’ scheme in the city.
-According to the police, the accused, identified as Salaam and Ajith, had opened a jewellery shop in Vidyaranyapura and lured customers by offering gold loans at 0% interest. Believing the offer, several people pledged their ornaments but received only 50% to 60 % of the actual value. They were also told not to redeem their jewellery for at least 11 months.
-During that period, the accused allegedly sold the pledged gold to another jewellery shop in HRBR Layout, making a profit of 40% to 50%. The accused later shut down the shop and went absconding after allegedly misappropriating around 4 kg of gold, the police said.
-The CCB traced and arrested the main accused from his residence in Peenya. From the HRBR Layout shop, officers seized 1.47 kg of gold ornaments and 5 kg of silver items, together valued at about ₹1.8 crore.
-Preliminary investigations have revealed that the accused were involved in similar fraudulent activities in Mangaluru district and in Kerala.
-Public advisory
-City Police Commissioner Seemant Kumar Singh advised people to be careful while dealing with gold loan firms. Before pledging gold, the public is advised to verify the authenticity and license of the financial institution. “Do not fall prey to deceptive schemes such as ‘0% interest loans’. If any suspicious or fraudulent schemes are noticed, please inform the nearest police station or CCB Economic Offences Wing immediately,” he said.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/two-arrested-for-running-fraudulent-gold-loan-scheme-gold-worth-18-crore-seized/article70239266.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:41:02 +0530</t>
-  </si>
-  <si>
-    <t>Expedite Vijayawada airport expansion works, Collector tells officials</t>
-  </si>
-  <si>
-    <t>Krishna District Collector D.K. Balaji has instructed officials to expedite the expansion and development works of Vijayawada International Airport at Gannavaram and ensure their completion within the stipulated timeframe.
-Chairing a review meeting with officials of various departments at the airport on Tuesday (November 4), Mr. Balaji directed them to prepare and submit proposals to the government for additional works as per prescribed guidelines. He also urged officials to resolve issues related to land acquisition, court disputes, construction of a bridge over the Eluru canal, and payment of compensation to farmers at the earliest.
-According to a press note issued by the district administration, the meeting discussed the progress of the new integrated terminal building, ceiling and elevation works, vehicle parking, drainage, and other infrastructure facilities, along with pending land acquisition matters. Airport officials gave a detailed presentation to the Collector on the status of ongoing works.
-Later, Mr. Balaji inspected the under-construction integrated terminal building, reviewed the pace of work on-site, and expressed satisfaction with the progress achieved so far. Officials from the Airports Authority of India, Revenue, Panchayat Raj, Irrigation, Drainage, Rural Water Supply (RWS), and Roads and Buildings departments participated in the meeting.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/andhra-pradesh/expedite-vijayawada-airport-expansion-works-collector-tells-officials/article70241092.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:40:57 +0530</t>
-  </si>
-  <si>
-    <t>Seminar on leadership for school Principals, head teachers begins</t>
-  </si>
-  <si>
-    <t>School leaders should be lifelong learners, facilitators of change, and catalyst for collaboration, Shashikala Wanjari, Vice-Chancellor, National Institute of Educational Planning and Administration (NIEPA), has said.
-She was delivering the keynote address on the theme ‘Leadership pathways for school improvement’ at a three-day ‘Inter-School Leadership Academy Regional Seminar of South Indian States on School Leadership’ in the State capital on Tuesday.
-Collaboration, Prof. Wanjari said, resulted in synergy that generated innovative ideas. She observed that as the education system evolved in response to socio-economic and technological changes, the role of school leaders had become more complex, dynamic, and critical than ever before. Earlier, school leadership was looked at from an administrative and managerial lens. Today, it was recognised as a transformative force, requiring vision, empathy, innovation, and the ability to mobilise people and resources in order to provide quality education.
-She also stressed the need for investing in professional development of school leaders on a continuous basis to enable knowledge sharing, supporting each other, and improving collective practices and outcomes.
-Director of General Education N.S.K. Umesh was the special guest at the seminar in which SIEMAT-Kerala Director Jayaprakash R.K. delivered the introductory speech. State Institute of Educational Technology Director B. Aburaj also spoke.
-The seminar has been organised by the School Leadership Academy – Kerala under the State Institute of Educational Management and Training – Kerala (SIEMAT-Kerala) in collaboration with the National Centre for School Leadership-NIEPA as part of initiatives to strengthen leadership capacity in school education.
-Representatives from Kerala, Tamil Nadu, Karnataka, Andhra Pradesh, Telangana, and Lakshadweep are attending the seminar that will include case study and empirical research presentations.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/kerala/seminar-on-leadership-for-school-principals-head-teachers-begins/article70241197.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:37:46 +0530</t>
-  </si>
-  <si>
-    <t>India, Israel sign MoU to deepen defence cooperation</t>
-  </si>
-  <si>
-    <t>India and Israel have taken a significant step forward in strengthening their long-standing defence partnership with the signing of a Memorandum of Understanding (MoU) on Defence Cooperation during the 17th Joint Working Group meeting held in Tel Aviv on Tuesday (November 4, 2025).
-The meeting was co-chaired by Defence Secretary Rajesh Kumar Singh and the Director General of the Israeli Ministry of Defence Major General (Res) Amir Baram.
-The MoU provides a unified framework and policy direction to further collaboration across multiple domains, including strategic dialogues, training, defence industrial cooperation, research and development, Artificial Intelligence (AI), cyber security, and technological innovation, the Ministry of Defence said. It aims to facilitate co-development, co-production, and sharing of advanced defence technologies between the two nations, it said.
-During the meeting, both sides reviewed ongoing initiatives and acknowledged that India and Israel have mutually benefited from their cooperation. The delegations discussed potential areas for future collaboration to bolster technological capabilities and operational preparedness.
-They also reaffirmed their joint commitment to combat terrorism and address shared security challenges, underscoring the deep mutual trust and shared strategic interests that continue to define the India-Israel defence relationship.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/india-israel-sign-mou-to-deepen-defence-cooperation/article70240946.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:35:37 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/news/national/q8g4s9/article70241276.ece/alternates/LANDSCAPE_1200/India%20Israel.jpg</t>
-  </si>
-  <si>
-    <t>Telangana bus-lorry crash: Tipper driver’s attempt to avoid pothole led to collision, says DGP</t>
-  </si>
-  <si>
-    <t>A day after the collision between a Telangana State Road Transport Corporation bus and a gravel-laden tipper lorry that left 19 people dead in Chevella, police have begun probing the permits, load capacity and operational condition of the lorry involved.
-Telangana Director General of Police B. Shivadhar Reddy, who inspected the spot on Tuesday, said that initial inquiries pointed to a driving error. “He tried to avoid a small pothole, swerved slightly to the right and collided with the bus. Otherwise, we do not see any issue with the road — the curve is not sharp, there are no trees blocking visibility and no other obstructions,” he said.
-The police are also examining the mechanical condition of the tipper lorry, including its engine and braking system, to determine whether any malfunction contributed to the crash. Tissue samples from both drivers have been sent to the Telangana Forensic Science Laboratory on Tuesday. “Samples have been sent to verify if any of the drivers were in an inebriated condition. That will be an important aspect of the investigation,” said Cyberabad Police Commissioner Avinash Mohanty.
-Preliminary findings also suggest that the Ashok Leyland 10-wheeler tipper was carrying between 60 and 70 tonnes of gravel, double its maximum capacity. Investigators suspect the excessive weight may have played a crucial role in the severity of the crash, which was reported on the narrow stretch of the Hyderabad-Tandur highway near Mirjaguda on Monday morning.
-“We are verifying the vehicle’s documents, the trail of transactions and the weight of the gravel loaded at Lakdaram in Patancheru, before it began its journey towards Manneguda via Shankarpally,” an officer involved in the investigation told The Hindu. “The possibility of overload cannot be ruled out.”
-Interestingly, in a statement to the police, the lorry owner, Lachiram Naik, who survived the crash with severe injuries, claimed that he had handed over the vehicle to driver Akash Danya Kamle near Shankarpally. He added that Kamle had been driving continuously for long hours without adequate rest. Less than two hours after the journey began, the tipper rammed into the RTC bus.
-Of the 72 passengers on board the bus, 38 were treated for injuries, while several others who escaped with minor or no wounds fled the site in shock. The Chevella police have urged these passengers to come forward and record their statements to aid the investigation.
-Monday’s collision, among the deadliest in recent months, occurred when the gravel-laden lorry heading from Shankarpally via Tandur collided head-on with the RTC bus traveling in the opposite direction. The impact crushed the front portion of the bus, causing the lorry’s load to spill over and trap passengers inside.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/cities/Hyderabad/police-probe-overloaded-vehicle-permits-in-chevella-crash-that-killed-19-drivers-samples-sent-to-fsl-to-rule-out-drunk-driving/article70240990.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:35:00 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/c2h77h/article70240987.ece/alternates/LANDSCAPE_1200/Chevella%20Bus%20Accident%2021.jpg</t>
-  </si>
-  <si>
-    <t>NDA government in Bihar neglected women’s safety, health: Congress</t>
-  </si>
-  <si>
-    <t>The Congress on Tuesday (November 4, 2025) accused the BJP–JD(U) government in Bihar of showing “consistent neglect” towards women’s safety, health, and dignity over the last two decades, while posing a set of questions to both Prime Minister Narendra Modi and Chief Minister Nitish Kumar.
-Party president Mallikarjun Kharge slammed the NDA government in Bihar over the security situation for women and asserted that the Mahagatbandhan (grand alliance)was fully committed to empowering and uplifting them.
-Also Read: Bihar Assembly polls Highlights on November 4, 2025
-Mr. Kharge said the Congress’ promises were not just to garner votes during elections or right before them, but rather, they were the same promises that the party would fulfil.
-“The BJP-JDU government in Bihar has been in power for 20 years. If even today, Modi ji has to say that in Bihar ‘daughters-in-law and daughters are not safe’, then this is his own self-admission that in 20 years, they have not made Bihar safe!” Mr. Kharge said in a post in Hindi on X.
-The Congress chief said the situation of women and children was extremely alarming and cited the National Family Health Survey (NFHS) data to say 70% of children were afflicted with anaemia and 40% were victims of malnutrition. Only 11% of infants received adequate nutrition as per the NHFS survey, he said.
-Listing the promises made to women by the grand alliance, Mr. Kharge said they would be given an assistance of ₹2,500 per month if the Opposition alliance came to power. A monthly pension of ₹1,500-3,000 would be given to the elderly, widows, and disabled, he added.
-Congress communication chief Jairam Ramesh, in a separate X post, said the Prime Minister “didn’t remember to check on Bihar’s women for an entire decade” and was now “staging a sham digital outreach for votes.”
-He alleged that the NDA government had failed women on every front — from safety and health to economic security. Mr. Ramesh claimed that crimes against women had increased by 336% under the BJP–JD(U) regime, with around 20,222 incidents reported annually and 2.8 lakh women victimised so far. He said 1,17,947 cases remained pending in Bihar’s courts, resulting in a 98.2% pendency rate, “the highest in the country.”
-“Despite record-breaking crimes against women, why has the BJP–JD(U) government failed to provide them security?” Mr. Ramesh asked.
-Quoting the NFHS, the Congress leader said the health condition of women and adolescent girls was “alarming,” with over 63% of women and 65.7% of adolescent girls suffering from anaemia. “Despite such a massive health crisis for women, why has the government turned a blind eye?” Mr. Ramesh said.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/elections/bihar-assembly/nda-government-in-bihar-neglected-womens-safety-health-congress/article70240662.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:34:59 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/wmfbel/article70241279.ece/alternates/LANDSCAPE_1200/20251103402L.jpg</t>
-  </si>
-  <si>
-    <t>Lokesh holds 70th consecutive Praja Darbar, assures swift action on grievances</t>
-  </si>
-  <si>
-    <t>Education and IT Minister Nara Lokesh held his 70th consecutive Praja Darbar at the TDP central office in Mangalagiri on Tuesday, drawing citizens and party workers from across Andhra Pradesh.
-Mr. Lokesh interacted with visitors, patiently listening to their appeals and issuing on-the-spot directions to officials. He reiterated that the coalition government is fully committed to protecting citizens’ rights and ensuring justice for all.
-Complaints received during the programme included false cases and land grabbing during the previous YSRCP regime, encroachment of ancestral lands, and unjust job terminations. Mr. Lokesh assured each petitioner that the government would investigate their cases and deliver justice swiftly.
-Representatives of the Unemployed Paramedical Health Assistants (Male) Association urged the Minister to fill pending vacancies in the Health Department. Delegates from the Nallamala Chenchu Welfare Association sought new schools for tribal and forest regions, while members of the Power Employees Union requested regularisation of 23,500 contract workers in GENCO, TRANSCO, and DISCOMs. Mr. Lokesh said all such demands would be examined carefully.
-Requests for Chief Minister’s Relief Fund (CMRF) medical aid, a new government junior college in Chittoor, and action against illegal land encroachments in Vijayawada Rural were also received.
-Reaffirming his open-door policy, Mr. Lokesh said such people-oriented forums would continue to ensure transparent governance and timely grievance redressal across the State.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/andhra-pradesh/lokesh-holds-70th-consecutive-praja-darbar-assures-swift-action-on-grievances/article70241163.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:33:38 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/7bqh0e/article70241286.ece/alternates/LANDSCAPE_1200/Lokesh-to-underGMGF20RAE.3.jpg.jpg</t>
-  </si>
-  <si>
-    <t>Man beaten to death  by wife’s family over marital dispute</t>
-  </si>
-  <si>
-    <t>A 36-year-old sales executive working with a telecom company was beaten to death allegedly by his wife and her family members over a domestic dispute in Kadugondanahalli on Tuesday.
-The deceased, Mohammed Shakeel, a resident of AMC Road in KG Halli, had been married to Raziya Sultan for 12 years. The couple, who have two sons, were reportedly facing marital discord and had filed for divorce, which was pending before a family court.
-According to police, around 4.30 p.m. on Saturday, Shakeel and his father Mohammed Samiuddin visited Raziya’s brother’s flat in an apartment behind Bilal Mosque to discuss a divorce settlement. During the meeting, Samiuddin was said to have urged Raziya’s family to finalise the settlement so that Shakeel could move on with his life.
-The discussion allegedly turned violent after Raziya’s family members got enraged. Her brothers reportedly attacked Shakeel, hitting him with helmets even after he collapsed. Shakeel succumbed to severe head injuries on the spot. Samiuddin later approached the K.G. Halli police and lodged a complaint.
-A case of murder has been registered against Zabiulla Khan, Imran Khan, Raziya Sultan, Fayaz Khan, and Mubeena Taj . The police have arrested Zabiulla, Imran, and Fayaz, while efforts are on to trace Raziya and Mubeena, a senior police officer said.
-Man hacked to death
-In another incident, an armed man allegedly hacked a 40-year-old businessman to death in Anekal on Tuesday.
-The deceased, identified as Madesh, a resident of Kachanayakanahalli, was a native of Tamil Nadu.
-According to the police, Madesh had gone to serve tea to the labourers constructing his house when the assailant barged in armed with a knife and an air gun, attacked him and slit his throat before fleeing the spot. Passers-by hearing the commotion tried to stop him, but the accused allegedly assaulted them and managed to flee. Upon receiving the alert, the Hebbagodi Police rushed to the spot and recovered an air gun, knife, metal detector, torch, helmet, and a bag left behind by the accused.
-Fingerprint experts and a dog squad were pressed into service to assist in the investigation.
-The police said Madesh had been residing in Bengaluru for the past 15 years, running a cigarette distribution business and a provision store and also owned a roadside eatery. He was building a new house using the proceeds from the sale of his ancestral property in Tamil Nadu. His family members were working at the tea stall.
-A special team has been formed to track down the assailant.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/man-beaten-to-death-by-wifes-family-over-marital-dispute/article70240153.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:32:47 +0530</t>
-  </si>
-  <si>
-    <t>Campaigning ends for 121 seats in the first phase of the Bihar Assembly election</t>
-  </si>
-  <si>
-    <t>As campaigning ended on Tuesday (November 4, 2025) for the first phase of the Bihar Assembly election, leaders of both the ruling NDA and the Opposition INDIA bloc went all out in their final appeal to voters in the 121 constituencies which will go to the polls on November 26.
-Both Union Home Minister Amit Shah and Leader of Opposition in the Lok Sabha Rahul Gandhi held three rallies each on a hectic final day, while the INDIA bloc’s Chief Ministerial candidate Tejashwi Yadav used a chopper to squeeze in visits to 17 constituencies in the final day of campaigning.
-The NDA trotted out the big guns with a slew of Union Ministers and BJP Chief Ministers while harping on a theme of corruption and jungle raj if the Opposition Rashtriya Janata Dal returns to power in the State. Mr. Gandhi and Mr. Yadav focussed on Bihar’s unemployed youth, asking why the NDA has failed to provide jobs despite many years in power in both the State and Centre.
-Warning against ‘jungle raj’
-Mr. Shah addressed three back-to-back public meetings in three different districts — Darbhanga, East Champaran, and West Champaran — covering nine Assembly constituencies. In Darbhanga, he attacked the Opposition Rashtriya Janata Dal (RJD), saying that Bihar has seen the jungle raj of ‘Lalu-Rabri’ for 15 years — referring to former Chief Ministers Lalu Prasad Yadav and his wife Rabri Devi — and nobody wants to bring those days back again.
-“Lalu ji did the fodder scam, land-for-job scam, hotel selling scam, bitumen scam, flood relief scam. Lalu-Rabri did so many scams and Congress has done scams worth ₹12 lakh crore. Can these people do any good for Bihar? Modi ji has ruled for 11 years and Nitish Babu has ruled for 20 years. There is not even a 4 paisa allegation of corruption against Nitish Babu and Modi ji,” he said, referring to Prime Minister Narendra Modi and Bihar Chief Minister Nitish Kumar. Mr. Shah also accused the INDIA bloc of conducting a Voter Adhikar Yatra to protect “infiltrators”.
-In Motihari, Mr. Shah warned that if any mistake happens on November 6, then kidnapping, ransom, and jungle raj will return to Bihar. “Lalu-Rabri wants to make their son [Tejashwi Yadav] the Chief Minister, and Sonia ji wants to make her son [Rahul Gandhi] the Prime Minister. I want to tell both of them that neither Lalu’s son will become the Chief Minister, nor will Sonia Gandhi’s son become the Prime Minister. In Bihar, Nitish ji is in the Chief Minister’s chair, and in Delhi, Modi ji is in the Prime Minister’s chair,” Mr. Shah asserted.
-‘Bihar’s development train’
-BJP president J.P Nadda pushed a development narrative during his rally in the Barhara seat, followed by a road show in Gaya. “It took 20 years for Bihar’s development train to get back on track, and now this train is moving forward rapidly. Therefore, this election is one that will bring stability to Bihar and connect it with development. We have taken Bihar from lanterns to LEDs,” he said.
-“The NDA talks about ‘development’, and these people [the Opposition] talk about ‘crime’. Wherever our government is formed, development happens there, not crime,” said Union Defence Minister Rajnath Singh, who addressed four public meetings in the Raghopur, Fatua, Simri Bakhtiyarpur, and Tarapur constituencies.
-Former Union Minister and Hamirpur MP Anurag Singh Thakur had a road show in Bankipur, along with Madhya Pradesh Chief Minister Mohan Yadav and Chhattisgarh Deputy Chief Minister Arun Saw, while Assam Chief Minister Himanta Biswa Sarma addressed a rally in Siwan.
-‘Jobs or reels’
-Congress leader Rahul Gandhi addressed three public meetings in the Aurangabad, Kutumba, and Wazirganj constituencies on the last day of the campaign, appealed to Bihar’s youth to voter for regime change, asking whether they want jobs or social media reels.
-Even after being in power for twenty years, Bihar CM Nitish Kumar has not done anything other than turning Bihar’s talented youth into labourers, forcing them to do menial work across the country, he said. Instead of talking about reels, the Prime Minister should have spelt out how he will provide employment, education, and better healthcare to people, Mr. Gandhi added.
-He claimed that Mr. Kumar is just the mask of the government, being manipulated by Mr. Modi and Mr. Shah. “His remote control is in their hands, and they make him act at their will, just like changing channels with a TV remote,” Mr. Gandhi said.
-He accused the BJP of spreading the venom of hatred across the country. “India is the land of love and this country cannot be run on hatred,” he said, promising that the Opposition Mahagathbandhan would form an inclusive and representative government including the extremely backward classes, backward classes, Dalits, Maha Dalits, minorities, and the general category as well.
-The INDIA bloc’s Chief Ministerial face, Tejashwi Yadav, managed to address public meetings in 17 Assembly constituencies on the final day of campaigning by using a helicopter. The Rashtriya Janata Dal (RJD) leader accused the JD(U) and BJP of ruining Bihar over the last 20 years and failing to tackle key issues like unemployment and migration.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/elections/bihar-assembly/campaigning-ends-for-121-seats-in-the-first-phase-of-the-bihar-assembly-election/article70240866.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:32:02 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/ypplzq/article70241273.ece/alternates/LANDSCAPE_1200/20251104147L.jpg</t>
-  </si>
-  <si>
-    <t>Halasuru gate police bust fake ₹2,000 notes racket, 10 arrested</t>
-  </si>
-  <si>
-    <t>Bengaluru
-Following a complaint from Reserve Bank of India (RBI) about fake currency notes, the Halasuru Gate Police busted a racket and arrested ten people for their alleged involvement in tampering with and selling ₹2,000 denomination notes withdrawn from circulation.
-According to the police, the RBI’s Manager filed a complaint on October 17, stating that ₹2,000 notes — already withdrawn from circulation — had been tampered with by changing their serial numbers before being deposited at the bank.
-Following the complaint, the police identified the depositor and arrested him from his residence in Cubbonpet on October 24.
-During interrogation, the accused allegedly revealed that he had deposited ₹40,000 worth of altered currency on behalf of two acquaintances, who promised him a commission. Based on his information, the police arrested both associates later near Mysore Bank Circle the same day.
-Further investigation revealed that the trio had received ₹8 lakh in ₹2,000 notes from three other individuals, who had convinced people to hand over such withdrawn notes under the pretext of performing a ‘special ritual’ that would ‘multiply’ their money hundredfold. The three men, arrested near Majestic Bus Stand on October 25, reportedly confessed to running the fraudulent scheme.
-Based on their information, the police apprehended three more suspects from Andhra Pradesh on October 28 and seized ₹6 lakh in ₹2,000 notes. The accused also disclosed the identity of their associate who had modified the serial numbers and printed details on the notes. He was traced to Yeshwantpur, where the police seized ₹6 lakh in fake ₹2,000 notes and equipment used to alter currency.
-In total, ₹18 lakh worth of fake ₹2,000 notes were seized in the case. All ten accused were produced before the court on November 3 and remanded in judicial custody. One female accused remains absconding, and efforts are under way to trace her.
-Explaining the modus operandi of the gang, the CCB officials said that it was a bizarre scam involving three men among the accused who posed as ‘swamis’ and tricked gullible people into believing they could bring a ‘rain of money’ through a special ritual using ₹2,000 denomination notes.
-The accused — identified as Basavaraj alias Satyananda Swami, Mallikarjun, and Mohan alias Muniswamy — would take turns dressing up as holy men to convince people that performing a ritual with specific series of ₹2,000 notes would multiply their money several times over.
-The trio told their victims that if they offered 100 notes of the (2018 HS series) ₹2,000 denomination, it would result in a miraculous ‘rain of money’. Claiming to have access to such notes, the fake Swamis would charge customers hefty sums- sometimes taking ₹2lakh and returning only ₹20,000 to ₹40,000 in so-called ‘ritual’ notes.
-The police said the accused used an associate identified as Mubarak and used to tamper original ₹2,000 notes by altering the printed year and serial number. These modified notes were then circulated through agents to unsuspecting victims.
-The swamis conducted the fake rituals near lakes or ponds, insisting that the ‘pooja’ must be performed alone, without any family members present.
-During the ritual, they told the victims to take a dip in the water to pray for the ‘rain of money’. While the victims submerged, the fake swamis would flee with the money.
-The gang operated in Bengaluru, Yadgir, Haveri, Andhra Pradesh, and Tamil Nadu, the police said. So far, the officers have seized ₹18 lakh worth of ₹2,000 denomination notes and the equipment used to tamper with them.
-The police were verifying whether the seized notes are genuine or altered.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/halasuru-gate-police-bust-fake-2000-notes-racket-10-arrested/article70239293.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:31:50 +0530</t>
-  </si>
-  <si>
     <t>TOI</t>
   </si>
   <si>
@@ -469,7 +474,7 @@
     <t>Zohran Mamdani (File photo)
 The TOI correspondent from Washington
 ‘JUST IGNORE HIM!’: Zohran Mamdani ‘HUMILIATES’ Trump As He Casts Ballot In NYC Mayoral Election
-: New Yorkers streamed into polling stations on Tuesday morning with the remarkable prospect of the undisputed global capital of finance, skyscrapers, and immense wealth paradoxically electing a socialist mayor.Turbocharged by a brilliant digital campaign, a raft of breathtaking promises, and a winning smile that launched a thousand quips, Zohran Mamdani , the Uganda-born Indian son of film-maker Mira Nair (born in Odisha) and academic Mahmood Mamdani (born in Mumbai), is all set to occupy the City Hall in the ground zero of capitalism, putative Muslim mayor of an iconic city that was attacked by Islamist terrorists on 9/11.Although the gap between Mamdani and his Democrat-turned-independent opponent Andrew Cuomo narrowed by Tuesday, the Indian-African New Yorker is expected to romp home comfortably despite President Trump coming out swinging at the prospect of a mayor who in his view is a communist and a “radical left lunatic.”On the eve of election day, Trump threw his weight behind Cuomo, a scandal-tarnished former Governor of New York, urging voters to even ditch Republican candidate Curtis Sliva (who is polling a distant third), saying “it is my strong conviction that New York City will be a Complete and Total Economic and Social Disaster should Mamdani win. I would much rather see a Democrat win than a Communist with no experience.”Trump also threatened to cut federal funds, “other than the very minimum as required, to my beloved first home,” saying the city has zero chances of success under a “communist,” kneecapping Mamdani even before he takes office.The irony of the most capitalist city on the planet electing a Muslim socialist mayor will go into political folklore but the reasons are not hard to fathom. While NYC is arguably the richest city in the world, with more than 350,000 millionaires, it is also a megalopolis of brutal economic inequality, with crippling housing costs ($3000 per month rent for a studio in Manhattan), failing public transit, and deep-seated poverty in its outer neighborhoods. The wealth that defines the city also creates the extreme, daily cost-of-living pressure for everyone else.Mamdani has tapped into this disaffection arising from what he calls the affordability crisis, promising, among other things, higher taxes on the wealthy, rent freeze, free city buses, city-run grocery stores and other sops that have some of its more affluent residents bolting the Big Apple fearing the incoming Mayor will demand a bigger slice of their pie.While non-hispanic whites form the single largest group of eligible voters at 42 percent in the Democratic-leaning city, the Mamdani surge is also powered by Hispanic/Latinos (24 percent), Black/African-American (19 percent), and Asian-American (15 percent). In fact, his campaign was evocative of the city’s diversity, with ads in Spanish and Hindi, including a liberal use of Bollywood song and dance and desi tropes like mango lassi.“When Americans fly in from across our land to JFK &amp; LaGuardia and hear over the loudspeaker, ‘I am Mayor @ZohranKMamdani, welcome to NYC,’ they will look to their children filled with pride and say, ‘In NY any dream is still possible!’” Congressman Ro Khanna, an Indian-American representing SIlicon Valley in California, said, echoing the vision of American liberals.A Mamdani victory, which even Trump appeared to concede is a foregone conclusion, is also expected to weigh in on the ideological future of the Democratic Party, pushing it further left and powering progressives against the moderate and centrist establishment wing of the party.“Our time has come, New York. Our time is now,” Mamdani posted on X Tuesday morning as he headed out to vote with his wife, Rama Duwaji, a Syrian-American.While all eyes are on polling in NYC, there are also mayoral elections in Boston, Atlanta, Seattle, and Minneapolis and gubernatorial elections in New Jersey and Virginia, offering a referendum of sorts on the ten months of Trump rule.In another closely watched election, voters in Virginia, abutting the capital, will be electing their first female governor, choosing between Democrat Abigail Spanberger, a former CIA agent and lawmaker, and Republican Winsome Earle-Sears, the current Jamaica-born Lieutenant governor who served in the US Marines. Across the country, California is also voting on a statewide ballot measure called Proposition 50 designed to create up to five additional Democratic-leaning seats in the House of Representatives to offset the gains Republicans have made nationally through their own map redraws.</t>
+: New Yorkers streamed into polling stations on Tuesday morning with the remarkable prospect of the undisputed global capital of finance, skyscrapers, and immense wealth paradoxically electing a socialist mayor.Turbocharged by a brilliant digital campaign, a raft of breathtaking promises, and a winning smile that launched a thousand quips, Zohran Mamdani , the Uganda-born Indian son of film-maker Mira Nair (born in Odisha) and academic Mahmood Mamdani (born in Mumbai), is all set to occupy the City Hall in the ground zero of capitalism, putative Muslim mayor of an iconic city that was attacked by Islamist terrorists on 9/11.Although the gap between Mamdani and his Democrat-turned-independent opponent Andrew Cuomo narrowed by Tuesday, the Indian-African New Yorker is expected to romp home comfortably despite President Trump coming out swinging at the prospect of a mayor who in his view is a communist and a “radical left lunatic.”On the eve of election day, Trump threw his weight behind Cuomo, a scandal-tarnished former Governor of New York, urging voters to even ditch Republican candidate Curtis Sliva (who is polling a distant third), saying “it is my strong conviction that New York City will be a Complete and Total Economic and Social Disaster should Mamdani win. I would much rather see a Democrat win than a Communist with no experience.”Trump also threatened to cut federal funds, “other than the very minimum as required, to my beloved first home,” saying the city has zero chances of success under a “communist,” kneecapping Mamdani even before he takes office.The irony of the most capitalist city on the planet electing a Muslim socialist mayor will go into political folklore but the reasons are not hard to fathom. While NYC is arguably the richest city in the world, with more than 350,000 millionaires, it is also a megalopolis of brutal economic inequality, with crippling housing costs ($3000 per month rent for a studio in Manhattan), failing public transit, and deep-seated poverty in its outer neighborhoods. The wealth that defines the city also creates the extreme, daily cost-of-living pressure for everyone else.Also read: New Trump Era: Laura Loomer gets credentials to cover US Department of Defense - why it's a big deal Mamdani has tapped into this disaffection arising from what he calls the affordability crisis, promising, among other things, higher taxes on the wealthy, rent freeze, free city buses, city-run grocery stores and other sops that have some of its more affluent residents bolting the Big Apple fearing the incoming Mayor will demand a bigger slice of their pie.While non-hispanic whites form the single largest group of eligible voters at 42 percent in the Democratic-leaning city, the Mamdani surge is also powered by Hispanic/Latinos (24 percent), Black/African-American (19 percent), and Asian-American (15 percent). In fact, his campaign was evocative of the city’s diversity, with ads in Spanish and Hindi, including a liberal use of Bollywood song and dance and desi tropes like mango lassi.“When Americans fly in from across our land to JFK &amp; LaGuardia and hear over the loudspeaker, ‘I am Mayor @ZohranKMamdani, welcome to NYC,’ they will look to their children filled with pride and say, ‘In NY any dream is still possible!’” Congressman Ro Khanna, an Indian-American representing SIlicon Valley in California, said, echoing the vision of American liberals.A Mamdani victory, which even Trump appeared to concede is a foregone conclusion, is also expected to weigh in on the ideological future of the Democratic Party, pushing it further left and powering progressives against the moderate and centrist establishment wing of the party.“Our time has come, New York. Our time is now,” Mamdani posted on X Tuesday morning as he headed out to vote with his wife, Rama Duwaji, a Syrian-American.While all eyes are on polling in NYC, there are also mayoral elections in Boston, Atlanta, Seattle, and Minneapolis and gubernatorial elections in New Jersey and Virginia, offering a referendum of sorts on the ten months of Trump rule.In another closely watched election, voters in Virginia, abutting the capital, will be electing their first female governor, choosing between Democrat Abigail Spanberger, a former CIA agent and lawmaker, and Republican Winsome Earle-Sears, the current Jamaica-born Lieutenant governor who served in the US Marines. Across the country, California is also voting on a statewide ballot measure called Proposition 50 designed to create up to five additional Democratic-leaning seats in the House of Representatives to offset the gains Republicans have made nationally through their own map redraws.</t>
   </si>
   <si>
     <t>https://timesofindia.indiatimes.com/world/us/its-mango-lassi-mamdani-morning-in-big-apple/articleshow/125091203.cms</t>
@@ -481,30 +486,28 @@
     <t>https://static.toiimg.com/thumb/msid-125091217,width-1070,height-580,imgsize-390229,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>Asia Cup controversy: ICC takes action against Pakistan's Haris Rauf; Suryakumar Yadav fined</t>
-  </si>
-  <si>
-    <t>Harsi Rauf and Suryakumar Yadav (ACC Photo)
-Go Beyond The Boundary with our YouTube channel. SUBSCRIBE NOW!
-BCCI sends a stern message to Mohsin Naqvi over Asia Cup trophy row
-The International Cricket Council (ICC) has announced the results of several Code of Conduct hearings arising from the India–Pakistan encounters during the ICC Asia Cup 2025. The disciplinary actions, confirmed on Tuesday, follow investigations into on-field incidents from the matches held on September 14, 21, and 28. These hearings were conducted by members of the ICC Elite Panel of Match Referees.The September 14 clash saw India’s Suryakumar Yadav and Pakistan’s Haris Rauf and Sahibzada Farhan charged with breaches of Article 2.21 of the ICC Code of Conduct, which addresses behaviour that brings the game into disrepute. ICC Match Referee Richie Richardson found all three guilty. Suryakumar was fined 30% of his match fee and given two demerit points. Farhan received an official warning and one demerit point, while Rauf was fined 30% of his match fee and handed two demerit points.A week later, on September 21, India pacer Arshdeep Singh was cleared of an alleged breach of Article 2.6, which pertains to using obscene or offensive gestures. ICC Match Referee Andy Pycroft found him not guilty, and no sanction was imposed.Also read: Diamond jewellery, solar panels and 297% prize money hike — India's World Cup queens rewarded royally
-In the September 28 final between India and Pakistan, further disciplinary action followed.Jasprit Bumrah accepted responsibility for a breach of Article 2.21 for conduct deemed to bring the game into disrepute. By accepting the charge and sanction—a formal warning and one demerit point—Bumrah avoided a hearing.However, Pakistan pacer Haris Rauf once again came under scrutiny for the same offence. Following a second hearing before Richie Richardson, Rauf was fined another 30% of his match fee and given two additional demerit points. This took his tally to four demerit points within a 24-month period, which automatically converts to two suspension points under ICC rules. As a result, Rauf has been suspended from Pakistan’s upcoming ODIs against South Africa on November 4 and 6, 2025.According to ICC regulations, Level 1 breaches carry a minimum penalty of an official reprimand and a maximum of a 50% match-fee fine, along with one or two demerit points. Once a player accumulates four or more demerit points in two years, they are converted into suspension points, resulting in a ban. Demerit points remain on record for 24 months before being expunged.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/cricket/news/asia-cup-controversy-icc-takes-action-against-haris-rauf-suryakumar-yadav-fined/articleshow/125090429.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 20:34:36 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125090467,width-1070,height-580,imgsize-61086,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+    <t>Air traffic congestion: Flight operations impacted in Delhi; IndiGo issues advisory</t>
+  </si>
+  <si>
+    <t>Representational file photo
+DGCA Plans New Rules For Power Banks On Flights After Fire Scare On IndiGo Plane
+NEW DELHI: Flight delays hit several passengers travelling through Delhi on Tuesday, as air traffic congestion led to long wait times across terminals.IndiGo posted an advisory on its official X account, saying: “Due to air traffic congestion in Delhi, flight operations are currently impacted. We understand that extended wait times, both on the ground and onboard, may cause inconvenience, and we sincerely appreciate your patience. ”Also read: Air India sends alternate aircraft to fly home passengers stranded in Mongolia The airline also assured passengers that its on-ground teams were working to make the wait as comfortable as possible. “We value your time and are doing everything we can to help you get on your way soon,” IndiGo said, advising travellers to check its website or mobile app for real-time flight updates.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/air-traffic-congestion-flight-operations-impacted-in-delhi-indigo-issues-advisory/articleshow/125091789.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:13:33 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091871,width-1070,height-580,imgsize-34734,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Chhattisgarh train accident: Toll reaches 8; compensation of 10 lakh announced</t>
   </si>
   <si>
     <t>Photo: PTI screengrab
-Rajasthan: At Least 15 Killed, 2 Injured As Tourist Bus Collides With Parked Trailer In Phalodi
+At Least 5 Killed, Several Injured As Passenger Train Collides With Goods Trains In Chhattisgarh
 Rs 10 lakh to the next of kin of the deceased (casualties).
 Rs 5 lakh to those grievously injured.
 Rs 1 lakh to those with minor injuries.
@@ -520,45 +523,38 @@
     <t>https://static.toiimg.com/thumb/msid-125087453,width-1070,height-580,imgsize-41276,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>Asia Cup controversy: ICC drops the hammer! Full list of players punished and warned</t>
-  </si>
-  <si>
-    <t>Suryakumar Yadav and Salman Agha (PTI Photo)
+    <t>Pakistan's Haris Rauf, once hammered by Virat Kohli, banned by ICC after Asia Cup controversy</t>
+  </si>
+  <si>
+    <t>Pakistan pacer Haris Rauf has been handed a two-match suspension by ICC (Photo credit: Agencies)
 Go Beyond The Boundary with our YouTube channel. SUBSCRIBE NOW!
 BCCI sends a stern message to Mohsin Naqvi over Asia Cup trophy row
-Players Penalised by ICC ( Asia Cup 2025 ):
-Suryakumar Yadav (India):
-Sahibzada Farhan (Pakistan):
-Haris Rauf (Pakistan):
-Jasprit Bumrah (India):
-Arshdeep Singh (India):
-NEW DELHI: The International Cricket Council (ICC) has confirmed disciplinary actions against multiple players from India and Pakistan following several heated encounters during the ICC Asia Cup 2025. The Code of Conduct hearings, led by members of the ICC Elite Panel of Match Referees, investigated incidents from the India–Pakistan matches played on September 14, 21, and 28.In the September 14 clash, India’s Suryakumar Yadav and Pakistan’s Haris Rauf and Sahibzada Farhan were found guilty of breaching Article 2.21 of the ICC Code of Conduct, which covers conduct that brings the game into disrepute.Suryakumar was fined 30% of his match fee and received two demerit points.Farhan was given an official warning and one demerit point.Rauf was fined 30% of his match fee and also received two demerit points.A week later, on September 21, India pacer Arshdeep Singh was charged under Article 2.6 for allegedly making an offensive gesture, but was found not guilty after a hearing conducted by Match Referee Andy Pycroft.The Asia Cup final on September 28 brought further disciplinary action. Jasprit Bumrah accepted a charge under Article 2.21 for conduct that brings the game into disrepute, accepting an official warning and one demerit point.Since he admitted to the offence, no formal hearing was held.Haris Rauf, meanwhile, was penalised again for the same offence after a hearing before Richie Richardson. He was fined another 30% of his match fee and received two additional demerit points, taking his total to four demerit points within 24 months. That triggered an automatic suspension, ruling him out of Pakistan’s ODIs against South Africa on November 4 and 6, 2025.According to ICC rules, Level 1 breaches carry a maximum fine of 50% of a player’s match fee and up to two demerit points. Accumulating four or more demerit points in two years converts to suspension points, leading to a ban.Fined 30% match fee, 2 demerit pointsOfficial warning, 1 demerit pointTwo separate offences; fined twice, 4 demerit points and 2-match suspensionOfficial warning, 1 demerit pointFound not guilty, no sanction</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/cricket/news/asia-cup-controversy-icc-drops-the-hammer-full-list-of-players-punished-and-warned/articleshow/125091140.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:29:06 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125091164,width-1070,height-580,imgsize-40780,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>'Highway man always high': Congress mocks Nitin Gadkari over Bihar poll promises</t>
-  </si>
-  <si>
-    <t>Union minister Nitin Gadkari (File photo)
-'Paid Campaign': Nitin Gadkari Slams Criticism Of E20 Program; Calls It 'Politically Motivated'
-NEW DELHI: The Congress on Tuesday took a swipe at Union road transport and highways minister Nitin Gadkari over his repeated promises to the people of Bihar, remarking that “it seems the highway man is always high.”Mocking Gadkari’s claims, Congress leader Pawan Khera shared a video on X compiling the minister’s old and recent statements in poll-bound Bihar, where he pledged to build “world-class” roads and assured the public that “the roads will be at par with American roads.”The video juxtaposed Gadkari’s promises from 2024 with his latest assurances during the ongoing election campaign in Bihar.Joining the attack, the Kerala Congress also took a jibe at the Union minister, calling him “the new jumla king in town.”Meanwhile, campaigning for the first phase of polling has concluded. Bihar will vote in the first phase on November 6 and the second on November 11, with counting of votes and announcement of results scheduled for November 14.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/highway-man-always-high-congress-mocks-nitin-gadkari-over-bihar-poll-promises-shares-old-us-style-roads-video/articleshow/125090791.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:02:42 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125090849,width-1070,height-580,imgsize-810362,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+NEW DELHI: Pakistan pacer Haris Rauf has been handed a two-match suspension and will miss the upcoming ODIs against South Africa after breaching the ICC Code of Conduct during the Asia Cup 2025 final against India on September 28, the International Cricket Council (ICC) announced on Tuesday.The ICC confirmed disciplinary actions arising from the India–Pakistan fixtures, with sanctions imposed following hearings by the Emirates ICC Elite Panel of Match Referees.“Following a hearing conducted by ICC Match Referee Richie Richardson, Haris Rauf was again found guilty of a breach of Article 2.21. He was fined 30 per cent of his match fee and received two additional demerit points,” the ICC said in a statement.“This takes Rauf’s total to four demerit points within a 24-month period, resulting in two suspension points. In line with the Code, Rauf is therefore suspended for Pakistan’s ODIs against South Africa on November 4 and 6,” it added.Rauf had earlier committed the same offence during the group-stage clash on September 14, for which he was fined 30 per cent of his match fee and given two demerit points.Meanwhile, Pakistan batter Sahibzada Farhan received an official warning and one demerit point for his “gun celebration” after scoring a fifty against India during the Super 4 clash in Dubai.In the same September 14 match, India captain Suryakumar Yadav was also found guilty of breaching Article 2.21, fined 30 per cent of his match fee, and given two demerit points.For the September 21 encounter, Indian pacer Arshdeep Singh was cleared of charges related to obscene or insulting gestures under Article 2.6.During the final on September 28, Jasprit Bumrah accepted a Level 1 offence under Article 2.21, receiving an official warning and one demerit point, thereby avoiding a formal disciplinary hearing.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/cricket/news/pakistans-haris-rauf-once-hammered-by-virat-kohli-banned-by-icc-after-asia-cup-controversy/articleshow/125091778.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:07:42 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091823,width-1070,height-580,imgsize-58174,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Photo shows how Telangana bus crash trapped passengers; 19 dead</t>
+  </si>
+  <si>
+    <t>Deadly Collision on Hyderabad-Bijapur Road: 19 Killed After Truck Rams Into RTC Bus Near Chevella
+CHEVELLA: A scream. Then, silence — broken only by cries muffled under stone and steel. The bus lay crushed beneath a mountain of gravel, its passengers trapped — some buried up to their necks — as minutes stretched into nearly an hour before rescuers could reach them.“It felt like the whole world had collapsed on us. We couldn’t move or breathe properly,” said R Venkataiah, 55, a head constable from Vikarabad. He was on a work trip, now lying on a hospital cot, his voice trembling. “We screamed for help. But no one could get to us for so long.”By the time emergency crews pulled survivors from the wreckage, many had suffered deep cuts, crushed limbs and spinal injuries. Women, students, and children were among those badly hurt.“It all happened in a flash,” said C Sri Sai, a 27-year-old govt school teacher from Chevella. Speaking from her hospital bed, her leg wrapped in bandages, she recalled boarding the Telangana State Road Transport Corporation busaround 5am. “I sat in the last row. About an hour later, suddenly there was a huge crash — the entire bus shook violently,people screamed, and within moments everything went dark and dusty.”Her family rushed from Tandur town after hearing the news. “It took nearly 30 minutes before the rescuers managed to pull us out,” she said.The truck smashed head-on into the Hyderabad-bound bus, tearing open its right side and spilling gravel. Those seated behind the bus driver never had a chance. “They were almost instantly buried under the gravel — I could only hear muffled cries,” said Abdul Razak, 38, another survivor. His hands still shook as he spoke. “It was nerve-wracking.”Mohammed Yunus, a businessman from Tandur, had climbed aboard the same bus. He escaped with bruises — but not without images he can’t forget. “I was standing in the middle of the bus. When the lorry hit, I fell sideways, and the gravel started pouring in. I thought I would die,” he said. “Because I wasn’t sitting, I managed to wriggle out through a broken window.” Others weren’t as lucky. Many remained pinned, gasping under the weight of stones.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/city/hyderabad/buried-in-gravel-frozen-in-fear-this-photo-shows-how-telangana-bus-crash-trapped-passengers-alive/articleshow/125075859.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 10:58:18 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125075919,width-1070,height-580,imgsize-1362596,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Big AI freebie: ChatGPT Go now free for 12 months in India; how to claim the offer</t>
@@ -590,52 +586,61 @@
     <t>https://static.toiimg.com/thumb/msid-125076745,width-1070,height-580,imgsize-41718,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>Junagadh horror: Teen celebrates double murder; used sugar to decompose bodies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-RAJKOT/AHMEDABAD: Disturbing details are emerging from the investigation into the horrific murder of a young couple in a village of Junagadh's Visavadar taluka, allegedly carried out by the man's 16-year-old brother.Investigators were stunned not only by the barbarity and the teenager's lack of remorse but the way he reportedly "celebrated" the killings with country liquor on Oct 16.The probe revealed that the elder brother frequently beat the boy for chewing mava (a mix of betel-nut pieces and tobacco), something which police suspect consumed him with deep hatred and anger. Villagers told investigators the boy was addicted to liquor.On Saturday, Visavadar had police arrested the juvenile who had dug a five- to six-foot pit outside the house and buried the bodies. His mother was also arrested."During questioning, he calmly recounted the entire sequence of events and the days that followed the murders. Initially, we thought he was trying to mislead us, but checks at the locations he mentioned and talking with people he contacted after the crime corroborated his statements," Rohit Dagar, ASP, Visavadar, told TOI.According to police, after burying the bodies the boy bought four pouches of country liquor for Rs 400 and drank to celebrate,sitting near the same pit. "He rejoiced in the successful execution of the crime and in not being caught, watching reels on Instagram and drinking," the officer added.The juvenile also allegedly confessed to raping his brother's wife, removing her jewellery and selling it for Rs 30,000.Police were further startled by the boy's intense compassion for the cattle in the animal shed he had tended for five years. He repeatedly pleaded with officers to arrange fodder for the animals, saying they would starve — something he said he could not bear. He also warned that the cattle would turn aggressive if anyone other than him tried to feed them."And this is exactly what happened. When we entered the farm, the animals became aggressive and would not allow anyone near them. Ultimately, we asked the sarpanch to let the cattle graze freely. We are surprised that a boy with so much love for his animals could resort to such brutality with a cold heart," said Dagar.Bought 52kgs of sugar for faster decay of bodiesPolice found the boy had searched YouTube and Instagram for methods to dispose of bodies. He discovered that sugar attracts insects and maggots and purchased a staggering 52 kg to pour over the corpses. " He dug the pit in the house compound and used his electrician brother's drilling machine to grind stones. He mixed the rubble with cement and created a double layer over the pit to conceal it," police said.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/city/rajkot/16-year-old-drank-liquor-to-celebrate-brothers-murder/articleshow/125066370.cms</t>
-  </si>
-  <si>
-    <t>Mon, 03 Nov 2025 23:59:22 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125077779,width-1070,height-580,imgsize-1106657,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Watch: China’s astronauts grill chicken, steak in space — why it matters</t>
-  </si>
-  <si>
-    <t>Screengrab (Picture source: X/CNSA)
-In a first for China’s manned space programme, astronauts on the Shenzhou-20 and Shenzhou-21 missions have used a specially developed oven to barbecue chicken wings and cook steak aboard the China Space Station.The new “space oven,” installed recently, allows smokeless cooking and is part of broader efforts to improve living conditions for astronauts on long-duration missions.Footage released by the Astronaut Center of China (ACC) showed crew members enjoying freshly grilled food after 28 minutes of cooking. The oven, which operates through advanced temperature control and high-temperature catalysis, can function continuously for up to 500 cycles.It represents a leap from earlier international experiments such as the 2020 baking test aboard the International Space Station (ISS), where astronauts took up to two hours to bake cookies, according to a BBC news, reported Chinese media Global Times.The oven also marks the rapid evolution of China’s in-orbit living standards, from simple pre-packaged meals during the Shenzhou-5 era to a diverse menu of over 190 items today. After long hours of scientific work, sharing a hot meal gives astronauts a sense of normalcy and connection to Earth.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/science/watch-chinas-astronauts-grill-chicken-steak-in-space-why-it-matters/articleshow/125090248.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:38:05 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125090258,width-1070,height-580,imgsize-29098,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Pakistan to deploy new submarines in 2026 — what it means for India’s naval strategy</t>
-  </si>
-  <si>
-    <t>Pakistan Issues Naval Warning as Its War Games Overlap with India’s Military Drills
-NEW DELHI: India’s major naval combat edge over Pakistan will begin to somewhat erode from next year onwards when the latter begins inducting eight advanced Hangor-class diesel-electric submarines from China. India’s long-pending conventional submarine-building plan, in sharp contrast, is yet to even kick off.Pakistan Navy chief Admiral Naveed Ashraf has confirmed in interviews to Chinese state media that the first Hangor-class submarine will enter active service next year. All eight boats, four each being built in China and Pakistan, under the estimated $5 billion deal, will be delivered by 2028. They will boost Pakistan’s ability to patrol the north Arabian Sea and Indian Ocean, he said.The Hangor or Type 039A Yuan-class submarines, in addition to having advanced sensors and weapons, are also equipped with the Stirling air-independent propulsion (AIP) to boost their underwater endurance.While nuclear-powered submarines can stay underwater for months on end, diesel-electric boats must surface or snorkel every couple of days to get oxygen to recharge their batteries. Those with AIP, however, can stay submerged for around two-three weeks to significantly boost their stealth and combat capabilities.India, at present, has no conventional submarine with AIP.“The submarines will undoubtedly boost Pakistan’s A2/AD (anti-access/area denial) capabilities in the Arabian Sea. We will have to find a solution for it. China, of course, is always there to help Pakistan, which was very evident during Operation Sindoor,” a senior Indian military official told TOI.The IAF during its strikes on terror hubs on May 7 was initially surprised by Pakistan’s use of Chinese-origin jets like J-10s armed with PL-15 air-to-air missiles, with ranges over 200-km, in a fully-networked sensor-shooter loop, as was reported by TOI earlier.Also read: India, US ink new defence framework for 10 years; aim to deepen cooperation in all domains The deep military collusion between China and Pakistan along the land borders has now well and truly expanded to the maritime domain. “After the overwhelming dominance demonstrated by the Indian Navy in the north Arabian Sea during Op Sindoor, Pakistan will be better prepared the next time, plugging gaps with help from China and Turkiye,” another officer said.The Indian Navy, of course, has the submarine-hunting P-8I long-range aircraft and MH-60R Seahawk helicopters of US-origin as well as anti-submarine warfare warships, all armed with advanced radars, sonars, missiles, torpedoes and multifunctional rockets.The depleting underwater combat arm, however, remains a big worry. The `Project-75 India’ to construct six new German-origin diesel-electric submarines with AIP at Mazagon Docks for over Rs 70,000 crore is still some months away from being inked. Under P-75I, which was granted the initial “acceptance of necessity” way back in November 2007, it will take at least seven-eight years for the first boat to roll out after the contract.Apart from the six new French-origin Scorpenes, the Navy is left with just six old Russian Kilo-class and four German HDW submarines in its conventional underwater fleet. It also has two nuclear-powered submarines armed with ballistic missiles (SSBNs) in INS Arihant and INS Arighaat, while a third one will be commissioned as INS Aridhaman early next year.China has over 50 diesel-electric and 10 nuclear submarines, while Pakistan has three French Agosta-90B and two Agosta-70 submarines at present. “Pakistan is trying to build its third leg of the nuclear triad by equipping its Agosta-90B boats with 450-km range Babur-3 cruise missiles. The Hangor-class boats will certainly have the Babur-3 missiles,” another officer said.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/india-will-have-to-contend-with-new-pakistan-submarines-from-next-year/articleshow/125072697.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 07:31:25 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125072708,width-1070,height-580,imgsize-209966,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+    <t>'Highway man always high': Congress mocks Nitin Gadkari over Bihar poll promises</t>
+  </si>
+  <si>
+    <t>Union minister Nitin Gadkari (File photo)
+'Paid Campaign': Nitin Gadkari Slams Criticism Of E20 Program; Calls It 'Politically Motivated'
+NEW DELHI: The Congress on Tuesday took a swipe at Union road transport and highways minister Nitin Gadkari over his repeated promises to the people of Bihar, remarking that “it seems the highway man is always high.”Mocking Gadkari’s claims, Congress leader Pawan Khera shared a video on X compiling the minister’s old and recent statements in poll-bound Bihar, where he pledged to build “world-class” roads and assured the public that “the roads will be at par with American roads.”The video juxtaposed Gadkari’s promises from 2024 with his latest assurances during the ongoing election campaign in Bihar.Joining the attack, the Kerala Congress also took a jibe at the Union minister, calling him “the new jumla king in town.”Meanwhile, campaigning for the first phase of polling has concluded. Bihar will vote in the first phase on November 6 and the second on November 11, with counting of votes and announcement of results scheduled for November 14.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/highway-man-always-high-congress-mocks-nitin-gadkari-over-bihar-poll-promises-shares-old-us-style-roads-video/articleshow/125090791.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:02:42 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125090849,width-1070,height-580,imgsize-810362,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>More power for Asim Munir? Pakistan plans amendment; revises military command</t>
+  </si>
+  <si>
+    <t>Pakistani army chief general Asim Munir
+The Pakistan government announced plans to introduce the 27th Constitutional Amendment, which includes proposed changes related to the command of the armed forces. The amendment will be tabled in Parliament soon, deputy prime minister and foreign minister Ishaq Dar confirmed on Tuesday.“Of course, the government is bringing it and will bring it … the 27th Amendment will arrive … and is about to arrive. We will try that it be tabled in accordance with principles, laws and the Constitution,” Dar said in the Senate, as quoted by PTI.According to sources, the proposed amendment includes provisions to set up a constitutional court, streamline the process for appointing the chief election commissioner, amend Article 243 dealing with matters of the armed forces, reduce the provinces’ share in federal resources, and transfer control of the education and population welfare ministries from provinces to the federal government.Article 243 of the Constitution states that “the federal government shall have control and command of the armed forces.” The proposal to revise this article is being viewed as a move that could further strengthen the position of Army Chief General Asim Munir and expand the military’s role in national affairs.Dar rejected concerns that the amendment might be passed without proper procedure. “It is not the case that the amendment is tabled and there is voting on it in a haphazard, ad hoc manner; this will not happen,” he said.He said the amendment would first be introduced in the Senate and then referred to a bipartisan committee for discussion, adding that the government would welcome positive suggestions to improve the draft.PPP Senator Raza Rabbani said the changes would damage provincial autonomy and “undo the good work of the 18th amendment,” which devolved powers to the provinces in 2010.The government has the required two-thirds majority in the 336-member National Assembly with the support of 233 members. In the 96-member Senate, it holds 61 seats and will need at least three opposition members to pass the amendment.The secrecy around the proposed changes, particularly the plan to amend Article 243, has drawn attention to whether the new constitutional move will give the armed forces greater influence in the country’s governance.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/world/pakistan/more-power-for-asim-munir-pakistan-plans-constitutional-amendment-includes-revisions-to-military-command-federal-powers/articleshow/125092057.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:33:05 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125092084,width-1070,height-580,imgsize-469567,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Asia Cup controversy: ICC drops the hammer! Full list of players punished and warned</t>
+  </si>
+  <si>
+    <t>Suryakumar Yadav and Salman Agha (PTI Photo)
+Go Beyond The Boundary with our YouTube channel. SUBSCRIBE NOW!
+BCCI sends a stern message to Mohsin Naqvi over Asia Cup trophy row
+Players Penalised by ICC ( Asia Cup 2025 ):
+Suryakumar Yadav (India):
+Sahibzada Farhan (Pakistan):
+Haris Rauf (Pakistan):
+Jasprit Bumrah (India):
+Arshdeep Singh (India):
+NEW DELHI: The International Cricket Council (ICC) has confirmed disciplinary actions against multiple players from India and Pakistan following several heated encounters during the ICC Asia Cup 2025. The Code of Conduct hearings, led by members of the ICC Elite Panel of Match Referees, investigated incidents from the India–Pakistan matches played on September 14, 21, and 28.In the September 14 clash, India’s Suryakumar Yadav and Pakistan’s Haris Rauf and Sahibzada Farhan were found guilty of breaching Article 2.21 of the ICC Code of Conduct, which covers conduct that brings the game into disrepute.Suryakumar was fined 30% of his match fee and received two demerit points.Farhan was given an official warning and one demerit point.Rauf was fined 30% of his match fee and also received two demerit points.A week later, on September 21, India pacer Arshdeep Singh was charged under Article 2.6 for allegedly making an offensive gesture, but was found not guilty after a hearing conducted by Match Referee Andy Pycroft.The Asia Cup final on September 28 brought further disciplinary action. Jasprit Bumrah accepted a charge under Article 2.21 for conduct that brings the game into disrepute, accepting an official warning and one demerit point.Since he admitted to the offence, no formal hearing was held.Haris Rauf, meanwhile, was penalised again for the same offence after a hearing before Richie Richardson. He was fined another 30% of his match fee and received two additional demerit points, taking his total to four demerit points within 24 months. That triggered an automatic suspension, ruling him out of Pakistan’s ODIs against South Africa on November 4 and 6, 2025.According to ICC rules, Level 1 breaches carry a maximum fine of 50% of a player’s match fee and up to two demerit points. Accumulating four or more demerit points in two years converts to suspension points, leading to a ban.Fined 30% match fee, 2 demerit pointsOfficial warning, 1 demerit pointTwo separate offences; fined twice, 4 demerit points and 2-match suspensionOfficial warning, 1 demerit pointFound not guilty, no sanction</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/cricket/news/asia-cup-controversy-icc-drops-the-hammer-full-list-of-players-punished-and-warned/articleshow/125091140.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:29:06 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091164,width-1070,height-580,imgsize-40780,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Musk vs Altman: OpenAI’s ex chief scientist testifies in court; reveals ‘6-day story’</t>
@@ -657,6 +662,38 @@
     <t>https://static.toiimg.com/thumb/msid-125089911,width-1070,height-580,imgsize-859288,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
+    <t>Watch: China’s astronauts grill chicken, steak in space — why it matters</t>
+  </si>
+  <si>
+    <t>Screengrab (Picture source: X/CNSA)
+In a first for China’s manned space programme, astronauts on the Shenzhou-20 and Shenzhou-21 missions have used a specially developed oven to barbecue chicken wings and cook steak aboard the China Space Station.The new “space oven,” installed recently, allows smokeless cooking and is part of broader efforts to improve living conditions for astronauts on long-duration missions.Footage released by the Astronaut Center of China (ACC) showed crew members enjoying freshly grilled food after 28 minutes of cooking. The oven, which operates through advanced temperature control and high-temperature catalysis, can function continuously for up to 500 cycles.It represents a leap from earlier international experiments such as the 2020 baking test aboard the International Space Station (ISS), where astronauts took up to two hours to bake cookies, according to a BBC news, reported Chinese media Global Times.The oven also marks the rapid evolution of China’s in-orbit living standards, from simple pre-packaged meals during the Shenzhou-5 era to a diverse menu of over 190 items today. After long hours of scientific work, sharing a hot meal gives astronauts a sense of normalcy and connection to Earth.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/science/watch-chinas-astronauts-grill-chicken-steak-in-space-why-it-matters/articleshow/125090248.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:38:05 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125090258,width-1070,height-580,imgsize-29098,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Pakistan to deploy new submarines in 2026 — what it means for India’s naval strategy</t>
+  </si>
+  <si>
+    <t>Pakistan Issues Naval Warning as Its War Games Overlap with India’s Military Drills
+NEW DELHI: India’s major naval combat edge over Pakistan will begin to somewhat erode from next year onwards when the latter begins inducting eight advanced Hangor-class diesel-electric submarines from China. India’s long-pending conventional submarine-building plan, in sharp contrast, is yet to even kick off.Pakistan Navy chief Admiral Naveed Ashraf has confirmed in interviews to Chinese state media that the first Hangor-class submarine will enter active service next year. All eight boats, four each being built in China and Pakistan, under the estimated $5 billion deal, will be delivered by 2028. They will boost Pakistan’s ability to patrol the north Arabian Sea and Indian Ocean, he said.The Hangor or Type 039A Yuan-class submarines, in addition to having advanced sensors and weapons, are also equipped with the Stirling air-independent propulsion (AIP) to boost their underwater endurance.While nuclear-powered submarines can stay underwater for months on end, diesel-electric boats must surface or snorkel every couple of days to get oxygen to recharge their batteries. Those with AIP, however, can stay submerged for around two-three weeks to significantly boost their stealth and combat capabilities.India, at present, has no conventional submarine with AIP.“The submarines will undoubtedly boost Pakistan’s A2/AD (anti-access/area denial) capabilities in the Arabian Sea. We will have to find a solution for it. China, of course, is always there to help Pakistan, which was very evident during Operation Sindoor,” a senior Indian military official told TOI.The IAF during its strikes on terror hubs on May 7 was initially surprised by Pakistan’s use of Chinese-origin jets like J-10s armed with PL-15 air-to-air missiles, with ranges over 200-km, in a fully-networked sensor-shooter loop, as was reported by TOI earlier.Also read: India, US ink new defence framework for 10 years; aim to deepen cooperation in all domains The deep military collusion between China and Pakistan along the land borders has now well and truly expanded to the maritime domain. “After the overwhelming dominance demonstrated by the Indian Navy in the north Arabian Sea during Op Sindoor, Pakistan will be better prepared the next time, plugging gaps with help from China and Turkiye,” another officer said.The Indian Navy, of course, has the submarine-hunting P-8I long-range aircraft and MH-60R Seahawk helicopters of US-origin as well as anti-submarine warfare warships, all armed with advanced radars, sonars, missiles, torpedoes and multifunctional rockets.The depleting underwater combat arm, however, remains a big worry. The `Project-75 India’ to construct six new German-origin diesel-electric submarines with AIP at Mazagon Docks for over Rs 70,000 crore is still some months away from being inked. Under P-75I, which was granted the initial “acceptance of necessity” way back in November 2007, it will take at least seven-eight years for the first boat to roll out after the contract.Apart from the six new French-origin Scorpenes, the Navy is left with just six old Russian Kilo-class and four German HDW submarines in its conventional underwater fleet. It also has two nuclear-powered submarines armed with ballistic missiles (SSBNs) in INS Arihant and INS Arighaat, while a third one will be commissioned as INS Aridhaman early next year.China has over 50 diesel-electric and 10 nuclear submarines, while Pakistan has three French Agosta-90B and two Agosta-70 submarines at present. “Pakistan is trying to build its third leg of the nuclear triad by equipping its Agosta-90B boats with 450-km range Babur-3 cruise missiles. The Hangor-class boats will certainly have the Babur-3 missiles,” another officer said.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/india-will-have-to-contend-with-new-pakistan-submarines-from-next-year/articleshow/125072697.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 07:31:25 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125072708,width-1070,height-580,imgsize-209966,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
     <t>Happy Guru Nanak Jayanti 2025: 50 Gurpurab wishes, messages, quotes &amp; images</t>
   </si>
   <si>
@@ -670,6 +707,21 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125089268,width-1070,height-580,imgsize-36166,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Nano Banana AI trend: How this popular model got its name; Google explains</t>
+  </si>
+  <si>
+    <t>Google's Gemini Nano Banana gained its viral name from a simple placeholder used by an employee named Nina during anonymous testing. This AI model distinguishes itself with remarkable character consistency and the ability to generate highly imaginative, complex visual concepts, impressing users with its accurate subject retention and creative blending of disparate ideas.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/technology/tech-news/how-googles-most-popular-photo-generation-model-got-nano-banana-name-and-what-it-is-officially-called/articleshow/125091519.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:50:17 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091500,width-1070,height-580,imgsize-1274627,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>‘10% control the Army’: Rahul's caste claim at Bihar rally; BJP terms remark disgraceful</t>
@@ -710,135 +762,71 @@
     <t>https://static.toiimg.com/thumb/msid-125089279,width-1070,height-580,imgsize-832459,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>Jeff Bezos’ ex-wife’s gift: MacKenzie Scott makes large donation; focus on education</t>
-  </si>
-  <si>
-    <t>MacKenzie Scott
-Donation arrives at critical moment for the school
-Mayhem at Amazon Amid 30,000 Job Cuts: AI - Easy Corporate Excuse? | Global Pulse
-Scott’s other donations as part of broader DEI initiatives
-Billionaire philanthropist and Jeff Bezos ’ ex-wife, MacKenzie Scott, has donated $80 million to Howard University, marking one of the largest single donations in the school’s 158-year history and continuing her recent surge of major contributions to diversity and equity causes. The donation, announced over the weekend by Howard University, comes as Scott – estimated to be worth $35.6 billion, as per The Wall Street Journal – has been on what observers are calling a philanthropic roll, making several multimillion-dollar gifts to DEI and disaster relief causes in recent weeks.The donation is unrestricted, allowing the university to allocate the funds as it sees fit. Of the $80 million, $63 million will go to Howard University's general operations, while $17 million will support the school's College of Medicine.“This historic investment will not only help maintain our current momentum, but will help support essential student aid, advance infrastructure improvements, and build a reserve fund to further sustain operational continuity, student success, academic excellence, and research innovation,” said Wayne A.I. Frederick, Howard interim president and president emeritus, in a statement.The university says the gift arrives at an "opportune time" as the federal government shutdown has delayed annual federal appropriations that Howard receives to support student success, academic programming, research, and operations at both the university and Howard University Hospital.The shutdown, which began October 1, has halted new grant awards from the Department of Education after nearly 95% of non-student aid staff were furloughed, leaving only essential personnel working.Scott’s donation to Howard builds on other recent donations focused on diversity, equity and inclusion. She recently gave $42 million to 10,000 Degrees, a Bay Area nonprofit expanding college access for low-income and largely non-white students, alongside other eight-figure commitments to Native student scholars and HBCU endowments through the United Negro College Fund (UNCF).The Howard donation comes just weeks after regulatory filings revealed Scott had reduced her Amazon stake by $12.6 billion.According to a Securities and Exchange Commission filing dated September 30 and first reported by Bloomberg, Scott has cut her holdings in the e-commerce giant by nearly 42%, reducing her stake to $12.6 billion. She now holds 81.1 million Amazon shares—down 58 million from a year earlier.The reduction occurred despite Amazon shares more than doubling in value since Scott's 2019 divorce from Jeff Bezos, the company's co-founder.Scott obtained most of her wealth following her divorce from Bezos and has pledged to give away the majority of it. After receiving approximately 4% of Amazon in the divorce settlement, she has donated $19 billion to more than 2,000 nonprofits over the past five years.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/technology/tech-news/after-reducing-her-amazon-stake-by-12-6-billion-jeff-bezos-ex-wife-mackenzie-scott-makes-one-of-the-largest-donations-to/articleshow/125086903.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 17:22:56 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125086896,width-1070,height-580,imgsize-26596,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Watch: Coach collapses mid-match, dies; players break down in heartbreaking scenes</t>
-  </si>
-  <si>
-    <t>Heartbroken players on the pitch after getting to know that their coach passed away mid-match (Screengrabs)
-Radnicki 1923 head coach Mladen Zizovic passed away after collapsing during his team’s Serbian SuperLiga match against Mladost Lucani on Monday. He was 44.The incident occurred midway through the first half, prompting an immediate halt to the game in the 22nd minute. Zizovic received on-field medical attention before being rushed to a nearby hospital. The match briefly resumed but was abandoned about 20 minutes later when news of his death reached players and staff.Television footage captured heartbreaking scenes as players from both teams reacted in disbelief and distress upon hearing the announcement.Several players dropped to their knees, collapsing on the pitch upon learning the news. Some looked distraught and inconsolable as cameras captured their reaction to the distressing news.Radnicki 1923 later confirmed the news in an official statement, saying, “With the deepest sorrow, we inform the public, fans and sports friends that our head coach, Mladen Zizovic, passed away during last night’s match between Mladost and Radnicki 1923 in Lucani. Our club has lost not only a great specialist but above all a good person, a friend, and a sports worker who, with his knowledge, energy, and nobility, left a deep mark in the hearts of all who knew him.The statement added, “Football Club Radnicki 1923 extends its sincerest condolences to his family, friends, and everyone who shared a love for football with him. Rest in peace, Mladen.”Zizovic, a former Bosnia and Herzegovina international midfielder, had only recently taken charge of Radnicki. He previously managed several clubs, including Borac Banja Luka, with whom he guided the side to their first-ever UEFA Conference League knockout tie last season.Borac also paid tribute to their former player and coach, noting, “You left us at 44, but your memory will live forever in every moment spent at our City Stadium – first as a player, then as a coach who achieved the greatest European success in our history.”Mladost Lucani coach Nenad Lalatovic told local media he had tried to help Zizovic before he lost consciousness.“I still can’t believe how life can turn upside down in a second,” he said. “Mladen was an exceptional man, a friend, and a professional. The football world has lost a great human being.”</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/football/top-stories/coach-collapses-mid-match-dies-players-fall-to-the-ground-in-heartbreaking-incident-watch/articleshow/125087900.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 18:22:09 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125088304,width-1070,height-580,imgsize-41700,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Cleared all police tests but lost job before joining; man wins case in HC</t>
-  </si>
-  <si>
-    <t>The circumstances preventing Rawal's joining were related to his being in judicial custody following the registration of an FIR against him. (AI image)
-What’s the case about?
-Why the Punjab and Haryana High Court ruled in the candidate’s favour
-Getting a job is no easy task, and losing it to untoward circumstances is unfortunate. One such case is of a Mr Rawal who got selected but couldn’t report within the specified time, and hence lost his job. He filed a case in the High court and won back his job.According to an ET report, following an advertisement on June 28, 2024, Mr Rawal submitted his application for a Constable position and completed the Common Eligibility Test. He successfully cleared both this test and a subsequent physical measurement assessment. However, when the Staff Selection Commission (SSC) issued him a call letter requiring him to join within 30 days, he failed to report for duty.The circumstances preventing Rawal's joining were related to his being in judicial custody following the registration of an FIR against him. Despite the court's eventual quashing of this FIR, the prescribed joining date and 30-day reporting period had already lapsed.Also Read | Income Tax department imposes Rs 2.2 lakh penalty on retired government employee for gratuity tax exemption claim - how she won case in ITAT Consequently, Rawal initiated legal proceedings under Articles 226/227 of the Constitution of India, seeking to challenge the order dated September 8, 2025, which had denied his request to assume the Constable position.As per the ET report, the sequence of events revealed that after Rawal's successful completion of the CET and physical measurement test, he qualified for the knowledge test.Shortly thereafter, he reported an incident where nine co-villagers allegedly attacked his family due to local factional disputes. This led to the registration of FIR No.232 on September 26, 2024, at the Panipat Police Station, invoking Sections 115, 126, 190, 191(3) and 351(2) of the Bharatiya Nyaya Sanhita, 2023 (BNS) against the accused individuals.The authorities lodged a cross FIR (FIR No. 234 dated September 28, 2024 under Sections 109(1), 115, 190, 191(2), 191(3), 351(2) of BNS) at the Panipat Police Station against Rawal and his family members, two days after the incident occurred.Subsequently, Rawal initiated legal proceedings (CRM-M-18856-2025) to nullify FIR No. 234, citing a compromise agreement as the basis.Through an order dated May 19, 2025, the Punjab and Haryana High Court invalidated the aforementioned FIR based on the compromise reached between parties.Also Read | Rs 8 lakh cash deposited in bank - man gets tax notice! Assessing officer deems it presumptive business income, but taxpayer wins case in ITAT - ruling explained Prior to the FIR's dismissal, the Haryana Staff Selection Commission had published the selected candidates' list on October 17, 2024, valid for one year. Police authorities notified him of his selection on November 11, 2024 and November 20, 2024, requesting him to commence service.Due to his judicial custody, his family requested an extension. Rawal submitted a personal request for extension through correspondence dated March 7, 2025.On July 16, 2025, the DGP transmitted Rawal's letter to the Superintendent of Police, instructing consideration of his case according to Rule 12.18 of Punjab Police Rules, 1934 (as applicable to the state of Haryana).The Superintendent of Police, respondent No.3, declined the candidate's application, citing government directives dated September 13, 2019, which stipulate a 30-day maximum period for assuming duties in fresh appointments.The state counsel of Haryana clarified to the court that the pending FIR or arrest were not the grounds for withholding the appointment letter. The rejection stemmed from the candidate's non-compliance with the 30-day joining window from the notification date.The state representative indicated that the joining notification was issued on November 20, 2024. Subsequently, the candidate's father submitted a written request on March 7, 2025, seeking an extension of the joining date. The government guidelines dated September 13, 2019, explicitly limit the joining period to 30 days.Also Read | Landlord vs tenant eviction case: Supreme Court rules in favour of landlord despite tenant’s son not signing rent receipts - here’s what the ruling means The state counsel emphasised that the petitioner's inability to join within the prescribed 30-day timeframe invalidated any subsequent attempts to assume the position. The respondent must adhere to state government regulations, which consequently prevents the petitioner from joining.On October 13, 2025, the Punjab and Haryana High Court issued a ruling in Rawal's favour.The Punjab and Haryana High Court, in its ruling (CWP-28252-2025), clarified that Rule 12.18 of PPR addresses circumstances when candidates face criminal implications. The court noted that the State counsel acknowledged that the petitioner (Rawal) was not affected by any negative conditions outlined in this Rule. His appointment was rejected solely because he failed to join within the stipulated 30-day period after receiving the appointment letter.The High Court observed that the respondent (government) denied the petitioner (Rawal) from joining service based on aforementioned directives, which were not statutory in nature.The court highlighted that Rule 12.18 of Punjab Police Rules (PPR) specifically deals with situations where candidates are implicated in criminal matters. However, the negative provisions of this Rule did not apply to the petitioner's (Rawal) situation.The High Court of Punjab and Haryana stated: "It is a settled proposition of law that instructions are binding on authorities, however, Courts are not bound by instructions."The High Court noted that rule 12.18(3) of PPR specifically addresses the current situation and does not mandate a 30-day joining period. The court observed that without statutory provisions, departmental guidelines could be considered directory rather than mandatory, additionally noting that courts are not bound by departmental directives.The Court expressed its considered view that the 30-day period specified in the instructions should not be applied in a rigid manner.The High Court asserted: "The difficulty of the candidate must be considered holistically and pragmatically. The instructions cannot be treated as sacrosanct to deny substantive benefit of appointment. It is a well known fact that there is scarcity of jobs in the country. The petitioner has cleared a rigorous selection process, thus, it would not be just and fair to deny him job opportunity on account of procedural lapse/delay. "In its deliberation, the Punjab and Haryana High Court issued the following directive: "In the wake of the above factual position, this Court is of the considered opinion that impugned order deserves to be set aside and accordingly set aside. The respondent is hereby directed to issue an appointment letter to the petitioner within two weeks from today and permit him to join subject to compliance of other terms and conditions of the appointment letter. Allowed. Pending application(s), if any, stands disposed of."Also Read | Income Tax department doubts Rs 10 lakh gift - brother gets tax notice for cash received from sisters; how he appealed &amp; won the case</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/business/india-business/he-cleared-all-police-tests-but-lost-his-job-before-joining-this-man-fought-back-in-court-why-high-court-ruled-in-his-favour/articleshow/125082698.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 19:17:03 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125084533,width-1070,height-580,imgsize-35618,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Dick Cheney: 'Darth Vader' who hated Donald Trump</t>
-  </si>
-  <si>
-    <t>Dick Cheney No More: Former VP's Family Drops Emotional Message, Reveals What Happened | WATCH
-The Wyoming Lineman Who Rose Too Far
-How the Hunter Became the Hunted
-The Cheney Doctrine
-FILE - Defense Secretary Dick Cheney poses with some of the U.S. Army troops stationed in southern Iraq in this May 7, 1991 file photo. (AP Photo/Bill Haber, File)
-Fire, Fury, and Forever Wars
-Redefining the Vice Presidency — and the Presidency Itself
-FILE - Richard "Dick" Cheney in White House, Washington on Nov. 4, 1975. He is nominated to be the White House chief of staff. (AP Photo/HB, file)
-The Halliburton Hangover and Other Idiosyncrasies
-The RINO Years and the Final Betrayal
-The Last Dick
-Long before Donald Trump, there was another American political figure ubiquitously reviled on late-night shows: Dick Cheney. He was often portrayed as evil incarnate, the epitome of late-stage capitalism, and in time would be compared to Darth Vader — Darth Sidious’s over-glorified apprentice whose claim to fame was murdering unarmed children.Disturbingly, or perhaps with a Freudian smile, Cheney leaned into the analogy, walking onto stages to the Imperial March and even putting a Darth Vader trailer hitch cover on his truck.Even Donald Trump despised him, labelling him a RINO (Republican in Name Only). In his final years, Cheney will be remembered for railing against Trump, even going so far as to endorse Kamala Harris — earning himself a Darth Vader–style redemption arc in the eyes of liberals, who instantly forgave his role as the “architect of the war on terror.” That war claimed millions of innocent lives when America invaded Iraq over non-existent weapons of mass destruction and unleashed regional instability that continues to haunt the world to this day.Born in Lincoln, Nebraska, and raised in the dusty town of Casper, Wyoming, Richard Bruce Cheney was not always destined for infamy. Twice arrested for DUI, expelled from Yale, and working as a power-line repairman, Cheney’s early life had all the makings of a cautionary tale.Instead, it became one of relentless reinvention. As he later recalled, it was his wife Lynne – “not interested in marrying a lineman for the county” – who gave him the ultimatum that pushed him back to university and into politics.By the 1970s, Cheney had become a disciple of Donald Rumsfeld (there are known knowns and known unknowns), rising through the ranks to become White House Chief of Staff under Gerald Ford. After serving six terms in Congress and a stint as George H. W. Bush’s Secretary of Defense, where he orchestrated Operation Desert Storm, Cheney was ready for retirement. Then came the call from a nepo-baby Texas governor looking for a vice-presidential running mate.George W. Bush’s 2000 campaign was supposed to be a return to steadier Republican values, and Dick Cheney was put in charge of vetting potential vice-presidential picks. Instead, he became the obvious choice. A Washington Post report remembers that Cheney initially demurred – he always preferred being the man behind the throne – rather than be on the ticket, but soon became inextricably linked to Dubyaman and his legacy. He brought gravitas, claimed Bush, but Cheney brought a lot more: complete mastery of the bureaucratic machine, a man who had a finger in every pie, knew how the wheels of Washington turned, and how to make the American political machine hum to his will. But then 9/11 struck and the world met a different Cheney: one whose legacy would go beyond greasing palms and convincing senators to fall in line.Unlike the Truman or Monroe doctrines, the ‘Cheney Doctrine’ was never truly worded, but its broad contours could still be understood by most folks. In one line, it could be summed up: strike first, ask later. Broadly, it meant pre-emptive war as self-defence (if there’s a one per cent chance that terrorists have WMDs, we have to treat it as a certainty), a radical shift from deterrence that led to the war against Saddam Hussein The second was his idea of the unitary executive theory, which took the words of the Constitution: “The executive power shall be vested in a President of the United States of America.” The line had always worried anti-federalists who believed that it was vesting too much power in the president without explaining the role of that executive power and how much power the executive ought to have.Cheney believed that the president (and by extension the vice president) ought to have total control over national security and foreign policy, with no interference from Congress, courts, or political oversight. It was this belief that led to the Patriot Act, warrantless wiretapping, and the expansion of surveillance and detention powers during the Bush era.And the third element was the notion that security outweighed liberty. “We have to work the dark side, if you will,” he said shortly after 9/11. “A lot of what needs to be done will have to be done quietly, without any discussion.” This became a guiding philosophy: fight unseen enemies with unseen methods. It justified CIA black sites, enhanced interrogation (torture), and a culture of secrecy that shielded executive decisions from scrutiny.It was Cheney, more than anyone else, who tied Saddam Hussein to al-Qaeda, pushing the now-debunked claim that hijacker Mohamed Atta met an Iraqi agent in Prague. “There’s overwhelming evidence there was a connection between al-Qaeda and the Iraqi government,” he said in 2004. There wasn’t.The so-called Cheney Doctrine combined pre-emptive war, regime change, and unchecked executive power into a dangerous cocktail. He believed in acting without waiting for threats to fully materialise — a philosophy that gave us the 2003 Iraq invasion. Cheney was the loudest voice claiming Saddam had WMDs. “Simply stated, there is no doubt that Saddam Hussein now has weapons of mass destruction,” he told the Veterans of Foreign Wars in August 2002.None were found. The cost: over 4,000 American soldiers, hundreds of thousands of Iraqi deaths, trillions of dollars, and a regional power vacuum that birthed ISIS. According to the Iraq Body Count project, more than 200,000 civilians have died violently since the invasion.Cheney also backed waterboarding, black sites, and indefinite detention at Guantanamo. “I was and remain a strong proponent of our enhanced interrogation program,” he wrote in his memoir. When confronted with the 2014 Senate Intelligence report calling such tactics brutal and ineffective, Cheney shrugged: “I’d do it again in a minute.”Cheney transformed the vice presidency into an unprecedented centre of power. He chaired secretive energy task forces, steered intelligence briefings, and personally approved portions of the CIA’s detention and interrogation program. He even argued that the vice president was not part of the executive branch for disclosure laws, but was when it came to privilege.He was Carl Schmitt in cowboy boots, crafting a state of exception for a post-9/11 America. Every crisis was an opportunity to expand presidential powers unchecked by Congress or courts. The “unitary executive theory” wasn’t just academic; under Cheney, it became operational doctrine.Even George W. Bush began to bristle. Their relationship fractured when Bush refused to pardon Cheney’s aide, Scooter Libby, convicted of perjury and obstruction of justice. Cheney was reportedly furious. “He left the presidency weaker than he found it,” said former aide Lawrence Wilkerson, who called Cheney “a vice president of a different kind — an unelected co-president.”Before he was vice president, Cheney was CEO of Halliburton, a global oil services giant. During the Iraq and Afghanistan wars, Halliburton was awarded billions in no-bid contracts to rebuild, supply, and fuel the US military machine. Cheney claimed he had divested his interests, but the optics were damning: a war that enriched one of America’s largest defence contractors — and its former CEO.Then there were the smaller, stranger moments. In 2006, he accidentally shot his hunting partner, 78-year-old attorney Harry Whittington, in the face during a quail hunt in Texas. The story broke a full day later through local press, not the White House. When Whittington apologised to Cheney for the inconvenience, it was peak Cheney: power so absolute it needn’t explain itself.Add to that his 2012 heart transplant, his deadpan humour about having “no pulse,” his fondness for fly-fishing, and his refusal to ever show remorse, and you get the man in full — impervious, unapologetic, and darkly absurd.In his final act, the Darth Vader of the Bush era found himself cast out by the empire he helped build. The Tea Party had no use for him. The MAGA movement despised him. And Donald Trump, ever the grudge-holder, called Cheney a “disaster” and a “RINO.” Cheney returned the favour with gusto.“In our nation’s 246-year history, there has never been an individual who is a greater threat to our republic than Donald Trump,” he said in a 2022 campaign ad for his daughter, Liz Cheney. That same year, he stood in the Capitol and condemned his own party: “It’s not leadership that resembles any of the folks I knew when I was here for ten years.”When Trump refused to concede the 2020 election, Cheney recoiled. When the Capitol was stormed on January 6, he called it “a tragedy” and an “ongoing threat.” And in a final, symbolic blow to the party he once helped define, Cheney said he voted for Kamala Harris in 2024. “Because duty to the Constitution,” he said, “must come before party.”Cheney died in November 2025 at the age of 84 from complications of pneumonia and heart disease. His family called him “a noble giant of a man.” His critics might call him the architect of ruin. But everyone agrees: he reshaped the American presidency, bent the arc of global history, and never once looked back. Long before Trump normalised authoritarian instincts in public, Cheney operationalised them in secret without even bothering to tweet about it. Cheney might have found redemption among Never-Trumper liberals, but for those who have to live in the world, Darth Vader has no redemption — only the haunting echo of the Imperial March.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/world/us/dick-cheney-the-war-on-terror-architect-who-loved-being-called-darth-vader/articleshow/125089487.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 19:37:48 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125089581,width-1070,height-580,imgsize-100878,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>‘Ensure elimination of all…’: Himanta links Shahabuddin's son to Laden</t>
-  </si>
-  <si>
-    <t>Himanta Biswa Sarma addressing the rally in Siwan (ANI)
-'Will Cut Off Your Tongue': Bihar Poll Campaign Turns Ugly, AIMIM Candidate Threatens Tejashwi Yadav
-NEW DELHI: Assam chief minister Himanta Biswa Sarma on Tuesday targeted RJD candidate Osama Shahab - son of late gangster-turned-politician Mohammad Shahabuddin - at an election rally in Bihar’s Siwan district, drawing a controversial comparison between him and terrorist Osama Bin Laden.Addressing a public meeting in the Raghunathpur assembly segment, Sarma said, “Before I came to Raghunathpur, I thought I would see Lord Ram, Lord Lakshman and Goddess Sita, but I was told that there are many Ram, Laxman and Sita here and there is also Osama. So I asked, who is Osama? This Osama is like the earlier Osama Bin Laden. We have to ensure the elimination of all Osama Bin Ladens in the state. What was Osama's father's name? He was called Shahabuddin. ..”The BJP leader also claimed that Osama Shahab’s electoral win would amount to a setback for Hindus.“If such an Osama wins from Raghunathpur, it will be a defeat for Hindus. I shall myself be watching the results of this constituency on November 14, sitting at the gates of Kamakhya temple in Assam. I am sure you people will reject Osama just as you had defeated his mother in Lok Sabha polls,” Sarma said, referring to Hina Shahab, widow of Mohammad Shahabuddin, who had contested the parliamentary election as an Independent.Osama Shahab, 31, is contesting from Raghunathpur on a Rashtriya Janata Dal ticket, making his political debut from what is considered his father’s stronghold. The Janata Dal (United) has fielded Vikash Kumar Singh from the seat, while Prashant Kishor’s Jan Suraaj has nominated Rahul Kirti. Osama faces several criminal cases, mostly under the Arms Act, 1959.Continuing his attack, Sarma also touched on issues from his home state, saying that as Assam’s chief minister he had worked to “free 50,000 acres of land from infiltrators” and stopped government funding for madrasa teachers. “The infiltrators also pose a threat to our womenfolk. The Congress had been footing the bill for the salaries of teachers at Madrasas. I put an end to it, making it clear the government is supposed to train doctors and engineers, and not mullahs,” he said.He further claimed he would soon bring a law in Assam to punish men marrying multiple times. “Later this month, I am also going to bring a law that would send to jail those who marry three to four times. I am going to shut down this shop,” he told the gathering.Also read: 'Bachaa hai': Tej Pratap's 'jhunjhuna' jibe at Tejashwi; threatens to campaign in Raghopur Appealing for support to the NDA, Sarma urged voters to back CM Nitish Kumar and reject the “Tejashwi-Osama duo.” He said, “Awakened Hindus defeated the legacy of Babur and Aurangzeb in Ayodhya, where a temple of Lord Ram stands. They will again beat Osama.”The upcoming Bihar assembly elections will be held in two phases on November 6 and 11, with results scheduled for November 14.The contest is primarily between the ruling NDA - comprising BJP, JD(U), LJP (Ram Vilas), HAM (Secular) and Rashtriya Lok Morcha - and the RJD-led Mahagathbandhan, which includes Congress, CPI(ML), CPI, CPM and the Vikasheel Insaan Party.(With inputs from agencies)</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/bihar-polls-ensure-elimination-of-all-himanta-links-shahabuddins-son-to-laden-warns-his-victory-will-be-defeat-for-hindus/articleshow/125086430.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 17:05:52 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125086442,width-1070,height-580,imgsize-729104,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Who is Michelle Scully? Twitch's global communications head leaving after a year and a half</t>
-  </si>
-  <si>
-    <t>Twitch (Image Courtesy: Twitch via Variety)
-What has Michelle Scully accomplished during her time at Twitch?
-Michelle Scully, Twitch’s Global Head of Communications, is stepping down after just a year and a half in the role. Her departure marks a major leadership change for the Amazon-owned streaming platform, which has been navigating rapid shifts in the creator and entertainment world. Before Twitch, Scully led brand communications for Amazon Studios and managed consumer communications for Amazon Devices and Alexa. She also spent over a decade at Edelman, where she worked with global brands on storytelling and reputation management.During her tenure, Scully helped shape how Twitch communicates with its global community, media, and fans, strengthening its voice in a fast-moving digital landscape. With her exit, Twitch is now searching for a successor who can continue building its identity while expanding its reach beyond gaming into broader entertainment and cultural spaces.Michelle Scully joined Twitch in March 2024, following Brielle Villablanca's move to Patreon. Announcing her departure, Scully wrote on LinkedIn,“After an incredible journey at Twitch, I’ve made the difficult decision to move on and pursue a new opportunity.Leaving is bittersweet — working at Twitch is the best job I’ve ever had, and I’ve loved being part of such an amazing team and community.”Her experience at Amazon Studios made her a natural fit for Twitch, where she strengthened the platform’s messaging and helped it navigate a rapidly evolving digital and cultural landscape. Scully’s exit opens the door for a new leader who will help define Twitch’s public identity.The company’s job posting outlines an ambitious vision: “You'll define how Twitch shows up from traditional media and podcasts, to community forums and the countless places where internet culture is made and conversation happens in real time.” The new hire will report to CMO Rachel Delphin and can work from San Francisco, Seattle, Los Angeles, New York City, or Irvine.The role is central to balancing Twitch’s community-driven identity with its expanding reach in mainstream media and entertainment. Scully laid a strong foundation, and the next communications leader will need to continue shaping the platform’s voice, ensuring it stays authentic while navigating its next phase of growth.Also read: Is Justin Bieber quitting music? His Halloween Twitch confession about his 'daunting tour' leaves fans heartbroken</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/world/us-streamers/who-is-michelle-scully-twitchs-global-communications-head-leaving-after-a-year-and-a-half/articleshow/125089361.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 20:19:42 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125090221,width-1070,height-580,imgsize-5868,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Blake Treinen’s viral Charlie Kirk hat: What’s the real story?</t>
-  </si>
-  <si>
-    <t>Did Blake Treinen really wear a Charlie Kirk hat during the World Series? The truth behind the viral photo (Image via X)
-Blake Treinen’s tribute hat photo sparks Charlie Kirk confusion after Dodgers’ World Series win
-Social media users wrongly claim Blake Treinen wore the Charlie Kirk hat in the World Series
-A new rumor about Los Angeles Dodgers pitcher Blake Treinen spread online after the team’s World Series win on Saturday, November 1, 2025. The claim said Treinen wore a hat with “Charlie Kirk” written on it during the World Series celebration. But this claim is false. The viral picture that started it all was not from the World Series.It was from a September 12 game against the San Francisco Giants, weeks before the championship series. The image began circulating after a Facebook post by user Scott Mandel falsely said Treinen wore the hat “during the World Series.” Several pages, including The Dodgers TOP, then reposted the same image, spreading the wrong information further.The photo is real, but it’s old. During the September 12, 2025 game in San Francisco, Blake Treinen wore a special white hat with “Charlie Kirk” written on it and two small Christian crosses. This was to honor Charlie Kirk, the founder of Turning Point USA (TPUSA), who was shot and killed on September 10 during an event at Utah Valley University.According to Fox News, Blake Treinen, who is known for his strong Christian faith, wore the tribute hat as a personal gesture. Musician Sean Feucht shared photos and a short video from that game on Instagram, writing:“My friend and pitcher for the Dodgers, Blake Treinen, played with this on his hat last night.”Feucht later posted another video from October 8, showing Treinen giving the hat away after a game against the Philadelphia Phillies, and thanked him for “remembering Charlie Kirk tonight.”After the Dodgers’ World Series win, the same September photo began to recirculate on Facebook and X. Some users wrongly claimed the hat appeared during the World Series celebration.Also Read: Barack Obama Sends Heartfelt Reaction To Los Angeles Dodgers’ World Series Triumph After Nerve-Racking Game 7 Over Toronto Blue Jays Fact-checking sites including Primetimer and Fox News confirmed that the image was not taken during the World Series. There are no verified photos or videos showing Blake Treinen wearing the Charlie Kirk tribute hat at the title celebration or any 2025 postseason game.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/mlb/news/did-blake-treinen-really-wear-a-charlie-kirk-hat-during-the-world-series-the-truth-behind-the-viral-photo/articleshow/125068415.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 01:30:29 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125068376,width-1070,height-580,imgsize-832071,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+    <t>Trump gushes over Taylor Swift as Travis Kelce stays quiet after Chiefs absence</t>
+  </si>
+  <si>
+    <t>Taylor Swift sparks political and NFL buzz as Donald Trump flips from “I HATE TAYLOR SWIFT” to calling her a “terrific person,” while the White House uses her song in a TikTok. Fans question her absence from the Kansas City Chiefs' game and Travis Kelce stays quiet as online speculation grows around the couple and the moment.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/nfl/news/i-hate-taylor-swift-to-terrific-person-trumps-taylor-tough-love-sparks-fan-buzz-over-her-chiefs-game-no-show-as-travis-kelce-stays-quiet/articleshow/125091230.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:38:31 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091285,width-1070,height-580,imgsize-87864,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Charlise Springer breaks silence after Blue Jays' World Series heartbreak</t>
+  </si>
+  <si>
+    <t>George Springer with his wife Charlise (Image via: Charlise Springer's IG)
+Charlise Springer’s words remind fans what baseball truly stands for
+A season that tested every ounce of heart, faith, and resilience
+Looking ahead as the Blue Jays promise to ‘run it back’
+When the Toronto Blue Jays’ dream run came to a heartbreaking end in Game 7 of the World Series, it wasn’t just the players who felt the pain—it was their families, the fans, and an entire nation that had believed in their story. After leading the series 3–2 and returning home to Rogers Centre with hopes of ending a 32-year title drought, the Blue Jays watched their fairytale slip away. Costly missed chances in Game 6 and a gut-wrenching ninth-inning home run by Miguel Rojas sealed their fate, leaving the stadium heavy with silence and disbelief.A day later, while the city was still nursing its heartbreak, George Springer’s wife, Charlise Springer, stepped forward with a message that struck deep emotional chords. Her heartfelt words, filled with gratitude, pride, and grace, reminded everyone that baseball is more than just wins and losses—it’s about resilience, connection, and moments that outlast the scoreboard. “I’m so proud of my husband, this team and every single family that poured their hearts into this season,” she wrote. “The highs, the late nights, the travel, the memories. Baseball doesn’t promise fairytale endings, but it gives you people and moments that last a lifetime.Feeling nothing but gratitude for the chance to represent Canada’s team and be part of something so special🇨🇦 💙 Until next season🐎#RunItBack.”Charlise’s post quickly spread across social media, not for its glamour, but for its sincerity. Thousands of fans flooded the comments, calling her words “beautiful,” “real,” and “exactly what the city needed to hear.” In a moment of collective heartbreak, her message brought perspective—it wasn’t about the loss, but about the love, loyalty, and shared memories that baseball creates. Her reflection reminded everyone that behind every player’s jersey is a family that lives every win and loss just as deeply.For the Blue Jays, this wasn’t just another playoff push—it was a season that redefined their identity. From battling injuries and midseason slumps to clawing their way into the postseason spotlight, Toronto defied every odd stacked against them. Charlise’s words, “This group showed nothing but heart, humility and resilience from day one and it was an honor to watch them chase this dream together ,” perfectly echoed what fans had witnessed all season long—a team that played for each other and carried the weight of a nation on their shoulders.George Springer, one of the veterans who has become the emotional heartbeat of the clubhouse, embodied that spirit of fight. Through every late-night comeback and pressure-packed inning, he stood as a symbol of belief and leadership. And while the final chapter didn’t end in celebration, it unfolded with the kind of grit that defines lasting legacies.Though the pain of this loss may linger through the winter, the message of hope remains loud and clear. With their core still intact and a fanbase unwavering in belief, the Blue Jays are already turning the page with one mantra: Run it back. As Charlise Springer so beautifully expressed, baseball may not always deliver fairytales—but it always delivers moments that stay forever. And for Toronto, that story is far from over. Because every heartbreak in this city, only fuels a stronger comeback.Also read: Shohei Ohtani’s rare Game 7 moment sparks fiery exchange as Toronto Blue Jays’ manager John Schneider confronts umpire in World Series showdown</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/mlb/news/no-fairytale-ending-george-springers-wife-charlise-breaks-silence-after-toronto-blue-jays-devastating-world-series-loss/articleshow/125046637.cms</t>
+  </si>
+  <si>
+    <t>Mon, 03 Nov 2025 09:52:24 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125046684,width-1070,height-580,imgsize-88814,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Lakers legend praises Bronny James after strong game vs Trail Blazers</t>
+  </si>
+  <si>
+    <t>Bronny James showcased a standout performance for the Los Angeles Lakers against the Portland Trail Blazers, contributing five points and six assists. Lakers legend James Worthy lauded the young guard's game, calling it potentially his best yet. Coach JJ Redick also praised Bronny's defensive intensity and physicality, highlighting his significant contributions in a crucial fourth-quarter stretch.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/nba/top-stories/former-los-angeles-lakers-legend-drops-huge-praise-for-lebron-james-son-bronny-james-after-stellar-show-against-portland-trail-blazers/articleshow/125083907.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 15:25:55 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125083894,width-1070,height-580,imgsize-768890,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Brittany Mahomes slams “disgusting” Bills fan stunt ahead of Chiefs vs Bills</t>
+  </si>
+  <si>
+    <t>Ahead of the Chiefs-Bills game, a past incident involving Brittany Mahomes and a fan display in Buffalo has resurfaced. She publicly condemned a disrespectful Kermit the Frog puppet mocking Patrick Mahomes, urging for basic decency. This reminder of respect underscores the intense rivalry, proving that even amidst fierce competition, human dignity remains paramount.
+Brittany Mahomes felt the line was crossed and she wanted the public to know it
+As Patrick Mahomes returns to Buffalo, the stakes are different — but emotions are always present
+For most NFL spouses, game week tends to mean travel, schedules, childcare adjustments, and a flood of national attention, but for Brittany Mahomes, there’s history attached to Buffalo. And not the fun, competitive kind. Before this weekend’s Chiefs-Bills showdown, an old incident involving a Bills supporter is circulating again online, reminding fans that not every rivalry moment lives only inside the stadium walls.Brittany, who has been in the public eye alongside Patrick Mahomes since college, once publicly reacted to a fan display that crossed a major line. Now, with yet another high-stakes meeting on the schedule, the memory of that moment is once again part of the conversation.Ahead of a previous Chiefs-Bills matchup, Brittany Mahomes addressed what she considered to be one of the ugliest fan moments she had ever seen involving her family. A Kermit the Frog puppet, wearing a Patrick Mahomes No. 15 jersey, was hung publicly in Buffalo.Brittany's reaction was immediate, emotional, and blunt. “Do we remember this, Buffalo? Absolutely disgusting,” she posted. She also followed that with a pointed reminder about basic decency in sports culture, writing, “So as you go home tonight, I pray we become better people.”Those words weren’t just about trash talk. They were about human respect and they still land heavily today.Sunday's meeting wasn't just another regular season date. Patrick Mahomes and Josh Allen have developed the kind of on-field rivalry that dictates national windows, defines postseason eras, and fuels nonstop football debate. Kansas City enters with momentum. Buffalo enters with swagger. Both enter with pressure.And on the periphery of all that football energy sits a memory from November 2024, a moment Brittany Mahomes hasn’t forgotten, and clearly never wanted normalized. It proves one thing: rivalries can be electric. But respect still matters, especially when the entire world is watching.Also Read: “A sad, pathetic, nobody loser”: Swifties unleash fury on Kayla Nicole after Halloween stunt reignites drama with Travis Kelce and Taylor Swift</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/nfl/news/absolutely-disgusting-brittany-mahomes-harsh-reaction-to-a-disturbing-bills-fan-stunt-is-trending-again-ahead-of-chiefs-vs-bills-game/articleshow/125032973.cms</t>
+  </si>
+  <si>
+    <t>Mon, 03 Nov 2025 04:20:00 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125032973,width-1070,height-580,imgsize-30970,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1271,7 @@
         <v>25</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1291,19 +1279,19 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1311,19 +1299,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1331,19 +1319,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1351,19 +1339,19 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1371,19 +1359,19 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1391,19 +1379,19 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1411,19 +1399,19 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1431,19 +1419,19 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1451,19 +1439,19 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1471,19 +1459,19 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1491,19 +1479,19 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1511,19 +1499,19 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1531,19 +1519,19 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1551,19 +1539,19 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>21</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1571,19 +1559,19 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>93</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1591,419 +1579,419 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B22" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E24" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E27" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E29" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C30" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B31" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E31" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C32" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E32" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C34" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E34" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B35" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B36" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C36" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E36" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B37" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C37" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E37" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B38" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B39" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C39" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E39" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B40" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C40" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E40" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B41" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C41" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E41" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AM made different endpoints instead of one
</commit_message>
<xml_diff>
--- a/server/RSS_FullText.xlsx
+++ b/server/RSS_FullText.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="199">
   <si>
     <t>Source</t>
   </si>
@@ -35,6 +35,49 @@
   </si>
   <si>
     <t>TheHindu</t>
+  </si>
+  <si>
+    <t>Suvendu Adhikari leads ‘Parivartan Yatra’ rally, demands ‘proper’ execution of SIR in West Bengal</t>
+  </si>
+  <si>
+    <t>Leader of Opposition Suvendu Adhikari led a Bharatiya Janta Party rally named ‘Parivartan Yatra’ (walk for change) on Tuesday (November 4) in the outskirts of Kolkata. The protestors demanded that every Bangladeshi infiltrator be deported from the country and the Special Intensive Revision (SIR) of the electoral rolls be completely undertaken across the State.
+This comes as the door-to-door distribution of enumeration forms began in the State on Tuesday (November 4, 2025), and simultaneously Chief Minister Mamata Banerjee held a rally in central Kolkata to protest against the SIR process.
+Earlier in the day on Tuesday, Mr. Adhikari led a BJP delegation and met with the Chief Electoral Officer, West Bengal at his Kolkata office to file a deputation to raise concerns about the irregularities in the SIR process in some parts of the State and the alleged interference of the ruling party members.
+Supporters of BJP raised slogans and accused Ms. Banerjee and the ruling Trinamool Congress of manipulating the death of every individual in West Bengal to link it to SIR.
+“We want a voter list free of errors and infiltrators. This rally is to respect the Election Commission, whereas, Ms. Mamata is conducting a rally with infiltrators,” Mr. Adhikari said.
+BJP supporters carried posters that said, “Detect. Delete. Deport” — a message directed towards alleged infiltrators. Mr. Adhikari also urged Booth Level Officers (BLOs) to not get trapped by any provocation caused by the ruling party members and let the Election Commission of India take all legal steps to protect them. This comes as there have been multiple allegations by BLOs across the State about facing threats from various factions of society.
+“If they [TMC] harm or attack any of our Booth Level Agents (BLA), BJP leaders like myself will settle the score with them,” Mr. Adhikari said. He also said that if the TMC does not allow the SIR process to be conducted and delay elections, they will ensure the State goes under President’s Rule.
+“SIR had been undertaken at least eight times and was necessary for the interest of the country and saving its integrity and democracy. Why has the TMC suddenly woken up to the issue and is trying to derail the process. People have seen through their games,” he said, calling for ‘parivartan’ (change) in West Bengal.
+Mr. Adhikari also dared the TMC to stop the SIR process in West Bengal and called their opposition of the exercise “unconstitutional”.
+According to official records shared by the CEO, West Bengal office, more than 16 lakh enumeration forms were distributed across the State on the first day of the door-to-door activity.
+At her rally, Ms. Banerjee vowed she would not let any single genuine voter to be removed from the voter list and accused the BJP of tagging everyone speaking in Bengali as Bangladeshi.
+“So many years after the partition, now I will have to prove my citizenship? The last SIR took 2 years, then why this time it is being hurried in 2 months?” Ms. Banerjee raised questions.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/west-bengal/suvenduadhikari-leadsparivartan-yatra-rally-demands-proper-execution-of-sir-in-west-bengal/article70240550.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:00:17 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/3zm0aq/article70241654.ece/alternates/LANDSCAPE_1200/20251104320L.jpg</t>
+  </si>
+  <si>
+    <t>Hyderabad sees intermittent rainfall on Tuesday, IMD forecasts more showers in next 24 hours</t>
+  </si>
+  <si>
+    <t>Several parts of Hyderabad witnessed moderate to heavy rainfall on Tuesday (November 4) bringing brief relief from the prevailing warm conditions during the day. The rains, which were intermittent throughout the day, did not result in waterlogging or major traffic disruptions. By evening, showers had largely subsided across most areas.
+According to data from the Telangana Development Planning Society (TGDPS), as of 9 p.m., Chandrayangutta recorded a rainfall of 38.8 mm followed by 29.5 mm in Hayathnagar, 26.8 mm in Uppal, 24 mm in Vanasthalipuram, 22.5 mm in Karvan, 21.3 mm in Bandlaguda, 20.8 mm in Falaknuma, 18 mm in LB Nagar, 17.3 mm in Kanchanbagh, 15 mm in Nagole and 10.8 mm in Mehdipatnam.
+The India Meteorological Department (IMD) has forecast light rain in Hyderabad and surrounding areas over the next 24 hours. “The city will see a partly cloudy sky. Light rain or thundershowers accompanied by gusty winds are very likely to occur. Mist or hazy conditions may prevail during morning and night hours. The maximum and minimum temperatures are expected to hover around 32°C and 23°C respectively,” the IMD bulletin stated.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/cities/Hyderabad/hyderabad-sees-intermittent-rainfall-on-tuesday-imd-forecasts-more-showers-in-next-24-hours/article70241222.ece</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 23:35:46 +0530</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/theme/images/og-image.png</t>
   </si>
   <si>
     <t>Asphalt Hebbal flyover immediately: GBA chief</t>
@@ -51,9 +94,6 @@
   </si>
   <si>
     <t>Tue, 04 Nov 2025 23:25:27 +0530</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/theme/images/og-image.png</t>
   </si>
   <si>
     <t>Kerala University PhD scholar alleges caste bias, abuse of power by Sanskrit department head</t>
@@ -406,55 +446,6 @@
   </si>
   <si>
     <t>Tue, 04 Nov 2025 22:14:55 +0530</t>
-  </si>
-  <si>
-    <t>SP renews push for full-fledged AMU centre in Kishanganj as Akhilesh’s Bihar campaign gathers pace</t>
-  </si>
-  <si>
-    <t>As Samajwadi Party (SP) president Akhilesh Yadav campaigns extensively in Bihar for the Assembly polls, his party on Tuesday reiterated its demand for the completion and full functioning of the satellite branch of Aligarh Muslim University (AMU) in Kishanganj district of Bihar.
-The party described the educational backwardness of the Seemanchal region, of which Kishanganj is a part, as the primary cause of its economic underdevelopment and that of Bihar. It added that the SP is keen to address Seemanchal’s developmental needs, calling for a broader solidarity of socialist and democratic forces to create world-class educational infrastructure.
-“We did advocate for the AMU Kishanganj campus, aligning with our broader social justice and PDA rights agenda. Bureaucratic hurdles such as land acquisition and thus infrastructure planning contributed to the delay. The SP is keen to address Seemanchal’s development, especially after the Sachar Committee Report, raising this issue for which the SP stands for its secular and socialist ideologies and being the third largest party in Parliament is playing the role of a national-level secular alternative. Championing AMU Kishanganj will serve as a symbolic and substantive commitment to educational equity,” SP spokesperson Naseer Salim said.
-Mr. Salim, who is the great-grandson of Lady Anees Imam, one of the founders of modern Bihar who played a distinctive role in the anti-colonial movement before Independence, added that the PDA (Pichhda, Dalit, Alpsankhyak) plank, which also includes aadhi aabadi (women) and upper castes, remains central to the SP’s vision.
-The AMU Kishanganj campus remains incomplete even after more than a decade, operating from temporary buildings with only one functional course. The branch, established in 2011 as part of a nationwide initiative for higher education among Muslim populations following recommendations by the Ministry of Human Resource Development, currently functions from a temporary structure at Halim Chowk in Kishanganj.
-The Seemanchal region is considered one of the most backward parts of India in terms of education and nearly all other indices of human development.
-Another senior SP leader and national spokesperson, Ram Pratap Singh, said, “The PDA ideology of the Samajwadi Party is for creating infrastructure and delivery of world-class education at all levels. This would mean that we not only have to strengthen our existing institutions of higher learning but replicate successful models across the country.”
-Mr. Yadav is currently campaigning across Bihar, addressing multiple rallies daily in support of INDIA bloc candidates.
-Speaking about the activism of Lady Anees Imam, Mr. Salim said, “Lady Anees Imam’s activism was deeply intertwined with social reform and the educational upliftment of women in Bihar. Her struggle was not just political; it was cultural and educational, aimed at transforming the mindset of a society that had long excluded women from public and intellectual life.
-“Lady Imam was among the first Muslim women in Bihar to publicly reject purdah, challenging entrenched patriarchal norms across both Hindu and Muslim communities. She founded institutions like Aghor Kamini Shilpalaya and Aghor Nari Pratishan, which provided industrial and vocational education to women, especially in Patna and surrounding regions. Her struggle was not just about resisting colonial rule; it was about reshaping society from within, empowering women to become agents of change.”
-Asked whether Lady Imam contributed to the anti-colonial movement in the United Provinces, present-day Uttar Pradesh, Mr. Salim said her primary base was Bihar, though her influence extended beyond regional boundaries.
-“She led a delegation to England on behalf of the All-India Congress to oppose the Montague-Chelmsford Reforms of 1919, a national-level intervention that impacted policies across British India, including the Hindi belt. Her contributions were more national in scope, rather than geographically centred in the Hindi belt. Her work bridged elite and grassroots activism, showing that upper-caste Muslim women could be powerful agents of change in a deeply stratified society,” the SP spokesperson said.
-When asked whether the magnitude of social injustice against women has declined in recent decades or merely reinvented itself, SP national spokesperson Ram Pratap Singh said, “Yes and no is my answer. Yes, education, healthcare and social welfare have marginally become better. More is being talked about to generate political optics but in real terms the delivery on the ground is a distant dream. The West-inspired model of development of the last two decades has not created any significant opportunities for women, as is evident from an abysmally low, around 15%, female participation in the labour force in most Indian States. Rural infrastructure, which impacts women the most, has also not much improved.”</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/bihar/sp-renews-push-for-full-fledged-amu-centre-in-kishanganj-as-akhileshs-bihar-campaign-gathers-pace/article70240274.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:13:36 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/news/national/erscb1/article70241434.ece/alternates/LANDSCAPE_1200/THJVNALIGARHMUSLIMUNIVERSITY.jpg</t>
-  </si>
-  <si>
-    <t>Karnataka releases a new Skill Development Policy; to train 3 million youth by 2033</t>
-  </si>
-  <si>
-    <t>Chief Minister Siddaramaiah on Tuesday unveiled Karnataka’s new Skill Development Policy 2025–32, here.
-Speaking at the inaugural ceremony of the Bengaluru Skill Summit, the Chief Minister said the policy came with a seven-year strategic blueprint, backed by a robust outlay of ₹4,432 crore.
-“This aims to position Karnataka as a global hub for a skilled, inclusive, and future-ready workforce,’’ he added.
-Mr. Siddaramaiah also said that his government has been, since 2023, redefining its skilling vision to align with the demands of a rapidly changing, post pandemic, global economy.
-According to Sharanaprakash Patil, Minister for Medical Education, Skill Development, Entrepreneurship &amp; Livelihood Ends, the new Karnataka State Skill Development Policy 2025–32 aims to train 3 million youth by 2032. “This policy document will serve as the backbone for the state’s skilling vision, integrating schemes, improving quality and aligning with the $1 trillion economic goal,” he added while speaking at the opening session of a two-day Skill Development Summit which began on Wednesday.
-The policy also envisages to increase women’s ITI enrolment to 33%, to double district-level skilling capacity, and to strengthen global placement linkages through the International Migration Centre–Karnataka (IMC-K). It focuses on lifelong learning, reskilling, and upskilling, with strong industry collaboration through apprenticeships and partnerships. It also proposes special interventions for women, persons with disabilities, marginalised communities, and the informal workforce.
-Speaking on the occasion, Deputy Chief Minister D.K Shivakumar said Karnataka’s commitment to global partnership in knowledge sharing was critical to shape its workforce development. He said the State produced more than 1.6 lakh engineering graduates annually through 270 colleges and operated 1,160 ITIs, contributing to a robust talent pipeline for domestic as well as global enterprises.
-The Skill summit is being organised by the Karnataka Skill Development Corporation (KSDC), Karnataka Skill Development Authority (KSDA) and the Karnataka Digital Economy Mission (KDEM). The Hindu is a media partner of the event.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/karnataka-releases-a-newskill-development-policy-to-train-3-million-youth-by-2033/article70241395.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:10:36 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/psmua3/article70241446.ece/alternates/LANDSCAPE_1200/_DSC4507.JPG</t>
   </si>
   <si>
     <t>TOI</t>
@@ -1308,7 +1299,7 @@
         <v>15</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1316,19 +1307,19 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1336,19 +1327,19 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1356,19 +1347,19 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1388,7 +1379,7 @@
         <v>32</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1396,19 +1387,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" t="s">
         <v>36</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1428,7 +1419,7 @@
         <v>41</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1436,19 +1427,19 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1468,7 +1459,7 @@
         <v>50</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1476,19 +1467,19 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" t="s">
         <v>54</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1496,19 +1487,19 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" t="s">
         <v>59</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1548,7 +1539,7 @@
         <v>69</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1556,19 +1547,19 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
         <v>71</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" t="s">
         <v>73</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1576,19 +1567,19 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
         <v>76</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" t="s">
         <v>78</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1628,7 +1619,7 @@
         <v>88</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1668,407 +1659,407 @@
         <v>97</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>98</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" t="s">
         <v>99</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>100</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" t="s">
         <v>102</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" t="s">
         <v>105</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" t="s">
         <v>107</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" t="s">
         <v>110</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" t="s">
         <v>112</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" t="s">
         <v>115</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" t="s">
         <v>117</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B26" t="s">
+        <v>119</v>
+      </c>
+      <c r="C26" t="s">
         <v>120</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" t="s">
         <v>122</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" t="s">
         <v>125</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="E27" t="s">
         <v>127</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B28" t="s">
+        <v>129</v>
+      </c>
+      <c r="C28" t="s">
         <v>130</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" t="s">
         <v>132</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29" t="s">
         <v>135</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" t="s">
         <v>137</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B30" t="s">
+        <v>139</v>
+      </c>
+      <c r="C30" t="s">
         <v>140</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" t="s">
         <v>142</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" t="s">
         <v>145</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" t="s">
         <v>147</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B32" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32" t="s">
         <v>150</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" t="s">
         <v>152</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B33" t="s">
+        <v>154</v>
+      </c>
+      <c r="C33" t="s">
         <v>155</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" t="s">
         <v>157</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B34" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34" t="s">
         <v>160</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" t="s">
         <v>162</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B35" t="s">
+        <v>164</v>
+      </c>
+      <c r="C35" t="s">
         <v>165</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" t="s">
         <v>167</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
+        <v>169</v>
+      </c>
+      <c r="C36" t="s">
         <v>170</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" t="s">
         <v>172</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B37" t="s">
+        <v>174</v>
+      </c>
+      <c r="C37" t="s">
         <v>175</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" t="s">
         <v>177</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B38" t="s">
+        <v>179</v>
+      </c>
+      <c r="C38" t="s">
         <v>180</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" t="s">
         <v>182</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B39" t="s">
+        <v>184</v>
+      </c>
+      <c r="C39" t="s">
         <v>185</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" t="s">
         <v>187</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B40" t="s">
+        <v>189</v>
+      </c>
+      <c r="C40" t="s">
         <v>190</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" t="s">
         <v>192</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B41" t="s">
+        <v>194</v>
+      </c>
+      <c r="C41" t="s">
         <v>195</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" t="s">
         <v>197</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed the non existing file
</commit_message>
<xml_diff>
--- a/server/RSS_FullText.xlsx
+++ b/server/RSS_FullText.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="200">
   <si>
     <t>Source</t>
   </si>
@@ -35,6 +35,26 @@
   </si>
   <si>
     <t>TheHindu</t>
+  </si>
+  <si>
+    <t>Ahmedabad’s Atal Bridge attracts 77.7 lakh visitors, generates ₹27 crore revenue</t>
+  </si>
+  <si>
+    <t>The Atal Bridge across the Sabarmati River in Ahmedabad has drawn more than 77.71 lakh visitors since its inauguration, generating ₹27.70 crore in revenue for the Ahmedabad Municipal Corporation (AMC) over three years, according to data released by the Sabarmati Riverfront Development Corporation Ltd. (SRFDCL).
+Inaugurated by Prime Minister Narendra Modi in August 2022, the ₹74-crore Atal Foot Over Bridge has become one of the city’s most visited attractions. The bridge continues to attract visitors from across India and abroad, especially during festivals and holiday seasons.
+Between April and October 2025, the bridge received 8.51 lakh visitors and collected ₹4.82 crore in revenue. From August 2022 to October 2025, the total footfall reached 77,71,269, reflecting its growing popularity among tourists and residents, officials.
+The AMC has already recovered nearly 37% of the project’s cost through tourism revenue, as the SRFDCL continues to manage the bridge’s operations and maintenance, they said.
+From August 31, 2022, to March 2023, the bridge recorded 21.62 lakh visitors and ₹6.44 crore in revenue, officials said. “Between April 2023 and March 2024, 26.89 lakh people visited, contributing ₹8.24 crore. The following year, April 2024 to March 2025, saw 20.67 lakh visitors and ₹8.19 crore in earnings. In the ongoing financial year (April to October 2025), 8.51 lakh visitors generated ₹4.82 crore,” they said.
+“Chief Minister Bhupendra Patel has strengthened the focus on urban tourism while preserving heritage landmarks. Tourist spots such as Gandhi Ashram, Sabarmati Riverfront, Kankaria Lake, Narendra Modi Stadium, the Heritage Walk, and the city’s traditional Pols continue to enhance Ahmedabad’s identity as a blend of heritage and modernity,” officials said.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/gujarat/ahmedabads-atal-bridge-attracts-777-lakh-visitors-generates-27-crore-revenue/article70240470.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:08:25 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/46es2f/article70241670.ece/alternates/LANDSCAPE_1200/VIS_5355.JPG</t>
   </si>
   <si>
     <t>Suvendu Adhikari leads ‘Parivartan Yatra’ rally, demands ‘proper’ execution of SIR in West Bengal</t>
@@ -432,40 +452,23 @@
     <t>https://th-i.thgim.com/public/incoming/1i2jyy/article70241369.ece/alternates/LANDSCAPE_1200/20251104172L.jpg</t>
   </si>
   <si>
-    <t>MLA allegedly ousted from inaugural function</t>
-  </si>
-  <si>
-    <t>Kerala Pradesh Congress Committee president and Peravoor MLA Sunny Joseph was allegedly ousted from a function by Communist Party of India (Marxist) [CPI(M)] workers while he was inaugurating the Chavassery road project in Irrirty municipality on Tuesday.
-Mr. Joseph maintained that since the road work was funded by the government, the local legislator should inaugurate it as per official protocol. However, CPI(M )workers allegedly raised slogans against him, forcing him to leave the venue.
-Addressing supporters at a nearby venue later, the MLA said funds to renovate the road in the Peravoor Assembly constituency were sanctioned following complaints raised during the Navakerala Sadas.
-Meanwhile, CPI(M) workers alleged that the MLA had boycotted the Navakerala Sadas and was now attempting to claim credit for the project. Following the protest, the road was inaugurated by the Irrity municipal chairperson.
-Mr. Joseph said that he attended the function in his capacity as a people’s representative. He added that the road project received administrative sanction on September 19 this year and dismissed the CPI(M)’s claim that the approval came in 2024. The MLA said he had proposed ₹5.75 crore for Kakkayangad-Palapuzha road and ₹1.5 crore for Chavassery road, and that the government approved the projects accordingly.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/kerala/mla-allegedly-ousted-from-inaugural-function/article70239641.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:14:55 +0530</t>
-  </si>
-  <si>
     <t>TOI</t>
   </si>
   <si>
-    <t>‘10% control the Army’: Rahul's caste claim at Bihar rally; BJP terms remark disgraceful</t>
-  </si>
-  <si>
-    <t>Rahul Gandhi (PTI photo)
-'Will Cut Off Your Tongue': Bihar Poll Campaign Turns Ugly, AIMIM Candidate Threatens Tejashwi Yadav
-NEW DELHI: Lok Sabha leader of opposition Rahul Gandhi on Tuesday made a striking claim in Bihar, alleging that country's 10 per cent, referring to upper castes, "hold control over the Army."Addressing a poll rally in Aurangabad's Kutumba, Rahul said, "90 per cent of the people come from extremely backward, backward, Dalit, and Adivasi communities." He went on to assert that these groups - forming the vast majority of India's population - remain largely excluded from power and privilege."All the wealth goes to them, all the jobs go to them. Look at the judiciary - they have control there, and even in the army," Rahul said, in one of his most direct attacks on the country's social and institutional hierarchy.He further added, "90 per cent of India's population is nowhere to be found," suggesting that marginalised communities have been systematically denied access to leadership and opportunity.The BJP hit back at Rahul Gandhi over his remarks on the Army. Party spokesperson Suresh Nakhua, in a post on X, said, "Rahul Gandhi is now searching for caste in the Armed Forces and says 10% of people control it. In his hate for PM Modi, he has already crossed the line into hating India."Another BJP spokesperson, Sanju Verma, also hit out at Rahul Gandhi over his remarks, saying, “Rahul Gandhi is shamelessly devious and deviously shameless.Listening to him in this clip leaves no doubt that this failed, forever-in-waiting PM is desperately trying to polarize. Now he is trying to divide the Army on caste lines — what an unhinged wreck this Leader of Opposition is. Disgraceful.”Directing his attack to Bihar government, Rahul painted a picture of unemployment in the state, blaming the Nitish Kumar government for pushing its youth into low-paying, menial labour across the country."The people of Bihar are doing manual labour across the entire country. In different parts of the country, people from Bihar are building large buildings, roads, tunnels, and factories," he said.Accusing the state government of failing its people, Rahul added, "In other words, the truth is this—that Nitish Kumar has wiped out employment here and turned the people of Bihar into the country’s labourers."</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/10-control-the-army-rahul-gandhis-caste-claim-at-bihar-rally-says-90-indians-nowhere-to-be-found/articleshow/125088800.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 18:48:06 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125088839,width-1070,height-580,imgsize-652610,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+    <t>'Mass chaos': US govt warns shutdown could force airspace closure - what it means</t>
+  </si>
+  <si>
+    <t>A traveler walks through the skyway leading to terminal 3 at O'Hare International Airport in Chicago, Monday, November 3, 2025. (AP)
+US transport secretary Sean Duffy on Tuesday warned that if the government shutdown continues for another week, it will disrupt air travel by worsening staff shortages, causing long queues at airports and forcing the closure of parts of US airspace."So if you bring us to a week from today, Democrats, you will see mass chaos... You will see mass flight delays," he said at a news conference in Philadelphia, as quoted by news agency AFP.“You'll see mass cancellations, and you may see us close certain parts of the airspace, because we just cannot manage it because we don't have the air traffic controllers.”With US Congress still deadlocked over health care funding, the shutdown is on track to become the longest in US history. Public services continue to be affected as Trump’s Republicans and Democrats remain unable to reach an agreement.More than 60,000 air traffic controllers and Transportation Security Administration (TSA) staff are currently working without pay. The White House has warned that rising absenteeism among staff could lead to delays at airport security checkpoints.During the 2019 shutdown, one of the two longest shutdowns at 35 days, similar staff shortages and sick calls from airport workers were a key factor in ending the standoff.In the latest effort to reopen the government, a House-approved resolution failed again in the Senate on Tuesday, marking the 14th rejection.Democrats say reopening the government requires negotiation led by Trump on their demand to extend subsidies that help millions of Americans afford health insurance. Trump has said he will not negotiate with Democrats until the shutdown ends.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/world/us/mass-chaos-us-transport-secretary-warns-shutdown-could-force-airspace-closure-what-it-means/articleshow/125094065.cms</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:13:28 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125094369,width-1070,height-580,imgsize-877846,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>'Chhath, Halloween &amp; jungle raj': Bihar phase 1 campaign blitz ends — a quick recap</t>
@@ -530,21 +533,21 @@
     <t>https://static.toiimg.com/thumb/msid-125092587,width-1070,height-580,imgsize-40268,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>Air traffic congestion: Flight operations impacted in Delhi; IndiGo issues advisory</t>
-  </si>
-  <si>
-    <t>Representational file photo
-DGCA Plans New Rules For Power Banks On Flights After Fire Scare On IndiGo Plane
-NEW DELHI: Flight delays hit several passengers travelling through Delhi on Tuesday, as air traffic congestion led to long wait times across terminals.IndiGo posted an advisory on its official X account, saying: “Due to air traffic congestion in Delhi, flight operations are currently impacted. We understand that extended wait times, both on the ground and onboard, may cause inconvenience, and we sincerely appreciate your patience. ”Also read: Air India sends alternate aircraft to fly home passengers stranded in Mongolia The airline also assured passengers that its on-ground teams were working to make the wait as comfortable as possible. “We value your time and are doing everything we can to help you get on your way soon,” IndiGo said, advising travellers to check its website or mobile app for real-time flight updates.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/air-traffic-congestion-flight-operations-impacted-in-delhi-indigo-issues-advisory/articleshow/125091789.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:13:33 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125091871,width-1070,height-580,imgsize-34734,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+    <t>‘10% control the Army’: Rahul's caste claim at Bihar rally; BJP terms remark disgraceful</t>
+  </si>
+  <si>
+    <t>Rahul Gandhi (PTI photo)
+'Will Cut Off Your Tongue': Bihar Poll Campaign Turns Ugly, AIMIM Candidate Threatens Tejashwi Yadav
+NEW DELHI: Lok Sabha leader of opposition Rahul Gandhi on Tuesday made a striking claim in Bihar, alleging that country's 10 per cent, referring to upper castes, "hold control over the Army."Addressing a poll rally in Aurangabad's Kutumba, Rahul said, "90 per cent of the people come from extremely backward, backward, Dalit, and Adivasi communities." He went on to assert that these groups - forming the vast majority of India's population - remain largely excluded from power and privilege."All the wealth goes to them, all the jobs go to them. Look at the judiciary - they have control there, and even in the army," Rahul said, in one of his most direct attacks on the country's social and institutional hierarchy.He further added, "90 per cent of India's population is nowhere to be found," suggesting that marginalised communities have been systematically denied access to leadership and opportunity.The BJP hit back at Rahul Gandhi over his remarks on the Army. Party spokesperson Suresh Nakhua, in a post on X, said, "Rahul Gandhi is now searching for caste in the Armed Forces and says 10% of people control it. In his hate for PM Modi, he has already crossed the line into hating India."Another BJP spokesperson, Sanju Verma, also hit out at Rahul Gandhi over his remarks, saying, “Rahul Gandhi is shamelessly devious and deviously shameless.Listening to him in this clip leaves no doubt that this failed, forever-in-waiting PM is desperately trying to polarize. Now he is trying to divide the Army on caste lines — what an unhinged wreck this Leader of Opposition is. Disgraceful.”Directing his attack to Bihar government, Rahul painted a picture of unemployment in the state, blaming the Nitish Kumar government for pushing its youth into low-paying, menial labour across the country."The people of Bihar are doing manual labour across the entire country. In different parts of the country, people from Bihar are building large buildings, roads, tunnels, and factories," he said.Accusing the state government of failing its people, Rahul added, "In other words, the truth is this—that Nitish Kumar has wiped out employment here and turned the people of Bihar into the country’s labourers."</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/10-control-the-army-rahul-gandhis-caste-claim-at-bihar-rally-says-90-indians-nowhere-to-be-found/articleshow/125088800.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 18:48:06 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125088839,width-1070,height-580,imgsize-652610,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Jeff Bezos’ ex-wife’s gift: MacKenzie Scott makes large donation; focus on education</t>
@@ -564,6 +567,23 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125086896,width-1070,height-580,imgsize-26596,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Air traffic congestion: Flight operations impacted in Delhi; IndiGo issues advisory</t>
+  </si>
+  <si>
+    <t>Representational file photo
+DGCA Plans New Rules For Power Banks On Flights After Fire Scare On IndiGo Plane
+NEW DELHI: Flight delays hit several passengers travelling through Delhi on Tuesday, as air traffic congestion led to long wait times across terminals.IndiGo posted an advisory on its official X account, saying: “Due to air traffic congestion in Delhi, flight operations are currently impacted. We understand that extended wait times, both on the ground and onboard, may cause inconvenience, and we sincerely appreciate your patience. ”Also read: Air India sends alternate aircraft to fly home passengers stranded in Mongolia The airline also assured passengers that its on-ground teams were working to make the wait as comfortable as possible. “We value your time and are doing everything we can to help you get on your way soon,” IndiGo said, advising travellers to check its website or mobile app for real-time flight updates.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/air-traffic-congestion-flight-operations-impacted-in-delhi-indigo-issues-advisory/articleshow/125091789.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 22:13:33 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091871,width-1070,height-580,imgsize-34734,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Pakistan's Haris Rauf, once hammered by Virat Kohli, banned by ICC after Asia Cup controversy</t>
@@ -602,30 +622,6 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125087453,width-1070,height-580,imgsize-41276,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Asia Cup controversy: ICC drops the hammer! Full list of players punished and warned</t>
-  </si>
-  <si>
-    <t>Suryakumar Yadav and Salman Agha (PTI Photo)
-Go Beyond The Boundary with our YouTube channel. SUBSCRIBE NOW!
-BCCI sends a stern message to Mohsin Naqvi over Asia Cup trophy row
-Players Penalised by ICC ( Asia Cup 2025 ):
-Suryakumar Yadav (India):
-Sahibzada Farhan (Pakistan):
-Haris Rauf (Pakistan):
-Jasprit Bumrah (India):
-Arshdeep Singh (India):
-NEW DELHI: The International Cricket Council (ICC) has confirmed disciplinary actions against multiple players from India and Pakistan following several heated encounters during the ICC Asia Cup 2025. The Code of Conduct hearings, led by members of the ICC Elite Panel of Match Referees, investigated incidents from the India–Pakistan matches played on September 14, 21, and 28.In the September 14 clash, India’s Suryakumar Yadav and Pakistan’s Haris Rauf and Sahibzada Farhan were found guilty of breaching Article 2.21 of the ICC Code of Conduct, which covers conduct that brings the game into disrepute.Suryakumar was fined 30% of his match fee and received two demerit points.Farhan was given an official warning and one demerit point.Rauf was fined 30% of his match fee and also received two demerit points.A week later, on September 21, India pacer Arshdeep Singh was charged under Article 2.6 for allegedly making an offensive gesture, but was found not guilty after a hearing conducted by Match Referee Andy Pycroft.The Asia Cup final on September 28 brought further disciplinary action. Jasprit Bumrah accepted a charge under Article 2.21 for conduct that brings the game into disrepute, accepting an official warning and one demerit point.Since he admitted to the offence, no formal hearing was held.Haris Rauf, meanwhile, was penalised again for the same offence after a hearing before Richie Richardson. He was fined another 30% of his match fee and received two additional demerit points, taking his total to four demerit points within 24 months. That triggered an automatic suspension, ruling him out of Pakistan’s ODIs against South Africa on November 4 and 6, 2025.According to ICC rules, Level 1 breaches carry a maximum fine of 50% of a player’s match fee and up to two demerit points. Accumulating four or more demerit points in two years converts to suspension points, leading to a ban.Fined 30% match fee, 2 demerit pointsOfficial warning, 1 demerit pointTwo separate offences; fined twice, 4 demerit points and 2-match suspensionOfficial warning, 1 demerit pointFound not guilty, no sanction</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/cricket/news/asia-cup-controversy-icc-drops-the-hammer-full-list-of-players-punished-and-warned/articleshow/125091140.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:29:06 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125091164,width-1070,height-580,imgsize-40780,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Big AI freebie: ChatGPT Go now free for 12 months in India; how to claim the offer</t>
@@ -655,6 +651,30 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125076745,width-1070,height-580,imgsize-41718,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Asia Cup controversy: ICC drops the hammer! Full list of players punished and warned</t>
+  </si>
+  <si>
+    <t>Suryakumar Yadav and Salman Agha (PTI Photo)
+Go Beyond The Boundary with our YouTube channel. SUBSCRIBE NOW!
+BCCI sends a stern message to Mohsin Naqvi over Asia Cup trophy row
+Players Penalised by ICC ( Asia Cup 2025 ):
+Suryakumar Yadav (India):
+Sahibzada Farhan (Pakistan):
+Haris Rauf (Pakistan):
+Jasprit Bumrah (India):
+Arshdeep Singh (India):
+NEW DELHI: The International Cricket Council (ICC) has confirmed disciplinary actions against multiple players from India and Pakistan following several heated encounters during the ICC Asia Cup 2025. The Code of Conduct hearings, led by members of the ICC Elite Panel of Match Referees, investigated incidents from the India–Pakistan matches played on September 14, 21, and 28.In the September 14 clash, India’s Suryakumar Yadav and Pakistan’s Haris Rauf and Sahibzada Farhan were found guilty of breaching Article 2.21 of the ICC Code of Conduct, which covers conduct that brings the game into disrepute.Suryakumar was fined 30% of his match fee and received two demerit points.Farhan was given an official warning and one demerit point.Rauf was fined 30% of his match fee and also received two demerit points.A week later, on September 21, India pacer Arshdeep Singh was charged under Article 2.6 for allegedly making an offensive gesture, but was found not guilty after a hearing conducted by Match Referee Andy Pycroft.The Asia Cup final on September 28 brought further disciplinary action. Jasprit Bumrah accepted a charge under Article 2.21 for conduct that brings the game into disrepute, accepting an official warning and one demerit point.Since he admitted to the offence, no formal hearing was held.Haris Rauf, meanwhile, was penalised again for the same offence after a hearing before Richie Richardson. He was fined another 30% of his match fee and received two additional demerit points, taking his total to four demerit points within 24 months. That triggered an automatic suspension, ruling him out of Pakistan’s ODIs against South Africa on November 4 and 6, 2025.According to ICC rules, Level 1 breaches carry a maximum fine of 50% of a player’s match fee and up to two demerit points. Accumulating four or more demerit points in two years converts to suspension points, leading to a ban.Fined 30% match fee, 2 demerit pointsOfficial warning, 1 demerit pointTwo separate offences; fined twice, 4 demerit points and 2-match suspensionOfficial warning, 1 demerit pointFound not guilty, no sanction</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/cricket/news/asia-cup-controversy-icc-drops-the-hammer-full-list-of-players-punished-and-warned/articleshow/125091140.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:29:06 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091164,width-1070,height-580,imgsize-40780,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Delhi gasps again: Cloud seeding, smog towers, odd-even — will any of it really clear the air?</t>
@@ -756,24 +776,6 @@
     <t>https://static.toiimg.com/thumb/msid-125090849,width-1070,height-580,imgsize-810362,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>It’s 'Mango Lassi' Mamdani morning in Big Apple</t>
-  </si>
-  <si>
-    <t>Zohran Mamdani (File photo)
-The TOI correspondent from Washington
-‘JUST IGNORE HIM!’: Zohran Mamdani ‘HUMILIATES’ Trump As He Casts Ballot In NYC Mayoral Election
-: New Yorkers streamed into polling stations on Tuesday morning with the remarkable prospect of the undisputed global capital of finance, skyscrapers, and immense wealth paradoxically electing a socialist mayor.Turbocharged by a brilliant digital campaign, a raft of breathtaking promises, and a winning smile that launched a thousand quips, Zohran Mamdani , the Uganda-born Indian son of film-maker Mira Nair (born in Odisha) and academic Mahmood Mamdani (born in Mumbai), is all set to occupy the City Hall in the ground zero of capitalism, putative Muslim mayor of an iconic city that was attacked by Islamist terrorists on 9/11.Although the gap between Mamdani and his Democrat-turned-independent opponent Andrew Cuomo narrowed by Tuesday, the Indian-African New Yorker is expected to romp home comfortably despite President Trump coming out swinging at the prospect of a mayor who in his view is a communist and a “radical left lunatic.”On the eve of election day, Trump threw his weight behind Cuomo, a scandal-tarnished former Governor of New York, urging voters to even ditch Republican candidate Curtis Sliva (who is polling a distant third), saying “it is my strong conviction that New York City will be a Complete and Total Economic and Social Disaster should Mamdani win. I would much rather see a Democrat win than a Communist with no experience.”Trump also threatened to cut federal funds, “other than the very minimum as required, to my beloved first home,” saying the city has zero chances of success under a “communist,” kneecapping Mamdani even before he takes office.The irony of the most capitalist city on the planet electing a Muslim socialist mayor will go into political folklore but the reasons are not hard to fathom. While NYC is arguably the richest city in the world, with more than 350,000 millionaires, it is also a megalopolis of brutal economic inequality, with crippling housing costs ($3000 per month rent for a studio in Manhattan), failing public transit, and deep-seated poverty in its outer neighborhoods. The wealth that defines the city also creates the extreme, daily cost-of-living pressure for everyone else.Also read: New Trump Era: Laura Loomer gets credentials to cover US Department of Defense - why it's a big deal Mamdani has tapped into this disaffection arising from what he calls the affordability crisis, promising, among other things, higher taxes on the wealthy, rent freeze, free city buses, city-run grocery stores and other sops that have some of its more affluent residents bolting the Big Apple fearing the incoming Mayor will demand a bigger slice of their pie.While non-hispanic whites form the single largest group of eligible voters at 42 percent in the Democratic-leaning city, the Mamdani surge is also powered by Hispanic/Latinos (24 percent), Black/African-American (19 percent), and Asian-American (15 percent). In fact, his campaign was evocative of the city’s diversity, with ads in Spanish and Hindi, including a liberal use of Bollywood song and dance and desi tropes like mango lassi.“When Americans fly in from across our land to JFK &amp; LaGuardia and hear over the loudspeaker, ‘I am Mayor @ZohranKMamdani, welcome to NYC,’ they will look to their children filled with pride and say, ‘In NY any dream is still possible!’” Congressman Ro Khanna, an Indian-American representing SIlicon Valley in California, said, echoing the vision of American liberals.A Mamdani victory, which even Trump appeared to concede is a foregone conclusion, is also expected to weigh in on the ideological future of the Democratic Party, pushing it further left and powering progressives against the moderate and centrist establishment wing of the party.“Our time has come, New York. Our time is now,” Mamdani posted on X Tuesday morning as he headed out to vote with his wife, Rama Duwaji, a Syrian-American.While all eyes are on polling in NYC, there are also mayoral elections in Boston, Atlanta, Seattle, and Minneapolis and gubernatorial elections in New Jersey and Virginia, offering a referendum of sorts on the ten months of Trump rule.In another closely watched election, voters in Virginia, abutting the capital, will be electing their first female governor, choosing between Democrat Abigail Spanberger, a former CIA agent and lawmaker, and Republican Winsome Earle-Sears, the current Jamaica-born Lieutenant governor who served in the US Marines. Across the country, California is also voting on a statewide ballot measure called Proposition 50 designed to create up to five additional Democratic-leaning seats in the House of Representatives to offset the gains Republicans have made nationally through their own map redraws.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/world/us/its-mango-lassi-mamdani-morning-in-big-apple/articleshow/125091203.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:32:57 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125091217,width-1070,height-580,imgsize-390229,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
     <t>Musk vs Altman: OpenAI’s ex chief scientist testifies in court; reveals ‘6-day story’</t>
   </si>
   <si>
@@ -793,6 +795,24 @@
     <t>https://static.toiimg.com/thumb/msid-125089911,width-1070,height-580,imgsize-859288,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
+    <t>It’s 'Mango Lassi' Mamdani morning in Big Apple</t>
+  </si>
+  <si>
+    <t>Zohran Mamdani (File photo)
+The TOI correspondent from Washington
+‘JUST IGNORE HIM!’: Zohran Mamdani ‘HUMILIATES’ Trump As He Casts Ballot In NYC Mayoral Election
+: New Yorkers streamed into polling stations on Tuesday morning with the remarkable prospect of the undisputed global capital of finance, skyscrapers, and immense wealth paradoxically electing a socialist mayor.Turbocharged by a brilliant digital campaign, a raft of breathtaking promises, and a winning smile that launched a thousand quips, Zohran Mamdani , the Uganda-born Indian son of film-maker Mira Nair (born in Odisha) and academic Mahmood Mamdani (born in Mumbai), is all set to occupy the City Hall in the ground zero of capitalism, putative Muslim mayor of an iconic city that was attacked by Islamist terrorists on 9/11.Although the gap between Mamdani and his Democrat-turned-independent opponent Andrew Cuomo narrowed by Tuesday, the Indian-African New Yorker is expected to romp home comfortably despite President Trump coming out swinging at the prospect of a mayor who in his view is a communist and a “radical left lunatic.”On the eve of election day, Trump threw his weight behind Cuomo, a scandal-tarnished former Governor of New York, urging voters to even ditch Republican candidate Curtis Sliva (who is polling a distant third), saying “it is my strong conviction that New York City will be a Complete and Total Economic and Social Disaster should Mamdani win. I would much rather see a Democrat win than a Communist with no experience.”Trump also threatened to cut federal funds, “other than the very minimum as required, to my beloved first home,” saying the city has zero chances of success under a “communist,” kneecapping Mamdani even before he takes office.The irony of the most capitalist city on the planet electing a Muslim socialist mayor will go into political folklore but the reasons are not hard to fathom. While NYC is arguably the richest city in the world, with more than 350,000 millionaires, it is also a megalopolis of brutal economic inequality, with crippling housing costs ($3000 per month rent for a studio in Manhattan), failing public transit, and deep-seated poverty in its outer neighborhoods. The wealth that defines the city also creates the extreme, daily cost-of-living pressure for everyone else.Also read: New Trump Era: Laura Loomer gets credentials to cover US Department of Defense - why it's a big deal Mamdani has tapped into this disaffection arising from what he calls the affordability crisis, promising, among other things, higher taxes on the wealthy, rent freeze, free city buses, city-run grocery stores and other sops that have some of its more affluent residents bolting the Big Apple fearing the incoming Mayor will demand a bigger slice of their pie.While non-hispanic whites form the single largest group of eligible voters at 42 percent in the Democratic-leaning city, the Mamdani surge is also powered by Hispanic/Latinos (24 percent), Black/African-American (19 percent), and Asian-American (15 percent). In fact, his campaign was evocative of the city’s diversity, with ads in Spanish and Hindi, including a liberal use of Bollywood song and dance and desi tropes like mango lassi.“When Americans fly in from across our land to JFK &amp; LaGuardia and hear over the loudspeaker, ‘I am Mayor @ZohranKMamdani, welcome to NYC,’ they will look to their children filled with pride and say, ‘In NY any dream is still possible!’” Congressman Ro Khanna, an Indian-American representing SIlicon Valley in California, said, echoing the vision of American liberals.A Mamdani victory, which even Trump appeared to concede is a foregone conclusion, is also expected to weigh in on the ideological future of the Democratic Party, pushing it further left and powering progressives against the moderate and centrist establishment wing of the party.“Our time has come, New York. Our time is now,” Mamdani posted on X Tuesday morning as he headed out to vote with his wife, Rama Duwaji, a Syrian-American.While all eyes are on polling in NYC, there are also mayoral elections in Boston, Atlanta, Seattle, and Minneapolis and gubernatorial elections in New Jersey and Virginia, offering a referendum of sorts on the ten months of Trump rule.In another closely watched election, voters in Virginia, abutting the capital, will be electing their first female governor, choosing between Democrat Abigail Spanberger, a former CIA agent and lawmaker, and Republican Winsome Earle-Sears, the current Jamaica-born Lieutenant governor who served in the US Marines. Across the country, California is also voting on a statewide ballot measure called Proposition 50 designed to create up to five additional Democratic-leaning seats in the House of Representatives to offset the gains Republicans have made nationally through their own map redraws.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/world/us/its-mango-lassi-mamdani-morning-in-big-apple/articleshow/125091203.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:32:57 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125091217,width-1070,height-580,imgsize-390229,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
     <t>Meghan Markle’s friend reveals why Prince Harry looked upset at Dodgers game</t>
   </si>
   <si>
@@ -827,22 +847,6 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125091969,width-1070,height-580,imgsize-490563,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>More power for Asim Munir? Pakistan plans amendment; revises military command</t>
-  </si>
-  <si>
-    <t>Pakistani army chief general Asim Munir
-The Pakistan government announced plans to introduce the 27th Constitutional Amendment, which includes proposed changes related to the command of the armed forces. The amendment will be tabled in Parliament soon, deputy prime minister and foreign minister Ishaq Dar confirmed on Tuesday.“Of course, the government is bringing it and will bring it … the 27th Amendment will arrive … and is about to arrive. We will try that it be tabled in accordance with principles, laws and the Constitution,” Dar said in the Senate, as quoted by PTI.According to sources, the proposed amendment includes provisions to set up a constitutional court, streamline the process for appointing the chief election commissioner, amend Article 243 dealing with matters of the armed forces, reduce the provinces’ share in federal resources, and transfer control of the education and population welfare ministries from provinces to the federal government.Article 243 of the Constitution states that “the federal government shall have control and command of the armed forces.” The proposal to revise this article is being viewed as a move that could further strengthen the position of Army Chief General Asim Munir and expand the military’s role in national affairs.Dar rejected concerns that the amendment might be passed without proper procedure. “It is not the case that the amendment is tabled and there is voting on it in a haphazard, ad hoc manner; this will not happen,” he said.He said the amendment would first be introduced in the Senate and then referred to a bipartisan committee for discussion, adding that the government would welcome positive suggestions to improve the draft.PPP Senator Raza Rabbani said the changes would damage provincial autonomy and “undo the good work of the 18th amendment,” which devolved powers to the provinces in 2010.The government has the required two-thirds majority in the 336-member National Assembly with the support of 233 members. In the 96-member Senate, it holds 61 seats and will need at least three opposition members to pass the amendment.The secrecy around the proposed changes, particularly the plan to amend Article 243, has drawn attention to whether the new constitutional move will give the armed forces greater influence in the country’s governance.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/world/pakistan/more-power-for-asim-munir-pakistan-plans-constitutional-amendment-includes-revisions-to-military-command-federal-powers/articleshow/125092057.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:33:05 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125092084,width-1070,height-580,imgsize-469567,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Charlise Springer breaks silence after Blue Jays' World Series heartbreak</t>
@@ -1319,7 +1323,7 @@
         <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1327,19 +1331,19 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1347,19 +1351,19 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1367,19 +1371,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1387,19 +1391,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1439,7 +1443,7 @@
         <v>46</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1447,19 +1451,19 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1467,19 +1471,19 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1539,7 +1543,7 @@
         <v>69</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>16</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1547,19 +1551,19 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1619,7 +1623,7 @@
         <v>88</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1627,19 +1631,19 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>93</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1659,407 +1663,407 @@
         <v>97</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>16</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B29" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C31" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C33" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B34" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E34" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B35" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E37" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B38" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C38" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B39" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C39" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E39" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B40" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E40" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C41" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E41" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AM removed hardcoded links
</commit_message>
<xml_diff>
--- a/server/RSS_FullText.xlsx
+++ b/server/RSS_FullText.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="203">
   <si>
     <t>Source</t>
   </si>
@@ -35,6 +35,279 @@
   </si>
   <si>
     <t>TheHindu</t>
+  </si>
+  <si>
+    <t>Bombay HC grants bail to 2011 Mumbai triple blast accused after 13 years</t>
+  </si>
+  <si>
+    <t>The Bombay High Court on Tuesday (November 4, 2025) granted bail to Kafeel Ahmed Mohd Ayub, an accused in the 2011 Mumbai triple bomb blast case, after he spent more than 13 years in prison without trial. The court said the right to a speedy trial under Article 21 of the Constitution cannot be sacrificed to statutory restrictions when the trial shows no sign of early conclusion.
+A Division Bench of Justices A.S. Gadkari and Ranjitsinha Raja Bhonsale set aside a February 2022 order of the special MCOCA court that had rejected Ayub’s bail plea. “According to us, the possibility of concluding the trial of the present case in near future is bleak,” the Bench observed, noting that Ayub, now 65, suffers from age-related ailments.
+The judges stressed that “speedy and expeditious trial is a facet of right to live as embodied under Article 21 of the Constitution of India.” They relied on the Supreme Court’s ruling in Union of India vs K.A. Najeeb (2021), which held that constitutional courts can grant bail when prolonged incarceration violates fundamental rights.
+Quoting the apex court, the Bench noted, “The rigours of such provisions will melt down where there is no likelihood of trial being completed within a reasonable time and the period of incarceration already undergone has exceeded a substantial part of the prescribed sentence.”
+The High Court added, “Had it been a case at the threshold, we would have outrightly turned down the respondent’s prayer. However, keeping in mind the length of the period spent by him in custody and the unlikelihood of the trial being completed anytime soon, the High Court appears to have been left with no other option except to grant bail.”
+2011 Mumbai triple blasts case
+Ayub, a resident of Mohalla Shivdhara in Darbhanga, Bihar, was arrested on February 22, 2012, by the Delhi Police and later taken into custody by the Maharashtra ATS on May 19, 2012. He is accused of giving shelter to co-conspirators, including Yasin Bhatkal, before or after the July 13, 2011, blasts at Opera House, Zaveri Bazaar and Dadar’s Kabutarkhana, which killed 27 people and injured over 100.
+“Prima facie, the role attributed to the Appellant is of giving shelter to co-accused either prior to or after commission of the alleged offence,” the court noted.
+Charges were framed only on March 5, 2021, nearly nine years after his arrest. The prosecution initially cited 700 witnesses, later reducing the number to 400. So far, only 167 have been examined, with 233 still pending.
+“In the last more than 4½ years, the prosecution has examined only 167 witnesses,” the Bench said, adding that the possibility of concluding the trial soon was “bleak”.
+The court has ordered him to furnish a personal bond of ₹1 lakh with local sureties and comply with strict conditions, including monthly reporting to the ATS, surrendering his passport, and not leaving the trial court’s jurisdiction without permission. He must also not tamper with evidence or influence witnesses and attend all trial dates unless exempted.
+The court observed, “It is made clear that the observations made herein are prima facie in nature and for deciding the Application for bail only.” The trial court will decide the case on its merits, the court said.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/cities/mumbai/bombay-hc-grants-bail-to-2011-mumbai-triple-blast-accused-after-13-years/article70240762.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:57:23 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/uexwfd/article70241731.ece/alternates/LANDSCAPE_1200/2011-07-15T103218Z_01_DEL13_RTRMDNP_3_INDIA-BLASTS-MUMBAI.JPG</t>
+  </si>
+  <si>
+    <t>Madras High Court pulls up Chennai cybercrime police for freezing bank account of publicly listed company</t>
+  </si>
+  <si>
+    <t>The Madras High Court has come down heavily on the cybercrime police in Chennai for having frozen publicly listed company V-Mart Retail’s overdraft current account, with a sanctioned limit of ₹75 crore, just because ₹4,194 of crime money was deposited into it by a customer for purchasing goods.
+Justice M. Nirmal Kumar said the cybercrime police should certainly act with alacrity to prevent the criminals from siphoning of the money collected from people but such action should not end up in collapsing the entire business operation of genuine individuals/companies unconnected to cybercrime.
+The judge, however, agreed with advocate Chevanan Mohanan, representing HDFC Bank, that his client could not be blamed since the bank had only complied with the police request to freeze the overdraft current account used by V-Mart to obtain customer payments through UPI and credit/debit card payments.
+Pointing out that indiscriminate freezing of bank accounts on the basis of complaints received through the National Cybercrime Reporting Portal (NCRP) had been a contentious issue for long, the judge recalled that the Greater Chennai Police Commissioner had issued a circular in this regard to all his subordinates in 2021.
+The circular had insisted that the police apply their mind before deciding to freeze bank accounts and not cause any inconvenience to genuine account holders.
+The Commissioner had also instructed that freezing of bank accounts should be restricted only to the extent of the fraudulent proceeds. Non-adherence to such a circular “cannot be taken lightly since it amounts to neglecting the duty and disrespecting the orders of superior officers,” Justice Kumar wrote, and said the police could not end up violating the fundamental right to livelihood and the right to involve in trade/business.
+Though the Chennai cybercrime police claimed V-Mart’s current account was connected to several other complaints with the total disputed fraudulent amount being ₹3.03 lakh, the judge said the petitioner company could not be equated with the operator of mule accounts often associated with cyber frauds.
+Even otherwise, the police could only maintain a lien over ₹3.03 lakh and not freeze the entire bank account, he said, and directed the petitioner company to always maintain a minimum balance of ₹3.03 lakh while continuing to operate the account for all other business purposes.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/tamil-nadu/madras-high-court-pulls-up-chennai-cybercrime-police-for-freezing-bank-account-of-publicly-listed-company/article70240245.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:55:56 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/skkxid/article70241710.ece/alternates/LANDSCAPE_1200/Madras%20High%20Court%20Building_2.jpg</t>
+  </si>
+  <si>
+    <t>Bihar’s electoral battles should be about land, not caste alone</t>
+  </si>
+  <si>
+    <t>Pick up any newspaper, scroll through social media, or attend a rally in Bihar ahead of the elections, and you will see a familiar political playbook in action.
+The Rashtriya Janata Dal (RJD) continues to field candidates from its core base — Yadavs and Muslims. But recognising the limits of this strategy, it now promises government jobs to a population desperate for steady income. Years of poor economic growth have forced millions to migrate out of Bihar in search of work. The RJD hopes to raise a fevered pitch on this subject and win support from an electorate for whom migration has become a major issue.
+The Congress, having lost its erstwhile support bases among ‘forward castes’ to the BJP, has brought its national narrative to Bihar: inclusivity, constitutional values, and secularism. It is pitting these against the Bharatiya Janata Party (BJP)’s divisive communalism. This message resonates in parts of semi-urban Bihar. But it is clear that the party’s heydays are behind it.
+Editorial | Migration debate: On the first phase of 2025 Bihar Assembly election
+The Left parties speak the language of rights and redistribution — land reforms, labour rights, dignity for workers. But except in some pockets, they have not built a mass base. Smaller players such as the Vikassheel Insaan Party have been brought in to peel away support from marginalised communities that have traditionally backed the ruling Janata Dal (United) or JD(U).
+The other side
+On the other side stands the JD(U) and its leader Nitish Kumar. The party is the inheritor of the Karpoori Thakur formula — mobilising Extremely Backward Classes (EBCs) and ‘Mahadalits’ alongside smaller but powerful non-Yadav Other Backward Classes (OBCs) such as Kurmis and Koeris. To expand beyond this base, Mr. Kumar has spent years cultivating women voters through welfare schemes. Now he is betting heavily on the popularity of a one-time cash transfer to women to carry him through this election.
+The BJP seeks to retain the support of ‘forward’ castes — those who view OBC political dominance with resentment. But it is also trying to build a broader coalition through Central government welfare schemes and a strident appeal to Hindutva, aiming to consolidate Hindu voters across caste lines. To keep the middle class and urban voters on board, it emphasises “development”, which in Bihar largely means building roads and bridges across the riverine landscape. In a State with some of India’s worst human development indicators, this limited definition of development speaks volumes.
+Beyond the BJP and JD(U), the National Democratic Alliance (NDA) includes smaller caste-based parties — the Lok Janshakti Party (LJP), Hindustani Awam Morcha, and Rashtriya Lok Morcha (RLM), each representing specific non-Yadav OBC and Dalit constituencies.
+And then there is the newcomer: the Jan Suraaj Party (JSP), which claims to offer something different — less focus on caste patronage, more emphasis on good governance and welfare through better administration.
+In short, Bihar’s 2025 election reflects the three forces that have shaped Indian politics since the 1990s: Mandal (caste-based reservations and identity politics), Mandir (Hindutva consolidation), and Market (developmentalism). Each party emphasises these in different combinations, but Mandal politics remains the most salient factor.
+This contest — with its promises of jobs, welfare, women’s empowerment, and development — obscures a fundamental reality. Except for the Left parties, which lack electoral strength, no major player is talking about Bihar’s core problem, which has two interconnected parts.
+The first is land. Despite decades of fragmentation, land ownership in Bihar remains skewed towards forward caste elites. This concentration of agricultural land is not just an economic issue; it is the foundation of social and political power that has persisted for generations. The second is the missing industry. Bihar has one natural strength: fertile agricultural land. This should have spawned a thriving agro-processing industry — food processing units, packaging facilities, supply chain infrastructure that creates jobs and adds value to farm produce. Instead, Bihar exports its raw agricultural output and its people. The concentration of land in the hands of an elite that has historically favoured rent-seeking over capital investment has stifled the emergence of a dynamic agro-industrial sector.
+These two issues — land concentration and the absence of agro-processing — are keys to understanding why Bihar remains poor despite decades of “social justice” politics and years of “development” governance. They are also the issues that every major party is carefully avoiding because addressing them would mean challenging entrenched interests: big landowners (including wealthy farmers from OBC communities), forward caste economic dominance, and the entire political economy that keeps the current system running.
+Bihar’s backward caste leaders — Lalu Prasad Yadav, Nitish Kumar, and others — rose to power in the late 1980s and early 1990s. Most people credit this to the socialist movements of the mid-20th century. But the roots go back further, to the Triveni Sangh movement of the 1920s-30s. Back then, backward caste leaders challenged the dominance of forward castes (Rajput, Bhumihar, Brahmin, Kayastha) who controlled land, wealth, and power. They wanted literacy, education, and a fairer distribution of resources.
+Nearly a century later, Bihar’s core problem remains the same: a tiny minority still controls most of the wealth. The Bihar caste survey reveals a stark reality. Forward castes make up just 15.5% of the population, yet they hold 31% of all government jobs. While 10% of forward caste households earn over ₹50,000 per month, this figure drops to only 4% among OBCs, 2% among EBCs and Scheduled Castes, and less than 1% among Scheduled Tribes. Over 80% of large landholdings (those exceeding 20 acres) belong to forward castes according to India Human Development Survey (2011) and the National Sample Survey Organisation (2019). This concentration of resources has not just persisted; it has reproduced itself through networks, influence, and access to power.
+Political power without economic change
+Bihar has achieved political democracy. Backward castes have held power for decades. But this has not translated into economic democracy. The wealth is still in the same hands.
+To understand why Bihar’ s political leaders — even those from backward castes who fought for social justice — have avoided these fundamental issues, we need to look at what battles they chose to fight. Mr. Prasad championed social justice aggressively. But he focused on challenging forward castes while ignoring, or even suppressing, other backward and extremely backward castes. He did not address land redistribution or economic inequality. He only fought “neighbourhood battles” — challenging the castes directly above Yadavs in the hierarchy rather than the entire system of inequality. This approach sharpened tensions between Yadavs and other OBC/EBC groups.
+Mr. Kumar took a different path. He built roads, schools, and provided electricity — infrastructure that benefits everyone. This looked like progress without threatening anyone’s wealth. He even formed a Land Reforms Commission early on, but quickly abandoned anything that would challenge big landowners. The result? Infrastructure improved, but wealth distribution didn’t change.
+Neither Mr. Prasad nor Mr. Kumar was willing to challenge big landowners within their own castes (Yadavs and Kurmis), even though these are relatively few in number. Mr. Kumar, who has been in power for two decades, would have been voted out by now if the state of the Bihar economy was an indication of governance. But the opposition Mahagatbandhan (MGB) has not presented itself as a clear alternative, despite successful rallies and mobilisations.
+Bihar now faces two possible paths. The first is development for the few — a continuation of the current model of growth that benefits big business and landowners, with some welfare schemes to pacifiy the masses. The second is inclusive growth — addressing the wealth gap, redistributing land, ensuring jobs and income reach all castes, and building agro-processing industries that create broad-based employment.
+The newer political entrants exemplify the first path. The LJP’s Chirag Paswan promises food processing industries, while the JSP’s Prashant Kishor emphasises service sector growth and better governance. Both talk of development, but neither addresses wealth redistribution or land reform. Their models accept the concentration of resources in the hands of big landowners, businesses, and bureaucrats, promising only to make the system work more efficiently.
+Both the NDA and MGB are multi-caste alliances, which prevents either from moving decisively in any direction. The MGB’s recent policy papers — ‘Parivartan Patra’, ‘Mai-Bahin Maan scheme’, and ‘Ati-Pichada Nyay Patra’ — do show some understanding of inclusive development, with plans to empower women, EBCs, and Dalits. But given past broken promises, voters remain sceptical.
+The Left parties have economic plans to redistribute wealth, but they have failed to connect these to social justice issues. Their politics is yet to reckon with facts such as a forward caste landless labourer faces very different barriers from a Dalit or EBC woman even if both are poor. Many Dalits who have been officially allotted land titles are unable to take physical possession due to social barriers.
+To be seen as a credible alternative to the NDA, the MGB needed to send a clear, credible message that they are serious about inclusive growth, not just winning elections. They should have taken a message of redistribution and opportunity to voters, rather than making wishful welfare promises. They should have drawn a sharper ideological contrast with the NDA. Now their hopes are pinned on anti-incumbency alone.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/opinion/op-ed/bihars-electoral-battles-should-be-about-land-not-caste-alone/article70240382.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:54:03 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/fafdue/article70179814.ece/alternates/LANDSCAPE_1200/Patna%20migrants.jpg</t>
+  </si>
+  <si>
+    <t>NGO begins campaign in Karnataka to display Constitution’s Preamble in private institutions</t>
+  </si>
+  <si>
+    <t>To spread awareness about the Constitution, the Netaji Subhash Chandra Bose Organisation, a non-government organisation, has launched a Statewide campaign to display the Preamble of the Constitution in the offices of cooperative societies, milk federations, private banks, and educational institutions across the State.
+Addressing presspersons in Kalaburagi city on Tuesday, organisation director Sommanna Sangoli said the initiative aims to instil constitutional responsibility among citizens and employees working in both government and private sectors.
+So far, the organisation has distributed around 14,000 framed copies of the Preamble to different institutions across Karnataka. Mr. Sangoli said that the organisation is charging around ₹2,000 per frame to cover the production and the distribution expenses.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/ngo-begins-campaign-in-karnataka-to-display-constitutions-preamble-in-private-institutions/article70240506.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:51:01 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/1urv94/article70241120.ece/alternates/LANDSCAPE_1200/10258_4_11_2025_19_43_42_3_KLB_SOMMANNA_SANGOLI_PREAMBLE_AWARENESS_CAMPAIGN_2.JPG</t>
+  </si>
+  <si>
+    <t>GI stamp sought for Sirumugai Menpattu Pudavaigal</t>
+  </si>
+  <si>
+    <t>Tamil Nadu, a land celebrated for its diverse handwoven sarees, has yet another gem stepping into the spotlight — the Sirumugai Menpattu Pudavaigal. This particular saree from the Coimbatore region is now seeking the prestigious Geographical Indication (GI) tag — a recognition that will preserve its heritage, protect its weavers, and celebrate its timeless legacy in the world of handloom artistry.
+The Sirumugai Anaithu Kaithari Pattu Selai Urpathi Mattrum Virpanaiyalargal Sangam and the Patent Information Centre of Tamil Nadu State Council for Science and Technology (TNSCST), Chennai have jointly filed the application. Bharathiar University, Coimbatore did an elaborate research for this filing.
+These sarees are woven from the finest Indian mulberry silk. Only cocoons reared on mulberry leaves are used. And every Sirumugai Menpattu saree comes with a Silk Mark certificate, issued by the Silk Mark Organisation of India, as proof of authenticity.
+“Traditional silk sarees are very heavy but Sirumugai sarees are lightweight and easy to wear. They are handwoven using traditional looms,” M. Nagarajan, President of Sirumugai Anaithu Kaithari Pattu Selai Urpathi Mattrum Virpanaiyalargal Sangam, told The Hindu.
+Each saree typically weighs between 500 and 600 grams. On average, it takes about two to three days to weave one. Prices start at around ₹6,000 and can go up to several lakh, depending on the design and craftsmanship.
+“Currently, these sarees are sold throughout India. On the export front, the sarees from here are sent to the US, Canada, Germany, Singapore, Malaysia and other countries,” Mr. Nagarajan said. “Getting a GI tag for this product will enhance the livelihood of the weavers. It will also motivate the next generation to take this business forward,” he added.
+According to details shared by S.Vincent, Member Secretary of Tamil Nadu State Council for Science and Technology, there are over 15,000 skilled weavers, 600 dyeing experts and 500 designers in this zone. The production units are situated in and around Mettupalayam and Annur taluk.
+The TNSCST has established IPR cells in 40 higher education institutions of Tamil Nadu, including one at Bharathiar University, to identify products pertaining to the region which have the potential to get GI tags.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/tamil-nadu/gi-stamp-sought-for-sirumugai-menpattu-pudavaigal/article70240631.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:50:09 +0530</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/theme/images/og-image.png</t>
+  </si>
+  <si>
+    <t>House-to-house enumeration begins in Tamil Nadu</t>
+  </si>
+  <si>
+    <t>The house to house enumeration, as part of the Special Intensive Revision of the electoral rolls, began across Tamil Nadu on Tuesday. Booth-level officers (BLOs) visited households to distribute partially pre-filled enumeration forms.
+Deputy Election Commissioner Bhanu Prakash Yeturu and Director Krishna Kumar Tiwari from the Election Commission of India visited Tamil Nadu on Tuesday to review the progress. Mr. Yeturu is scheduled to undertake field visits to districts.
+According to a senior official, about 68,700 booth-level officers were engaged in the enumeration. Tamil Nadu Chief Electoral Officer (CEO) Archana Patnaik had earlier said if the BLO finds any house locked or closed, she/he shall make at least three visits.
+Electors may also download their enumeration forms and submit the filled-in forms online. The BLOs will collect the filled up forms and provide an acknowledgement in one copy of the enumeration form which will be retained by the elector, it said. Online submissions will also be verified by the BLOs during their house visits.
+The CEO also said electors can fill up the details of their names or the names of the parents or grandfather or grandmother in the electoral rolls of the previous SIR. The BLOs will assist the electors in filling up these details.
+The names of all the electors who have submitted their duly filled enumeration forms to the BLOs during the house to house enumeration will be included in the draft electoral roll, which will be published on December 9.
+For electors, who have not furnished complete details, the officials will initiate enquiry and the electors can submit necessary documents during the hearing. The final electoral rolls will be published on February 7, 2026.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/tamil-nadu/house-to-house-enumeration-begins-in-tamil-nadu/article70240771.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:45:04 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/zfs8hc/article70241387.ece/alternates/LANDSCAPE_1200/4871_4_11_2025_16_55_21_1__DSC7457.JPG</t>
+  </si>
+  <si>
+    <t>Coimbatore gang-rape: survivor scaled compound wall of house for refuge</t>
+  </si>
+  <si>
+    <t>A few families living at Brindhavan Nagar near Coimbatore International Airport had come to the aid of the 20-year-old college girl, who sought refuge in one of the houses while fleeing from the three men who allegedly gang-raped her on the intervening night of November 2 and 3 on a deserted area nearby.
+According to witnesses, who did not want to be identified, the girl scaled the compound wall of a house around 4 a.m. on November 3 and knocked on the front door. However, the residents were asleep and did not hear the knocks. As the calling bell did not work, she pressed the switch of a motor in a desperate move to seek support.
+Seeing no response, the girl climbed the open stair to reach the terrace, from where she stepped into the verandah of the very adjacent house on the first floor.
+The residents of the first floor were astounded to see a girl in distress in front of their door at an unexpected hour, seeking help. Soon, the residents of the house alerted a few neighbours, including the family residing on the ground floor to deal with the unforeseen situation.
+Meanwhile, the girl came to the ground floor of the house, where she switched on a light on the porch and knocked on the door for help. Soon the neighbours, from eight families altogether, rushed to the house on the ground floor.
+“The girl was in a panic state beyond words. She said she was fleeing from three persons, who assaulted her boyfriend on a vacant land nearby. The first words that came from me were ‘You are safe here. Nobody will harm you’. She wanted to speak to her mother over the phone and I gave her my phone,” said a man at the spot.
+Sensing that the girl was in need of a replacement for the dress she was wearing, a woman from the neighbourhood immediately arranged one. The survivor was given water and moral support.
+Hearing the ordeal of the girl, two men from the neighbourhood rushed to the vacant land off Brindhavan Nagar where her boyfriend was assaulted by the three men. They found police personnel at the place and alerted them about the girl, for whom nearly 100 policemen were combing the vacant land and adjacent deserted areas from 11.45 p.m.
+The police team rushed to the house and shifted her to a nearby private hospital.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/tamil-nadu/coimbatore-gang-rape-how-a-neighbourhood-sheltered-backed-survivor/article70241095.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:42:09 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/tn665p/article70241029.ece/alternates/LANDSCAPE_1200/Brindhavan%20Nagar%20near%202.jpg</t>
+  </si>
+  <si>
+    <t>KTR accuses Revanth govt. of denying poor students access to education</t>
+  </si>
+  <si>
+    <t>Bharat Rashtra Samithi (BRS) working president K.T. Rama Rao has accused Chief Minister A. Revanth Reddy of deliberately withholding fee reimbursement dues amounting to over ₹10,000 crore, thereby depriving lakhs of poor and middle-class students of access to higher education.
+Addressing a roadshow in Somajiguda as part of the Jubilee Hills bypoll on Tuesday, Mr. Rao alleged that the Congress government is conspiring to weaken Telangana’s educated youth and undermine the aspirations of thousands of families dependent on the scheme.
+He said the Revanth Reddy government, instead of clearing the pending dues, had been intimidating private colleges and educational institutions already struggling to survive.
+He further alleged that the Congress government had stopped several welfare schemes introduced by the previous BRS regime, including Rythu Bandhu, Rythu Bima, KCR Kits, Bathukamma saree distribution, Ramzan and Christmas gifts, and had even discontinued the free water supply scheme in Hyderabad.
+Mr. Rao appealed to voters in Jubilee Hills to use the bypoll to teach the Congress a lesson on behalf of the four crore people of Telangana who were ‘betrayed’.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/telangana/ktr-accuses-revanth-govt-of-denying-poor-students-access-to-education/article70241350.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:41:34 +0530</t>
+  </si>
+  <si>
+    <t>Action sought after photo of inspector celebrating birthday with history-sheeters in Yadgir goes viral</t>
+  </si>
+  <si>
+    <t>A photograph of the circle police inspector in Yadgir district allegedly celebrating his birthday with history-sheeters has gone viral on social media drawing strong reaction from members of Dalit organisations who have sought action against him.
+The officer seen in the photograph has been identified as Shorapur police inspector M. Umesh. In the photograph, he is allegedly vseen celebrating his birthday with history-sheeters near Gandhi Chowk in Shorapur.
+The Karnataka State Dalit Sangharsh Samiti (Krantikari wing) submitted a memorandum addressed to the Inspector-General of Police, North Eastern Range, Kalaburagi, through the Yadgir Superintendent of Police on November 3, alleging that the officer celebrated his birthday with history-sheeters.
+In the memorandum, the samiti has also alleged that the law and order situation in the city had collapsed after Mr. Umesh took charge. Because of his inept handling, the rift between the Dalit and the Valmiki communities over a garden near Ambedkar Circle had escalated, the samiti has also alleged.
+This was the second such incident in the district within a month. Earlier, sub inspector attached to the Narayanapur station Raj Shekhar was found celebrating his birthday on the station premises with a history-sheeter.
+Superintendent of Police Pruthvik Shankar had placed him under suspension in the second week of October, after former Minister Narasimha Naik (Rajugowda) submitted a memorandum, demanding action.
+Referring to the earlier action, Mallikarjun Kranti, State organiser of KSDSS, who had submitted a memorandum, demanded similar action against Mr. Umesh too. In the memorandum, he has warned of an agitation before the SP’s office in Yadgir on November 26, if no action was taken immediately.
+Mr. Shankar told The Hindu that he had sought a detailed report on the incident and further action will be initiated based on it. Meanwhile, sources revealed that the DSP Shorapur has submitted his report to Mr. Shankar.
+When contacted, Mr. Umesh said that while he was proceeding to the police station via Gandhi Chowk, members of a private organisation, who had already made preparations for his birthday celebrations, forced him to take part in the celebrations. “I didn’t notice the history-sheeters among the gathering. My birthday was celebrated in September. I don’t know the intention behind making it an issue after a month,” he said.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/action-sought-after-photo-of-inspector-celebrating-birthday-with-history-sheeters-in-yadgir-goes-viral/article70240692.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:38:43 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/ue7w9r/article70241064.ece/alternates/LANDSCAPE_1200/YDRKN_4_11_2025_20_28_2_1_IMG_20251104_WA0126.JPG</t>
+  </si>
+  <si>
+    <t>Drugs worth ₹1 crore destroyed in Hyderabad</t>
+  </si>
+  <si>
+    <t>The Excise Department on Tuesday destroyed narcotic substances valued at around ₹1 crore that were seized in 104 cases across various excise stations in the city.
+The confiscated drugs, collected under the jurisdictions of Ameerpet, Dhoolpet, Kachiguda, Musheerabad and Nampally excise stations, were incinerated at GJ Multicove Private Limited in Shadnagar. The destruction was carried out under the supervision of AES Srinivasa Rao.
+Among the substances destroyed were 295 kilograms of marijuana, 7.65 grams of MDMA, 1.25 kilograms of straw poppy, small quantities of cocaine and hashish oil, penile injections, and 35 millilitres of hydrochloride. Officials said the total value of the destroyed drugs is estimated to be nearly ₹1 crore.
+In a separate operation, the State Task Force (STF) - B team, led by Sub-Inspector Balaraju, conducted raids in Shaikpet in view of the Jubilee Hills by-elections.
+During the raids, the team seized 66 quarter bottles of liquor from three individuals who were allegedly selling alcohol illegally. The accused and the seized liquor were handed over to the Golconda police station for further action.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/cities/Hyderabad/drugs-worth-1-crore-destroyed-in-hyderabad/article70241204.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:37:53 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/g1i97f/article70241211.ece/alternates/LANDSCAPE_1200/WhatsApp%20Image%202025-11-04%20at%2018.07.12_36db395f.jpg</t>
+  </si>
+  <si>
+    <t>Ensuring clean environment to the next generation is everyone’s responsibility, says KSPCB chairman</t>
+  </si>
+  <si>
+    <t>MLA and chairman of Karnataka State Pollution Control Board (KSPCB) P.M. Narendraswamy has said that passing on a clean environment to the next generation is the responsibility of everyone and there should be collective contribution towards reducing pollution and people should use eco-friendly vehicles.
+He was speaking after inaugurating the golden jubilee celebrations of the KSPCB organised at Nehru Stadium in Hubballi on Tuesday. Regional offices of KSPCB in Dharwad, Gadag, and Uttara Kannada districts had jointly organised the event.
+Mr. Narendraswamy said that in Gadag, Dharwad, and Uttara Kannada, over 3.5 lakh milk packets were getting into the soil everyday. “Steps have to be taken to prevent it by creating awareness. A country should have forests in 33% of the total land but we have it in less than 20%. The National Green Tribunal too has emphasised on environment conservation. The challenge is excessive use of chemical pesticides and huge solid waste generated in urban areas and it has to be addressed through collective efforts,” he said.
+He said that to create awareness, quizzes and debates were being held in schools and colleges, and prizes were being given for those making reels on environment conservation. The KSPCB would set up six air quality monitoring centres in Dharwad district, he said.
+Mr. Narendraswamy emphasised the need for the public to be involved more in initiatives of environment conservation and said that the impact would be more through concerted efforts. He also listed various initiatives taken at the global level through conventions and emphasised that the board was working towards achieving global goals and mandates.
+Presiding over the function, MLA Mahesh Tenginakai called on people to join hands in various initiatives to make towns and cities free of garbage and plastic. He said that extensive training was required to make industries reduce the amount of waste generated. People should also contribute towards saving waterbodies, he said.
+MLA and chairman of Karnataka Slum Development Board Prasad Abbayya elaborated on various measures taken by the government in addressing the issue. The KSPCB had taken a good initiative of sensitising the children, the future citizens of the country towards environment conservation, he said.
+A host of political leaders including MLA Arabail Shivaram, former MP I.G. Sanadi, Hubballi Dharwad Mayor Jyoti Patil, Chairman of HDUDA Shakir Sanadi and various officials were present. On occasion those who were involved in environmental conservation initiatives were honoured.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/ensuring-clean-environment-to-the-next-generation-is-everyones-responsibility-says-kspcb-chairman/article70240961.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:36:17 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/xyqh8v/article70241223.ece/alternates/LANDSCAPE_1200/2699_4_11_2025_20_31_53_1_05HUBLIKSPCBGOLDEN.JPG</t>
+  </si>
+  <si>
+    <t>Adoptions of girls outnumber those of boys in Kalaburagi district</t>
+  </si>
+  <si>
+    <t>In a remarkable shift in adoption trends, more girls have been adopted than boys in Kalaburagi district over the last six years, according to the Department of Women and Child Development.
+District Child Protection Officer (DCPO) Manjula Patil, addressing a press conference in Kalaburagi on Tuesday, said that 110 children were admitted under the department’s care between 2020-2025, of which 54 were adopted. Among them, 34 were girls and 20 boys.
+“It is heartening to note that the mindset of the people is gradually changing, and many couples are now coming forward to adopt girls,” Ms. Patil said.
+Among the 54 adoptions, nine were by foreign couples, reflecting growing international interest in adoption through legal Indian procedures. The remaining adoptions were by parents from Karnataka and other parts of the country, she said.
+Ms. Patil said that the adoption procedures are monitored through the department authorities to prevent illegal or unregistered adoptions, she added.
+The Women and Child Development Department has also launched a month-long campaign across Kalaburagi district to educate the public about the legal adoption process.
+As part of the initiative, awareness programmes are being held in religious places, educational institutions, and public spaces. Officials are conducting interactive sessions to educate people about applying for adoption legally.
+Ms. Patil emphasised that adopting through proper procedures not only protects the child but also safeguards adoptive parents from future legal complications.</t>
+  </si>
+  <si>
+    <t>https://www.thehindu.com/news/national/karnataka/adoptions-of-girls-outnumber-those-of-boys-in-kalaburagi-district/article70240489.ece</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:33:57 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/le5waj/article70241393.ece/alternates/LANDSCAPE_1200/10258_4_11_2025_19_43_42_1_KLB_DISTRICT_CHILD_PROTECTION_OFFICER_MANJULA_PATIL_1.JPG</t>
   </si>
   <si>
     <t>Ahmedabad’s Atal Bridge attracts 77.7 lakh visitors, generates ₹27 crore revenue</t>
@@ -97,9 +370,6 @@
     <t>Tue, 04 Nov 2025 23:35:46 +0530</t>
   </si>
   <si>
-    <t>https://www.thehindu.com/theme/images/og-image.png</t>
-  </si>
-  <si>
     <t>Asphalt Hebbal flyover immediately: GBA chief</t>
   </si>
   <si>
@@ -114,6 +384,9 @@
   </si>
   <si>
     <t>Tue, 04 Nov 2025 23:25:27 +0530</t>
+  </si>
+  <si>
+    <t>https://th-i.thgim.com/public/incoming/pxmjxa/article70241760.ece/alternates/LANDSCAPE_1200/IMG_Hebbal_flyover_traff_2_1_DRC51N7Q.jpg</t>
   </si>
   <si>
     <t>Kerala University PhD scholar alleges caste bias, abuse of power by Sanskrit department head</t>
@@ -194,264 +467,6 @@
     <t>https://th-i.thgim.com/public/incoming/rfmkku/article70239239.ece/alternates/LANDSCAPE_1200/PTI11_04_2025_000017B.jpg</t>
   </si>
   <si>
-    <t>BRS cannot seek sympathy after ignoring grieving families in the past, says Revanth</t>
-  </si>
-  <si>
-    <t>Chief Minister A. Revanth Reddy on Tuesday said the Bharat Rashtra Samiti (BRS) has no moral right to seek votes on sympathy grounds for its Jubilee Hills bypoll candidate Maganti Sunitha, asserting that a party which once disregarded grieving families like that of P. Janardhan Reddy (PJR) “can not now appeal to voters on sentiment.”
-Mr. Reddy also said the BJP’s repeated allegation that the Kaleshwaram project had become an “ATM” for the KCR family is hollow unless it pursued the matter through proper investigation, and challenged that if the case were handed to the CBI, KCR and his son would be arrested within 48 hours.
-Mr. Reddy demanded that the CBI register an FIR in the Kaleshwaram case by November 11 and called for the arrest of K. Chandrashekar Rao, Harish Rao and K.T. Rama Rao, while asking why Mr. Rama Rao is not being allowed to be arrested in the Formula E race case
-Addressing a corner meeting in Rahmath Nagar, he said the BRS leadership is asking for support following the death of sitting MLA Maganti Gopinath, but had earlier violated long-standing political practices meant to leave the seat to members of bereaved families.
-The Chief Minister recalled that after the sudden demise of former Minister P. Janardhan Reddy (PJR) in 2007, both the TDP and BJP stepped back from contesting to ensure the family was not put under pressure. “It was the TRS, now BRS, that broke the tradition by fielding a candidate against the PJR family,” he said. He added that PJR’s family members were made to wait outside for hours when they sought an appointment with K. Chandrashekar Rao, describing it as evidence of “disrespect and insensitivity.”
-“Those who ignored a grieving family then are now asking for votes in the name of sentiment. What was wrong for them then cannot become right for us now,” he said. He added that the party, which offered no ministerial space to women during its time in power, is now speaking of women’s sentiment for electoral gain.
-Pradesh Congress Committee president Mahesh Kumar Goud, Ministers Komatireddy Venkat Reddy and Mohammed Azharuddin, MP Anil Kumar Yadav, MLAs, MLCs and Congress candidate Naveen Yadav were present.
-Mr. Revanth Reddy reiterated that the Congress government had delivered key welfare measures in Jubilee Hills, including 14,197 ration cards, 200 units of free power to 25,925 families, and the distribution of 23,311 quintals of rice every month. Girl children were availing free travel in RTC buses, he said, contrasting this with what he described as “ten years of neglect” under the previous government.
-He accused the BRS and BJP of coordinating their political strategy in the bypoll and challenged Union Minister G. Kishan Reddy to ensure that the CBI registers an FIR in the Kaleshwaram project case by November 11 if the BJP believes its own allegations against the former Chief Minister’s family. He questioned the delay in acting on the Governor’s request to arrest K.T. Rama Rao in the Formula E race case, alleging that both parties are shielding each other.
-He urged voters to support Congress candidate Naveen Yadav, saying the government would sanction 4,000 houses for the poor in the constituency after the byelection.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/telangana/brs-cannot-seek-sympathy-after-ignoring-grieving-families-in-the-past-says-revanth/article70241246.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:58:01 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/lqnft/article70241323.ece/alternates/LANDSCAPE_1200/_DSC9626.JPG</t>
-  </si>
-  <si>
-    <t>Bengaluru: Disgruntlement in BJP over 11-member committee to oversee GBA polls</t>
-  </si>
-  <si>
-    <t>Many senior city BJP MLAs and party leaders are reportedly upset over not being included in the 11-member party committee to oversee Greater Bengaluru Authority (GBA) polls.
-Four-time MLA for Yelahanka and former chairman of Bangalore Development Authority (BDA) S.R. Vishwanath openly expressed his disappointment over not being included in the committee. “BJP State president B.Y. Vijayendra seems to have no time for Bengaluru. I have time and again told him that the road to capture power in the State runs through Bengaluru. But he seems to have no hold in the city,” he said.
-“I have been an MLA four times, and I have earlier been deputed by the party for elections even in Hyderabad. But I have been asked to only focus on my constituency, Yelahanka. Senior MLA Satish Reddy, Union Minister V. Somanna, who has a hold in two assembly constituencies, have also not been made members of the party committee. This is a local election where the party needs to be strengthened at the grassroots level. I hope the responsibility for the election results is also taken by this committee and not pushed on to us,” he told media persons on Tuesday.
-The committee includes Leaders of Opposition in both Houses, R. Ashok and Chalavadi Narayanaswamy, five MPs of Bengaluru and the neighbouring Chikkaballapur, to which the Yelahanka constituency comes under, former chief minister and former Bengaluru MP D.V. Sadananda Gowda and senior MLA S. Suresh Kumar among others.
-Another senior BJP leader, who did not wish to be named, said that not one of the former mayors, floor leaders from the erstwhile Bruhat Bengaluru Mahanagara Palike (BBMP) was included, and this did not augur well for the party. “Barring one MP, none of the MPs have a strong organisational hold in the city. Keeping out senior MLAs and former mayors and floor leaders who will actually fight the elections on the ground only shows that a small, insecure clique wants to control the party apparatus and keep others out,” he said.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/bengaluru-disgruntlement-in-bjp-over-11-member-committee-to-oversee-gba-polls/article70240842.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:53:40 +0530</t>
-  </si>
-  <si>
-    <t>Centre releases pending Samagra Shiksha funds to Kerala</t>
-  </si>
-  <si>
-    <t>The Union government has released pending Samagra Shiksha funds to the tune of ₹92.41 crore to Kerala.
-Another ₹17 crore from the sanctioned amount of ₹109 crore is expected to be released in a few days.
-The funds for the Centrally sponsored Samagra Shiksha scheme that will reach the government account will be transferred to the Samagra Shiksha Kerala (SSK) account after the SSK sends a request to this effect.
-The total approved amount for the Samagra Shiksha scheme for 2025-26 is ₹761 crore of which ₹456 crore is the Central share.
-Kerala had signed up for the PM SHRI scheme recently after the Union government had withheld Samagra Shiksha funds to the tune of ₹1,158.13 crore.
-However, the scheme was put on hold following dissension within the ruling Left Democratic Front (LDF). Coalition partner the CPI was especially upset that the agreement was signed without any discussion in the Cabinet or within the front.
-It remained adamant about a review or withdrawal of the MoU signed with the Union government. Finally, the Cabinet agreed to freeze the scheme and announced a subcommittee to study the CPI’s concerns on the scheme. It was also decided to formally inform the Union government of the State’s decision.
-However, almost a week later Kerala is yet to send a letter in this regard. Minister for General Education V. Sivankutty on Tuesday said procedures were under way and the communication would be sent soon.
-The Union government had informed the Supreme Court recently that Samagra Shiksha funds due to Kerala will be released soon. The court was considering a case related to appointment of special educators in the State.
-Samagra Shiksha hopes to send another proposal soon for the second instalment. However, uncertainty surrounds further release of funds, particularly once the State sends the communication on PM SHRI.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/kerala/centre-releases-pending-samagra-shiksha-funds-to-kerala/article70241547.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:52:34 +0530</t>
-  </si>
-  <si>
-    <t>BJP announces week-long campaign against garbage and pothole issues in Bengaluru</t>
-  </si>
-  <si>
-    <t>The Opposition Bharatiya Janata Party (BJP) has announced a week-long campaign against Bengaluru’s “garbage disposal problem and pothole issues”.
-BJP held a meeting of all Bengaluru MLAs and MPs on Tuesday, following which the party announced a signature campaign against the ruling Congress government.
-“Due to the misgovernance of the Congress government, Bengaluru has turned into a garbage city. Potholes and piles of garbage are visible on all roads. We need to fight against the government that has betrayed the city, and it has been decided to conduct inspections for one week. Along with this, a signature collection campaign will be held in every assembly constituency from November 6 to 15,” Leader of Opposition in the Assembly, R. Ashok announced after the meeting.
-“We will also collect people’s opinion on the B Khata to A Khata conversion scheme, which we think is a scheme to extract money. The government has no funds for Bengaluru’s development. There is no need to take such steps to arrange that money. People cannot afford to pay so much. People do not want such an expensive brand Bengaluru. We need a Bengaluru that thinks about common people,” he said.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/bjp-announces-week-long-campaign-against-garbage-and-pothole-issues-in-bengaluru/article70240783.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:49:54 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/iom0dd/article70241558.ece/alternates/LANDSCAPE_1200/_JAI1974.JPG</t>
-  </si>
-  <si>
-    <t>Minister promotes Andhra Pradesh tourism at World Travel Market 2025 in London</t>
-  </si>
-  <si>
-    <t>Andhra Pradesh Tourism Minister Kandula Durgesh on Tuesday said the State would soon find a prominent place on the global tourism map, given its rich tourism potential. Participating in the World Travel Market (WTM) 2025 being held in London from November 4 to 6, the Minister said Andhra Pradesh was striving to emerge as a global tourism leader through a series of investor-friendly initiatives. He said the State aims to promote its diverse attractions — including natural landscapes, heritage sites such as Gandikota, and spiritual destinations — while focusing on sustainable development and enhanced visitor experiences.
-Mr. Durgesh, along with Special Secretary (Tourism) Ajay Jain, inaugurated both the Indian Ministry of Tourism and Andhra Pradesh Tourism stalls at the event. The State’s stall featured a Kuchipudi dance performance, highlighting Andhra Pradesh’s vibrant culture, and showcased its scenic beauty, historical forts, coastline, and cultural heritage.
-The Minister held discussions with more than 20 international tour operators, hotel groups, and investors from the MICE (Meetings, Incentives, Conferences and Exhibitions) sector, as well as travel media and tourism boards. He apprised them of the investment opportunities and tourism packages offered by the Andhra Pradesh government. Visitors to the stall were also treated to Araku coffee, Pootharekulu, and displays of colourful Etikoppaka and Kondapalli toys.
-Mr. Durgesh briefed the international media on the Andhra Pradesh Tourism Policy 2024–29, which accords industrial status to the tourism sector, and assured full government support to investors. Addressing groups of international visitors, he reiterated the government’s commitment to earning global recognition for Andhra Pradesh Tourism.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/andhra-pradesh/minister-promotes-andhra-pradesh-tourism-at-world-travel-market-2025-in-london/article70241312.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:48:29 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/3yxdnd/article70241546.ece/alternates/LANDSCAPE_1200/9604_4_11_2025_22_4_28_1_IMG_20251104_WA0032.JPG</t>
-  </si>
-  <si>
-    <t>GSAT-7R will strengthen Indian Navy’s surveillance and communication in the Indian Ocean Region</t>
-  </si>
-  <si>
-    <t>The successful launch of India’s CMS-03 (GSAT-7R) satellite aboard the LVM3-M5 rocket on November 2, 2025, from the Satish Dhawan Space Centre in Sriharikota will provide a major boost to the country’s pursuit of maritime security and technological self-reliance.
-The 4,400 kg multi-band communication satellite, designed and developed indigenously by the Indian Space Research Organisation (ISRO), is the heaviest communication satellite launched into the Geosynchronous Transfer Orbit (GTO) from Indian soil. It will play a crucial role in enhancing the Indian Navy’s operational reach, situational awareness, and surveillance capabilities across the Indian Ocean Region.
-Secure communication coverage
-The GSAT-7R is the successor to the GSAT-7 “Rukmini,” India’s first dedicated military satellite, launched in 2013. While Rukmini revolutionised naval communications by providing real-time data links across the Arabian Sea and the Bay of Bengal, the GSAT-7R significantly upgrades these capabilities. Equipped with multi-band transponders (UHF, S, C, and Ku bands), the GSAT-7R enables seamless voice, data, and video communication between naval ships, submarines, aircraft, and Maritime Operations Centres (MOCs). The satellite’s advanced payload ensures high-capacity, secure, and jam-resistant communication — vital for network-centric warfare and joint operations with the Army and the Air Force.
-With a lifespan of 15 years, the GSAT-7R extends secure communication coverage up to 2,000 km from India’s coastline, encompassing vast stretches of the Indian Ocean Region. This expanded coverage will allow the Indian Navy to monitor critical sea lanes, chokepoints, and potential maritime threats more effectively. It will support continuous coordination among naval assets deployed on anti-piracy, anti-submarine, and humanitarian missions, ensuring real-time situational updates and rapid response capabilities.
-Moreover, the GSAT-7R will enhance maritime domain awareness (MDA) by integrating space-based communication with surveillance platforms, such as coastal radars, reconnaissance aircraft, and unmanned systems. This synergy will allow the Navy to maintain an uninterrupted watch over the region’s dynamic maritime environment, strengthening India’s ability to deter and respond to any hostile activity.
-According to experts, the launch of the GSAT-7R underscores India’s growing self-reliance in defence space technology under the vision of Aatmanirbhar Bharat. By securing robust and indigenous satellite communication infrastructure, the Navy can operate independently of foreign systems, ensuring confidentiality and reliability in strategic operations.
-Quantum leap
-In essence, the GSAT-7R represents a quantum leap in India’s maritime communication and surveillance architecture, empowering the Indian Navy to maintain a vigilant, connected, and technologically advanced presence across the Indian Ocean Region.
-The Navy’s satellites, sensors, radars, unmanned aerial vehicles, and surveillance aircraft relay real-time data to the Information Management and Analysis Centre (IMAC), now being upgraded into a National Maritime Domain Awareness (NMDA) platform. The NMDA will integrate data from multiple sources to create a unified operational picture for naval commanders. Using AI-enabled analytics, it will enhance situational awareness, improve surveillance, and support swift decision-making. The system will help detect and counter threats such as illegal fishing, smuggling, piracy, and maritime terrorism, strengthening India’s maritime security and safeguarding its strategic interests across the Indian Ocean Region.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/sci-tech/gsat-7r-will-strengthen-indian-navys-surveillance-and-communication-in-the-indian-ocean-region/article70240234.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:42:47 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/seagfz/article70240681.ece/alternates/LANDSCAPE_1200/02th-SAURABH-muG30F42DOF.4.jpg.jpg</t>
-  </si>
-  <si>
-    <t>Karnataka issues guidelines for use of fines collected under tobacco control law</t>
-  </si>
-  <si>
-    <t>The State Health Department has issued revised guidelines for the proper utilisation of fines collected under the Cigarettes and Other Tobacco Products Act (COTPA), 2003, in Karnataka.
-Under the National Tobacco Control Programme (NTCP), implemented as part of the National Health Mission, authorised officers are empowered to levy spot fines on violators of COTPA. The fines collected are to be deposited in a joint account operated by the Deputy Commissioner and the District Health and Family Welfare Officer.
-According to the latest circular issued by the Health Commissioner on Tuesday, the fine amount should be used exclusively for tobacco control activities at the district level. District Tobacco Control Cells have been directed to prepare annual action plans outlining the use of the funds, which must be discussed and approved by the District-Level Coordination Committee (DLCC), chaired by the Deputy Commissioner.
-At least 70% of the fine amount should be used for strengthening tobacco de-addiction services. The permissible activities include the purchase of Nicotine Replacement Therapy (NRT) drugs and equipment such as CO monitors and spirometers, conducting training programmes and workshops, implementing tobacco-free educational institution and village guidelines, and undertaking IEC (Information, Education and Communication) campaigns., according to the revised guidelines.
-Districts have also been instructed to maintain proper records and submit annual audit reports as per NHM norms. Any proposal involving expenditure of more than ₹1 lakh from the fine amount will require approval from the Commissioner, the circular stated.
-The order further clarified that the fines collected under COTPA are to be treated as additional funds and can be used only after fully utilising the regular annual allocation provided under the NTCP.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/karnataka-issues-guidelines-for-use-of-fines-collected-under-tobacco-control-law/article70241013.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:42:13 +0530</t>
-  </si>
-  <si>
-    <t>Eight killed in car-truck collision in Barabanki</t>
-  </si>
-  <si>
-    <t>Eight people were killed after a truck collided with a car on the Deva-Fatehpur road in Barabanki district on Tuesday, officials said.
-The incident occurred when a speeding truck collided head-on with an Ertiga vehicle that reportedly did not have a licence plate. The impact of the collision was severe, leaving the car completely crushed and causing panic among bystanders.
-Among the deceased identified are driver Shrikant Shukla, Pradeep Soni, his wife Madhuri Soni, and their son Nitin, all residents of Fatehpur town. The identities of the other victims are yet to be confirmed.
-According to officials, all occupants of the Ertiga were returning home after taking a holy dip in the Ganges at Bithoor in Kanpur.
-Uttar Pradesh Chief Minister Yogi Adityanath expressed grief over the loss of lives and directed district officials to expedite relief measures.
-“The loss of life in the unfortunate accident is extremely sad and heart-wrenching. My condolences are with the bereaved families. I pray to Lord Shri Ram to grant salvation to the departed souls, strength to the bereaved families to bear this immense loss, and speedy recovery to the injured. Om peace,” an official statement quoted the Chief Minister as saying.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/uttar-pradesh/eight-killed-in-car-truck-collision-in-barabanki/article70241421.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:30:18 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/news/national/gfvskd/article70241478.ece/alternates/LANDSCAPE_1200/Accident%20stock.jpeg</t>
-  </si>
-  <si>
-    <t>EBC voters hold the key to Bihar polls, Nitish remains their preferred choice</t>
-  </si>
-  <si>
-    <t>For Kaushalendra Chouhan, a daily wage labourer from Makhdumpur, work is erratic, often requiring him to travel long distances. Yet he claims that travel has become easier and far safer under the present government. “There is no fear of being robbed while travelling at night,” he says.
-Some 250 km at the Keoti Assembly constituency, Ram Nath Thakur says life has not materially changed for him. He works in Kolkata and has returned home for the festivals and elections. He is a barber by profession and caste. “One can’t make a living here. There are hardly any customers here,” he says.
-Mr. Chouhan and Mr. Thakur are both from the Extremely Backward Class (EBC), a diverse group of castes comprising 36% of the State’s population, as per the caste count in Bihar. This group is entirely Bihar Chief Minister and Janata Dal (United) leader Nitish Kumar’s creation, ostensibly for ensuring better reach of welfare policies. This classification is based on a reservation policy of 1978 implemented by Karpoori Thakur.
-Thakur, a Nai (barber) by caste, remains the tallest EBC leader in the State. He reserved 26% of new government positions for “Backward Classes”, in addition to existing quotas for Scheduled Castes and Adivasis (24% combined). The Backward Classes were further divided into two lists. Annexure I, who among the backwards were economically and socially worse off, got 12% reservation and 8% for Annexure II communities who were socially better placed. The Annexure II is now categorised as Other Backward Classes and include the Yadavs among others. The EBC has historically been loyal to Mr. Kumar. The Mahagatbandhan’s success in the upcoming elections will largely depend on its ability to win over a portion of this crucial vote bank.
-In the last two decades that Mr. Kumar has been in power, Mr. Chouhan’s and Mr. Thakur’s economic condition has not significantly improved. Yet, their electoral choice remains unchanged. Both have voted for the NDA in the past elections and continue to do so. Their choices are based partly on aversion for the Rashtriya Janata Dal (RJD) and partly on their loyalty for Mr. Kumar.
-In the 2020 Assembly elections, the victory margin was less than 5,000 in 52 of the 243 constituencies in Bihar. Even a minor shift in caste-based political loyalties could change the results.
-The Hilsa constituency in Nalanda district exemplifies this volatility. In the 2020 election, JD(U) won the seat. “People’s mandate was in my favour,” RJD leader Atri Muni says. He had been declared victor by a margin of 549 votes at 5 p.m. The JD(U)’s candidate Krishnamurari Sharan congratulated Mr. Muni and left the counting centre. But an hour later, Mr. Sharan was declared the winner with a difference of 12 votes. Mr. Muni had challenged the result, but the Patna High Court took three-and-a-half years to admit the plea, only to eventually dismiss it.
-Mr. Muni reels off the caste arithmetic of Hilsa: with Yadavs and Kurmis evenly matched, the fragmented EBC vote will once again be decisive.
-But not all are happy. Birendra Mistri is upset at the bribes he has to pay to get any paperwork done in the block office. He comes from the Badai caste that falls under EBC group. “Nitish stands for caste-based politics. He has filled the departments with officials from his caste… all his policies are limited to the paper. Nothing translates on the ground,” he says. Having voted for the JD(U) in multiple elections, he is now looking for options.
-Rajesh Kumar Sahu, also an EBC, nods along to Mr. Mistri’s appraisal. He runs a small grocery shop. The business has been slow. His quibble with the government is the mass migration. “If everyone leaves, then how will I have customers,” Mr. Sahu says. He too, like Mr. Mistri, is looking for options, but he rules out the RJD. “I could vote for Jan Suraaj,” he replies after thinking for a while. He is familiar with Jan Suraaj founder Prashant Kishor, but the candidate for Hilsa is not a familiar face. “I will see closer to the election, depending on which way everyone is voting,” he says.
-RJD, though aware of its limitation in breaking Mr. Kumar’s stranglehold, has only 13 EBC candidates, as opposed to JD(U) which has 21. The Mahagatbandhan this time has two EBC parties – Mukesh Sahani’s Vikashsheel Insaan Party that represents the Mallahs and Nishads, and I.P. Gupta’s Indian Inclusive Party that represents Tanti-Pan Samaj. But whether these relatively new entrants can mobilise enough support to shift the balance remains to be seen.
-For now, Nitish Kumar continues to be the preferred choice for a majority of EBC voters.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/elections/bihar-assembly/ebc-voters-hold-the-key-to-bihar-polls-nitish-remains-their-preferred-choice/article70240667.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:21:06 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/4irvh2/article70241485.ece/alternates/LANDSCAPE_1200/20251103256L.jpg</t>
-  </si>
-  <si>
-    <t>After visit to Vantara, global wildlife committee recommends India pause animal import</t>
-  </si>
-  <si>
-    <t>A committee of CITES, the globe’s most influential agreement on wildlife conservation, whose strictures on the cross-border movement of protected animal species inform national wildlife laws, has recommended that India’s wildlife authorities pause the issue of permits that allow endangered animals to be imported by zoos, and wildlife rescue and rehabilitation centres.
-This, CITES says, should be in place until India comprehensively reviews its practices and ensures that “due diligence is exercised systematically and consistently”, and animal trade is not carried out in “violation of the Convention”.
-India became a signatory to the Convention on International Trade in Endangered Species of Wild Flora and Fauna (CITES) in 1976. Currently, 185 countries are signatories.
-The recommendations are part of a report prepared by a CITES-designated committee after a visit to the Greens Zoological Rescue and Rehabilitation Centre (GZRRC) in Jamnagar, a part of the Vantara animal rescue and rehabilitation centre affiliated to the Reliance Foundation. The Radha Krishna Temple Elephant Welfare Trust (RKTEWT) is also a part of Vantara, and while primarily focussed on elephant welfare, also has permissions to manage other imported species of fauna.
-In September, a Supreme Court-appointed Special Investigation Team, constituted to conduct an “independent factual appraisal” of complaints against Vantara, said it found no statutory irregularities in the acquisition of animals.
-The CITES committee found that the facilities in Vantara kept “exceptionally high standards”, and had “advanced facilities” with appropriate “veterinary care standards”. It also noted that it “could not find evidence” that the facility brought in animals for commercial purposes nor evidence that animals being imported to India lacked import, export, and re-export CITES permits.
-However, the committee’s report, uploaded on October 31 on the CITES website, noted that “...several imports [by GZRRC and RKTEWT] still raise questions regarding the origin of the specimens… the use of source and purpose-of-transaction codes, and the exercise of due diligence by India”.
-The committee visited Vantara from September 15-20, after it was asked by the CITES Secretariat to look into India’s processes for verifying whether the manner in which live animals were procured reflected the conditions under which they were sourced (for example, ‘W’ — from the wild, or ‘C’ — bred in captivity) and purpose-of-transaction (’Z’ — to be placed in a zoo, or ‘B’ — breeding in captivity).
-The visit was following a 2023 recommendation by the Secretariat to look into “trade in live animals with purpose code Z” by the GZRRC.
-In the last two years, there have been several journalistic investigations into procurement practices at Vantara, as well as reports by environmental groups that alleged animals were being procured in large numbers, both within India and from abroad, in ways that contravened the CITES stipulation.
-The GZRRC is registered as a zoo, rescue centre, a conservation breeding centre, and a centre for studying animals. Under Indian laws, a “zoo” cannot function as a licensed dealer in captive animals. Moreover, rescued or confiscated animals shall not be displayed to the public.
-Under CITES conventions, it is legal to trade animals commercially, provided relevant conditions are met, and permits state so explicitly. It is also permissible to buy animals for the purposes of breeding in captivity for conservation purposes, provided paperwork attests to it, and it is registered under appropriate rules of the Convention.
-The CITES committee’s reservations stemmed from observations where permit codes did not appropriately reflect the arrangement between the exporting country and India.
-The GZRRC, for instance, imported several animals from the Republic of Czechia.
-That country, according to the committee, “had no doubts” that the animals were being “sold” to the GZRRC and were not exported for the “purpose of rescue”. The Czech authorities provided invoices showing lists of animals acquired, price per unit, and taxes.
-The GZRRC’s interpretation, however, was that the animals weren’t “sold”, and the expense involved was the “cost of insurance, freight and customs duties”. India’s wildlife authorities, in explaining this, cited a Supreme Court order of September 15 that said these were indeed costs as the GZRRC said so, and another order said that if an animal was procured under a “valid” export permit, it couldn’t be a contravention of Indian law or the CITES.
-In a case involving the import by the GZRRC of two captive-bred snow leopards from Germany, the latter issued permits under the codes ‘C’ (origin as captive bred) and ‘T’ (for commercial purposes). When the animals reached India, the Indian authorities raised a query on the purpose of import (because of the ‘T’ label). The GZRRC said the animals were ‘donated’ by a facility in Germany. Following this, the Indian authorities changed the ‘T’ label to a ‘Z’ (zoological). The committee said that India ideally ought to have checked with German authorities, their reason for labelling it a commercial transaction instead of “only relying on the information by the importer (GZRRC)”.
-The committee highlighted an instance where Indian authorities issued permission allowing the import of chimpanzees from Cameroon by the GZRRC. It later turned out that the export permits by Cameroon were forged. The GZRRC did not proceed with the import as it couldn’t verify the antecedents of the chimpanzees at the Cameroonian facility. The committee noted that, ideally, Indian authorities should have known that, based on the CITES database, which they can access, Cameroon has not traded any chimpanzees since 2000, and there was no captive breeding of chimpanzees ongoing in that country.
-“The fake permits brought to the attention of the Secretariat may suggest that the large number of acquisitions of live animals by the GZRRC.. has attracted attention, and that certain individuals or entities could attempt to exploit this as a way to traffic animals. This shows that there is a need for caution to ensure that imports of large numbers of animals by these facilities are not inadvertently creating a demand for illegally sourced animals. Reinforced due diligence in this regard is crucial,” the committee noted.
-There were a litany of similar other examples raised by the committee on imports that were permitted by the Indian authorities of hundreds of animals. Indian authorities seemed to be acknowledging these lapses. “...Representatives from India...expressed appreciation for the guidance provided on these issues and confirmed that they would work on improving their processes and procedures. The Indian Management Authority has reiterated this commitment in writing in its submission to the Secretariat for the preparation of the present document. The management of the GZRRC also indicated their willingness to be in full compliance with CITES and to develop their own due diligence approach,” the committee report noted.
-The Hindu reached out with detailed questionnaires to Vantara, and the Union Ministry of Environment, Forest and Climate Change for comment but had not heard back till the time of going to press.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/sci-tech/energy-and-environment/after-visit-to-vantara-global-wildlife-committee-recommends-india-pause-animal-import/article70241099.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:18:00 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/6w0de1/article70241464.ece/alternates/LANDSCAPE_1200/IMG_vantaraelephant_2_1_6SETEGBD.jpg</t>
-  </si>
-  <si>
-    <t>7 years on, 2 convicted for killing private firm employee in road rage incident</t>
-  </si>
-  <si>
-    <t>The Additional City Civil and Sessions Court on Monday convicted and sentenced two youths to rigorous life imprisonment for allegedly bludgeoning a 25-year-old private firm employee to death over a trivial road rage incident in the limits of the Mico Layout police station limits seven years ago.
-Coincidentally, the verdict came on the birthday of the victim, Siddarth Koushal, a native of Bihar, who was working for a private firm in the city.
-According to the prosecution, Siddarth and his friend — who owned a restaurant in Electronics City — were returning home in a car on June 26, 2018 around 3 a.m. after closing the eatery. Two of their friends followed them on a bike. The duo had stopped the car by the roadside to relieve themselves when the accused — Girish, son of a builder, and his friend Mahesh — brushed their bike against the car.
-An argument broke out after Siddarth noticed a dent and shouted at them. Enraged, the duo allegedly returned, picked up a stick lying nearby, and attacked Siddarth. By the time his friends rushed to his rescue, the assailants had fled, leaving him grievously injured.
-A nearby paan beeda shop owner, who was sleeping outside his shop near a bar and restaurant, woke up to the commotion and recognised one of the attackers. Siddarth, who was profusely bleeding, was rushed to a private hospital, where he succumbed to injuries later.
-Based on a complaint, then the Mico Layout Inspector, R.M. Ajay, registered a case of murder and, with the help of the shop owner’s statement, tracked down Girish and later arrested Mahesh. The police collected technical evidence and witness statements before filing a charge sheet in the court.
-While Girish remained in judicial custody due to the gravity of the offence, Mahesh was released on bail. During the trial, several eyewitnesses, including the paan shop owner and two of Siddarth’s friends, turned hostile, causing delays in the proceedings. However, strong technical evidence and the effective arguments of Public Prosecutor Mahalingappa ensured the conviction of both accused.
-Siddarth’s father, Koushalendra Kumar, an advocate by profession, attended every hearing, even during the COVID-19 lockdown. Following the verdict, he met the police team and distributed sweets as a gesture of gratitude.
-“Siddarth was my elder son. We have not celebrated any festival since his death, but today we lit a lamp after the judgment,” Mr. Kumar told the police team.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/karnataka/7-years-on-2-convicted-for-killing-private-firm-employee-in-road-rage-incident/article70240915.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:17:24 +0530</t>
-  </si>
-  <si>
-    <t>SCTIMST an inspiration for all government institutions in the country: Vice-President</t>
-  </si>
-  <si>
-    <t>Vice-President C.P. Radhakrishnan has hailed the Sree Chitra Tirunal Institute for Medical Sciences and Technology (SCTIMST), which has performed heart valve surgeries on nearly two lakh patients, as an inspiration for all government institutions in the country.
-Research becomes a true success only when it touches common people and creates a larger and meaningful impact on society, a goal that the SCTIMST has achieved commendably, Mr. Radhakrishnan said.
-The Vice-President was addressing a gathering on Tuesday after visiting the SCTIMST’s newly inaugurated hospital building under the Pradhan Mantri Swastha Suraksha Yojana (PMSSY), which boasts high-end medical infrastructure, sophisticated medical equipment and expanded intensive care unit facilities.
-He also visited the medical exhibition arranged at the SCTIMST, showcasing the medical innovations and new technologies indegenously developed at the Institute. He said that the government’s ultimate goal was health for all and called for better services to the poorest of the poor.
-Governor Rajendra Vishwanath Arlekar, Union Minister of State for Petroleum, Natural Gas, and Tourism Suresh Gopi, State Finance Minister K.N. Balagopal, and SCTIMST Director Sanjay Behari also addressed the meeting.</t>
-  </si>
-  <si>
-    <t>https://www.thehindu.com/news/national/kerala/sctimst-an-inspiration-for-all-government-institutions-in-the-country-vice-president/article70241346.ece</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:15:24 +0530</t>
-  </si>
-  <si>
-    <t>https://th-i.thgim.com/public/incoming/1i2jyy/article70241369.ece/alternates/LANDSCAPE_1200/20251104172L.jpg</t>
-  </si>
-  <si>
     <t>TOI</t>
   </si>
   <si>
@@ -469,6 +484,22 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125094369,width-1070,height-580,imgsize-877846,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Number of road fatalities in 2024 likely to surpass 2023 figure, the highest ever</t>
+  </si>
+  <si>
+    <t>Number of road fatalities in 2024 likely to surpass 2023 figure, the highest ever
+NEW DELHI: The number of road deaths in 2024 is set to surpass that in 2023 with over two dozen states and UTs, including Uttar Pradesh, Tamil Nadu, Maharashtra, Madhya Pradesh, Rajasthan, Odisha, Telangana, Assam and Delhi reporting higher number of fatalities last year. As per provisional data compiled from states/UTs, excluding West Bengal, a little over 1.7 lakh people died in road crashes last year.In 2023, road crashes had claimed around 1.73 lakh lives, the highest ever for a year, and West Bengal had reported 6,027 of these fatalities. Sources said that once data from West Bengal is included, the number of deaths would be more than that in the previous year. Data sent by states on crashes, fatalities, injuries and the factors responsible for them are being rechecked and reconciled before the final report is published, they added.While the rise in fatalities despite efforts of the govt to curb them remains a huge concern, there is a silver lining to the provisional data for 2024: nine states and UTs have reported a decline in the number of deaths. For example, Kerala reported 3,846 fatalities in 2024 compared to 4,080 in the previous year, and Gujarat recorded 7,717 deaths last year compared to 7,854 in 2023.Experts maintain that unless there is a significant dip in fatalities in the 10 states that report a large share of the overall figure, achieving the goal to reduce the number of road deaths by half will not be possible.“There is a need for focussed efforts to reduce fatal crashes and deaths on National Highways and state highways, which account for nearly 60% of all fatalities,” said a former Union road transport secretary.Though data on road accidents do not fully represent the magnitude of the problem given that not all such incidents are reported or recorded by police, the provisional data show that 35 states and UTs reported over 4.7 lakh crashes in 2024 compared to 4.8 lakh in the previous year.Meanwhile, the road transport ministry plans to amend the Motor Vehicle Act by introducing stricter norms for issuing driving licence and negative points for bad driver behaviour that can result in suspension and even cancellation of licences.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/number-of-road-fatalities-in-2024-likely-to-surpass-2023-figure-the-highest-ever/articleshow/125095336.cms</t>
+  </si>
+  <si>
+    <t>Wed, 05 Nov 2025 00:45:26 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125095390,width-1070,height-580,imgsize-771448,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>'Chhath, Halloween &amp; jungle raj': Bihar phase 1 campaign blitz ends — a quick recap</t>
@@ -533,23 +564,6 @@
     <t>https://static.toiimg.com/thumb/msid-125092587,width-1070,height-580,imgsize-40268,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>‘10% control the Army’: Rahul's caste claim at Bihar rally; BJP terms remark disgraceful</t>
-  </si>
-  <si>
-    <t>Rahul Gandhi (PTI photo)
-'Will Cut Off Your Tongue': Bihar Poll Campaign Turns Ugly, AIMIM Candidate Threatens Tejashwi Yadav
-NEW DELHI: Lok Sabha leader of opposition Rahul Gandhi on Tuesday made a striking claim in Bihar, alleging that country's 10 per cent, referring to upper castes, "hold control over the Army."Addressing a poll rally in Aurangabad's Kutumba, Rahul said, "90 per cent of the people come from extremely backward, backward, Dalit, and Adivasi communities." He went on to assert that these groups - forming the vast majority of India's population - remain largely excluded from power and privilege."All the wealth goes to them, all the jobs go to them. Look at the judiciary - they have control there, and even in the army," Rahul said, in one of his most direct attacks on the country's social and institutional hierarchy.He further added, "90 per cent of India's population is nowhere to be found," suggesting that marginalised communities have been systematically denied access to leadership and opportunity.The BJP hit back at Rahul Gandhi over his remarks on the Army. Party spokesperson Suresh Nakhua, in a post on X, said, "Rahul Gandhi is now searching for caste in the Armed Forces and says 10% of people control it. In his hate for PM Modi, he has already crossed the line into hating India."Another BJP spokesperson, Sanju Verma, also hit out at Rahul Gandhi over his remarks, saying, “Rahul Gandhi is shamelessly devious and deviously shameless.Listening to him in this clip leaves no doubt that this failed, forever-in-waiting PM is desperately trying to polarize. Now he is trying to divide the Army on caste lines — what an unhinged wreck this Leader of Opposition is. Disgraceful.”Directing his attack to Bihar government, Rahul painted a picture of unemployment in the state, blaming the Nitish Kumar government for pushing its youth into low-paying, menial labour across the country."The people of Bihar are doing manual labour across the entire country. In different parts of the country, people from Bihar are building large buildings, roads, tunnels, and factories," he said.Accusing the state government of failing its people, Rahul added, "In other words, the truth is this—that Nitish Kumar has wiped out employment here and turned the people of Bihar into the country’s labourers."</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/10-control-the-army-rahul-gandhis-caste-claim-at-bihar-rally-says-90-indians-nowhere-to-be-found/articleshow/125088800.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 18:48:06 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125088839,width-1070,height-580,imgsize-652610,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
     <t>Jeff Bezos’ ex-wife’s gift: MacKenzie Scott makes large donation; focus on education</t>
   </si>
   <si>
@@ -569,6 +583,23 @@
     <t>https://static.toiimg.com/thumb/msid-125086896,width-1070,height-580,imgsize-26596,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
+    <t>‘10% control the Army’: Rahul's caste claim at Bihar rally; BJP terms remark disgraceful</t>
+  </si>
+  <si>
+    <t>Rahul Gandhi (PTI photo)
+'Will Cut Off Your Tongue': Bihar Poll Campaign Turns Ugly, AIMIM Candidate Threatens Tejashwi Yadav
+NEW DELHI: Lok Sabha leader of opposition Rahul Gandhi on Tuesday made a striking claim in Bihar, alleging that country's 10 per cent, referring to upper castes, "hold control over the Army."Addressing a poll rally in Aurangabad's Kutumba, Rahul said, "90 per cent of the people come from extremely backward, backward, Dalit, and Adivasi communities." He went on to assert that these groups - forming the vast majority of India's population - remain largely excluded from power and privilege."All the wealth goes to them, all the jobs go to them. Look at the judiciary - they have control there, and even in the army," Rahul said, in one of his most direct attacks on the country's social and institutional hierarchy.He further added, "90 per cent of India's population is nowhere to be found," suggesting that marginalised communities have been systematically denied access to leadership and opportunity.The BJP hit back at Rahul Gandhi over his remarks on the Army. Party spokesperson Suresh Nakhua, in a post on X, said, "Rahul Gandhi is now searching for caste in the Armed Forces and says 10% of people control it. In his hate for PM Modi, he has already crossed the line into hating India."Another BJP spokesperson, Sanju Verma, also hit out at Rahul Gandhi over his remarks, saying, “Rahul Gandhi is shamelessly devious and deviously shameless.Listening to him in this clip leaves no doubt that this failed, forever-in-waiting PM is desperately trying to polarize. Now he is trying to divide the Army on caste lines — what an unhinged wreck this Leader of Opposition is. Disgraceful.”Directing his attack to Bihar government, Rahul painted a picture of unemployment in the state, blaming the Nitish Kumar government for pushing its youth into low-paying, menial labour across the country."The people of Bihar are doing manual labour across the entire country. In different parts of the country, people from Bihar are building large buildings, roads, tunnels, and factories," he said.Accusing the state government of failing its people, Rahul added, "In other words, the truth is this—that Nitish Kumar has wiped out employment here and turned the people of Bihar into the country’s labourers."</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/10-control-the-army-rahul-gandhis-caste-claim-at-bihar-rally-says-90-indians-nowhere-to-be-found/articleshow/125088800.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 18:48:06 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125088839,width-1070,height-580,imgsize-652610,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
     <t>Air traffic congestion: Flight operations impacted in Delhi; IndiGo issues advisory</t>
   </si>
   <si>
@@ -602,26 +633,6 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125091823,width-1070,height-580,imgsize-58174,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Chhattisgarh train accident: Toll reaches 8; compensation of 10 lakh announced</t>
-  </si>
-  <si>
-    <t>Photo: PTI screengrab
-At Least 5 Killed, Several Injured As Passenger Train Collides With Goods Trains In Chhattisgarh
-Rs 10 lakh to the next of kin of the deceased (casualties).
-Rs 5 lakh to those grievously injured.
-Rs 1 lakh to those with minor injuries.
-NEW DELHI: A passenger train coach hit a goods train near Chhattisgarh's Bilaspur station on Tuesday, killing eight people and leaving 14 injured in the incident, as news agency ANI reported. Measures are being taken to ensure the treatment of the injured.In a video showing the aftermath of the train collision, one train coach is seen lifted and resting atop another, with its front end crumpled from the impact.Several people, including police personnel, were visible on the tracks below, appearing to assess the wreckage.MEMU (Mainline Electric Multiple Unit train) train coach hit a goods train near Bilaspur station at about 16:00 hours. Two people have been injured in the incident. Railways have moved all the resources, and all measures are being ensured for the treatment of the injured, reported news agency ANI citing Railway officials."The last bogie and first bogie of a local train and a goods train collided near Bilaspur. Four people have lost their lives in the accident. Rescue operation is underway," Sanjay Agrawal, DC, Bilaspur told news agnecy ANI.Calling the accident extremely distressing, chief minister Vishnu Deo Sai said he has instructed the Bilaspur district collector to provide victims with all possible assistance and relief efforts."The news of the train accident near Bilaspur is extremely distressing. The Bilaspur District Collector has been consulted and instructions have been issued to provide them with all possible assistance and relief efforts. The state government stands with the affected families during this difficult time," the Chattisgarh CM wrote on X.He further wrote: "Teams from the railways and administration have immediately sprung into action for relief and rescue operations. All necessary resources and medical assistance are being ensured for the treatment of the injured. The state government is closely monitoring the situation with complete diligence and sensitivity."Chhattisgarh deputy CM Arun Sao said: "A very tragic incident has occurred. The goods train was stationary, and a MEMU train collided with it from behind. The engine is in the front coach, and some passengers also sit there. That coach has been damaged. Senior railway officials and state government officers have reached the spot. Relief and rescue operations have begun. The injured are being taken to the hospital."The government has announced the following ex-gratia compensation for the affected persons:</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/chhattisgarh-passenger-train-coach-collides-with-goods-train-near-bilaspur-injured-toll/articleshow/125086775.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 17:20:27 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125087453,width-1070,height-580,imgsize-41276,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Big AI freebie: ChatGPT Go now free for 12 months in India; how to claim the offer</t>
@@ -651,6 +662,26 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125076745,width-1070,height-580,imgsize-41718,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Chhattisgarh train accident: Toll reaches 8; compensation of 10 lakh announced</t>
+  </si>
+  <si>
+    <t>Photo: PTI screengrab
+At Least 5 Killed, Several Injured As Passenger Train Collides With Goods Trains In Chhattisgarh
+Rs 10 lakh to the next of kin of the deceased (casualties).
+Rs 5 lakh to those grievously injured.
+Rs 1 lakh to those with minor injuries.
+NEW DELHI: A passenger train coach hit a goods train near Chhattisgarh's Bilaspur station on Tuesday, killing eight people and leaving 14 injured in the incident, as news agency ANI reported. Measures are being taken to ensure the treatment of the injured.In a video showing the aftermath of the train collision, one train coach is seen lifted and resting atop another, with its front end crumpled from the impact.Several people, including police personnel, were visible on the tracks below, appearing to assess the wreckage.MEMU (Mainline Electric Multiple Unit train) train coach hit a goods train near Bilaspur station at about 16:00 hours. Two people have been injured in the incident. Railways have moved all the resources, and all measures are being ensured for the treatment of the injured, reported news agency ANI citing Railway officials."The last bogie and first bogie of a local train and a goods train collided near Bilaspur. Four people have lost their lives in the accident. Rescue operation is underway," Sanjay Agrawal, DC, Bilaspur told news agnecy ANI.Calling the accident extremely distressing, chief minister Vishnu Deo Sai said he has instructed the Bilaspur district collector to provide victims with all possible assistance and relief efforts."The news of the train accident near Bilaspur is extremely distressing. The Bilaspur District Collector has been consulted and instructions have been issued to provide them with all possible assistance and relief efforts. The state government stands with the affected families during this difficult time," the Chattisgarh CM wrote on X.He further wrote: "Teams from the railways and administration have immediately sprung into action for relief and rescue operations. All necessary resources and medical assistance are being ensured for the treatment of the injured. The state government is closely monitoring the situation with complete diligence and sensitivity."Chhattisgarh deputy CM Arun Sao said: "A very tragic incident has occurred. The goods train was stationary, and a MEMU train collided with it from behind. The engine is in the front coach, and some passengers also sit there. That coach has been damaged. Senior railway officials and state government officers have reached the spot. Relief and rescue operations have begun. The injured are being taken to the hospital."The government has announced the following ex-gratia compensation for the affected persons:</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/chhattisgarh-passenger-train-coach-collides-with-goods-train-near-bilaspur-injured-toll/articleshow/125086775.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 17:20:27 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125087453,width-1070,height-580,imgsize-41276,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Asia Cup controversy: ICC drops the hammer! Full list of players punished and warned</t>
@@ -759,23 +790,6 @@
     <t>https://static.toiimg.com/thumb/msid-125076167,width-1070,height-580,imgsize-13798,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
-    <t>'Highway man always high': Congress mocks Nitin Gadkari over Bihar poll promises</t>
-  </si>
-  <si>
-    <t>Union minister Nitin Gadkari (File photo)
-'Paid Campaign': Nitin Gadkari Slams Criticism Of E20 Program; Calls It 'Politically Motivated'
-NEW DELHI: The Congress on Tuesday took a swipe at Union road transport and highways minister Nitin Gadkari over his repeated promises to the people of Bihar, remarking that “it seems the highway man is always high.”Mocking Gadkari’s claims, Congress leader Pawan Khera shared a video on X compiling the minister’s old and recent statements in poll-bound Bihar, where he pledged to build “world-class” roads and assured the public that “the roads will be at par with American roads.”The video juxtaposed Gadkari’s promises from 2024 with his latest assurances during the ongoing election campaign in Bihar.Joining the attack, the Kerala Congress also took a jibe at the Union minister, calling him “the new jumla king in town.”Meanwhile, campaigning for the first phase of polling has concluded. Bihar will vote in the first phase on November 6 and the second on November 11, with counting of votes and announcement of results scheduled for November 14.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/india/highway-man-always-high-congress-mocks-nitin-gadkari-over-bihar-poll-promises-shares-old-us-style-roads-video/articleshow/125090791.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 21:02:42 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125090849,width-1070,height-580,imgsize-810362,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
     <t>Musk vs Altman: OpenAI’s ex chief scientist testifies in court; reveals ‘6-day story’</t>
   </si>
   <si>
@@ -795,6 +809,41 @@
     <t>https://static.toiimg.com/thumb/msid-125089911,width-1070,height-580,imgsize-859288,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
+    <t>'Highway man always high': Congress mocks Nitin Gadkari over Bihar poll promises</t>
+  </si>
+  <si>
+    <t>Union minister Nitin Gadkari (File photo)
+'Paid Campaign': Nitin Gadkari Slams Criticism Of E20 Program; Calls It 'Politically Motivated'
+NEW DELHI: The Congress on Tuesday took a swipe at Union road transport and highways minister Nitin Gadkari over his repeated promises to the people of Bihar, remarking that “it seems the highway man is always high.”Mocking Gadkari’s claims, Congress leader Pawan Khera shared a video on X compiling the minister’s old and recent statements in poll-bound Bihar, where he pledged to build “world-class” roads and assured the public that “the roads will be at par with American roads.”The video juxtaposed Gadkari’s promises from 2024 with his latest assurances during the ongoing election campaign in Bihar.Joining the attack, the Kerala Congress also took a jibe at the Union minister, calling him “the new jumla king in town.”Meanwhile, campaigning for the first phase of polling has concluded. Bihar will vote in the first phase on November 6 and the second on November 11, with counting of votes and announcement of results scheduled for November 14.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/india/highway-man-always-high-congress-mocks-nitin-gadkari-over-bihar-poll-promises-shares-old-us-style-roads-video/articleshow/125090791.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 21:02:42 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125090849,width-1070,height-580,imgsize-810362,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
+    <t>Former Bruins forward Milan Lucic lands another PTO, eyes contract with Blues' AHL affiliate</t>
+  </si>
+  <si>
+    <t>Former Boston Bruins forward Milan Lucic has secured a new professional try-out (PTO) contract with AHL (Credit: AP Photo/Charles Krupa, File)
+Milan Lucic lands another PTO with St. Louis Blues affiliate Springfield Thunderbirds
+Also read:
+Former Boston Bruins forward Milan Lucic has secured a new professional try-out (PTO) contract with AHL’s Springfield Thunderbirds, the St. Louis Blues announced on Tuesday. According to reports, Lucic is already on PTO with the Blues during training camp, but his chances were derailed when the 6-foot-3 left winger suffered a lower-body injury during preseason play.However, after landing this new PTO with the Blues' AHL affiliate, he is now getting another chance to try to earn a contract for the season. The signing, officially announced by the Blues, marks a fresh attempt for the 37-year-old winger to earn a spot in a full-season contract. With the new PTO in Springfield, Lucic now has a clear opportunity to show his strength and prowess on ice, with the hope of becoming an impactful player of the team. Milan Lucic has landed another PTO on Tuesday with the AHL’s Springfield Thunderbirds. According to the NHL, St. Louis Blues President of Hockey Operations and General Manager Doug Armstrong announced today that forward Milan Lucic will join the Blues’ AHL affiliate, the Springfield Thunderbirds.Earlier, he joined the St. Louis Blues on a PTO ahead of the 2025 training camp, but his chances were derailed when the former Boston Bruins veteran suffered a lower-body injury.With the new PTO in Springfield, Lucic now has a clear opportunity to show his effectiveness on ice.It is to be noted that Lucic last played in the NHL during the 2023-24 season with the Bruins. In four games for the Bruins that campaign, the left winger recorded two assists, 12 hits, and a minus-1 rating. However, his stint with the Bruins was cut short, as he entered the NHL Player Assistance Program after being arrested for an alleged domestic incident. Though the legal charges were dropped, the incident created a hindrance in his game.Despite this, Milan Lilac managed to play with the Bruins, where he appeared in 570 games and accumulated 139 goals, 205 assists, 344 points, 774 penalty minutes, and 1,592 hits. Besides, he also captured a Stanley Cup title with Boston Bruins in 2011, proving his position as a top-tier power forward of his generation.</t>
+  </si>
+  <si>
+    <t>https://timesofindia.indiatimes.com/sports/nhl/news/former-bruins-forward-milan-lucic-lands-another-pto-eyes-contract-with-blues-ahl-affiliate/articleshow/125092439.cms</t>
+  </si>
+  <si>
+    <t>Tue, 04 Nov 2025 23:33:28 +0530</t>
+  </si>
+  <si>
+    <t>https://static.toiimg.com/thumb/msid-125093239,width-1070,height-580,imgsize-74700,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
+  </si>
+  <si>
     <t>It’s 'Mango Lassi' Mamdani morning in Big Apple</t>
   </si>
   <si>
@@ -811,42 +860,6 @@
   </si>
   <si>
     <t>https://static.toiimg.com/thumb/msid-125091217,width-1070,height-580,imgsize-390229,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>Meghan Markle’s friend reveals why Prince Harry looked upset at Dodgers game</t>
-  </si>
-  <si>
-    <t>Meghan Markle’s friend reveals the real reason Prince Harry looked upset after Dodgers’ World Series win (Image via Getty)
-Meghan Markle’s joyful Dodgers celebration shows her team spirit
-Prince Harry’s calm reaction to the Dodgers’ World Series win surprises fans
-On November 1, the Dodgers beat the Toronto Blue Jays 5-4 in Game 7 after 11 innings. Meghan Markle’s close friend Kelly McKee Zajfen shared the couple’s reaction on her Instagram Stories, joking, “Best game ever! Sorry H, your team didn’t win but mine diiiiiiid. @Dodgers I LOVE YOU!!!!”Meghan, 44, was seen laughing and dancing with Kelly as they celebrated the Dodgers’ win at home. Prince Harry, 41, sat quietly in a recliner, looking less excited. In the short clip shared online, Meghan Markle sealed her celebration with a kiss, while Prince Harry’s puzzled look quickly caught fans’ attention.Kelly McKee Zajfen’s video showed a big difference between Meghan’s energy and Harry’s mood. Meghan cheered for the Dodgers, shouting and laughing, while Harry seemed to be quietly supporting the Blue Jays instead. Kelly later teased Harry for his reaction, calling it “the best game ever.”Just a few days earlier, the royal couple had attended Game 4 of the World Series in Los Angeles on October 28. Both wore matching Dodgers baseball caps and smiled for the crowd. Fans now say Prince Harry’s reaction at home showed where his true loyalties might lie.Prince Harry and Meghan Marklemoved to California in 2020 after stepping down as senior royals. Since then, they’ve often been spotted at local sports events and family outings.Meghan Markle recently called Prince Harry “my biggest supporter” during an April interview on Jamie Kern Lima’s podcast. “He loves me so much,” she said. “We’ve built a beautiful life and have two healthy, happy kids.”Also Read: Victor Conte, Man Behind MLB’s Biggest Steroid Scandal, Dies At 75 The couple share a six-year-old son, Prince Archie, and a four-year-old daughter, Princess Lilibet. Meghan said they still feel like they’re in a “honeymoon period” even after seven years of marriage. She also spoke about her new Netflix series With Love, Meghan and her return to Instagram to share her family life.While Meghan Markle’s cheering moment has gone viral, fans can’t stop talking about Prince Harry’s calm face during the Dodgers’ big win, a look that said everything without a word.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/mlb/news/meghan-markles-friend-reveals-the-real-reason-prince-harry-looked-upset-after-dodgers-world-series-win/articleshow/125071926.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 05:01:47 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125071924,width-1070,height-580,imgsize-716408,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
-  </si>
-  <si>
-    <t>‘I can make you smile’: SRK's heartfelt reply to Gambhir; fans go berserk</t>
-  </si>
-  <si>
-    <t>SRK responded with a heartfelt message to Team India head coach Gautam Gambhir's birthday wish (Image via X/@GautamGambhir)
-SRK's response to Gautam Gambhir on X
-SRK's response to Suresh Raina's birthday wishes on X
-Bollywood superstar Shah Rukh Khan on Tuesday replied to several birthday wishes that poured in on social media, including one from India head coach Gautam Gambhir, with a heartfelt message that highlighted their bond.On Sunday, Gambhir had shared a warm note for the actor on his 60th birthday, calling him “the brightest star shining in our lives” and praising his “humility and grace.” The India coach’s post featured a picture of the two from their Kolkata Knight Riders days, a partnership that delivered IPL titles in 2012, 2014 and again in 2024 when Gambhir returned as mentor.Responding to Gambhir’s message, Shah Rukh wrote on X , “Thank u my captain!! Nicest thing is I can make you smile… ha ha. Congrats on all the success.” His reply quickly drew attention, with fans celebrating the exchange between two of KKR’s most influential figures.The actor also responded to several other cricketing names who had sent him birthday wishes. To former India batter Suresh Raina, SRK wrote, “Thank u @ImRaina … all the best to you. Lots of love always!!”When Rinku Singh, one of KKR’s current stars, wished him, Shah Rukh responded with a personal touch: “Thank u Rinku.Lots of love… and shaadi kab hai?” Rinku is engaged to MP Priya Saroj. The couple got engaged in a ceremony in Lucknow on June 8, 2025. The date of the wedding is not yet know, with Shah Rukh Khan's light-hearted query adding a bit of fun to the suspense.He also replied to former India intetnational Harbhajan Singh, saying, “Thank you Paaji. Been a long time since we met. Catch you soon. Lots of love.”Shah Rukh’s responses reflected his trademark warmth and humour, qualities that have long stood out to both fans and colleagues across industries.The actor’s 60th birthday celebrations saw social media flooded with wishes from cricketers, celebrities and admirers alike, marking yet another reminder of his popularity.</t>
-  </si>
-  <si>
-    <t>https://timesofindia.indiatimes.com/sports/cricket/news/my-captain-shah-rukh-khans-i-can-make-you-smile-comment-for-gautam-gambhir-goes-viral/articleshow/125091858.cms</t>
-  </si>
-  <si>
-    <t>Tue, 04 Nov 2025 22:38:00 +0530</t>
-  </si>
-  <si>
-    <t>https://static.toiimg.com/thumb/msid-125091969,width-1070,height-580,imgsize-490563,resizemode-75,overlay-toi_sw,pt-32,y_pad-40/photo.jpg</t>
   </si>
   <si>
     <t>Charlise Springer breaks silence after Blue Jays' World Series heartbreak</t>
@@ -1343,7 +1356,7 @@
         <v>25</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1351,19 +1364,19 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1371,19 +1384,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1391,19 +1404,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1411,19 +1424,19 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1431,19 +1444,19 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1451,19 +1464,19 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1471,19 +1484,19 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1491,19 +1504,19 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1511,19 +1524,19 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1531,19 +1544,19 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1551,19 +1564,19 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1571,19 +1584,19 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E17" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1591,19 +1604,19 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>84</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1611,19 +1624,19 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1631,19 +1644,19 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1651,419 +1664,419 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E22" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E24" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B25" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C25" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E26" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E27" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B29" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C29" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E29" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B30" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C30" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E30" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B31" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C31" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E31" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B32" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C32" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C33" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E33" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B34" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C34" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E34" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B35" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C35" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E35" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B36" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C36" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E36" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B37" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C37" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E37" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C38" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E38" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B39" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C39" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E39" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B40" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C40" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E40" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C41" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E41" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>